<commit_message>
УЗП: vary D/E prose, put tool class before examples; add .gitattributes
- Reworded the opening sentence of Пояснение (D) and the frame sentence
  of each Реализация (E) subsection for the 21 measures filled/rewritten
  in the previous pass, so the text reads as varied, human-written prose
  instead of a repeated template. F and G are untouched.
- Reordered technical examples: the tool class is now named first,
  followed by a blank line and then the three-category product list
  (previously the 'Примеры средств защиты' label came before the class
  was named).
- Added .gitattributes marking Office file extensions as binary, to
  rule out line-ending normalization as a source of file corruption.
</commit_message>
<xml_diff>
--- a/docs/WIKI GOST R 57580.1.xlsx
+++ b/docs/WIKI GOST R 57580.1.xlsx
@@ -80,7 +80,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -137,6 +137,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -328,7 +334,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -751,6 +757,42 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1166,13 +1208,13 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D5" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в том, что каждый пользователь и представитель эксплуатационного персонала осуществляет логический доступ к ресурсам финансовой организации исключительно под собственной учётной записью, однозначно идентифицирующей конкретного субъекта, а не под общими (групповыми), анонимными или обезличенными учётными записями.
+      <c r="D5" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы каждый пользователь и представитель эксплуатационного персонала осуществлял логический доступ к ресурсам финансовой организации исключительно под собственной учётной записью, однозначно идентифицирующей конкретного субъекта, а не под общими (групповыми), анонимными или обезличенными учётными записями.
 Главная цель меры — обеспечить персональную ответственность каждого субъекта логического доступа за совершённые им действия: без уникальной персонификации невозможно достоверно установить, кто именно выполнил то или иное действие в информационной системе, что делает бессмысленным любое последующее расследование инцидентов и обесценивает результаты регистрации событий.</t>
         </is>
       </c>
-      <c r="E5" s="125" t="inlineStr">
+      <c r="E5" s="145" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1183,23 +1225,12 @@
           </r>
           <r>
             <t xml:space="preserve">
-Поскольку мера реализуется только техническими методами, её внедрение предполагает:
-1. Настройку операционных систем, СУБД, прикладного и сетевого программного обеспечения (ПО) таким образом, чтобы вход в систему и выполнение любых операций были возможны только после успешной идентификации и аутентификации под персональной учётной записью;
+Так как мера носит сугубо технический характер, её внедрение сводится к следующим шагам:
+1. Настройка операционных систем, СУБД, прикладного и сетевого программного обеспечения (ПО) таким образом, чтобы вход в систему и выполнение любых операций были возможны только после успешной идентификации и аутентификации под персональной учётной записью;
 2. Технический запрет создания и использования групповых, общих, анонимных и гостевых учётных записей для логического доступа пользователей и эксплуатационного персонала (за исключением технологических учётных записей, для которых персонализируется ответственный за их использование);
 3. Централизованное управление учётными записями через каталог (например, Active Directory, LDAP-каталог) или систему класса IdM (Identity Management), обеспечивающее уникальность идентификаторов и исключающее их повторное использование;
 4. Технический контроль (блокировку) попыток входа под неперсонифицированными или разделяемыми учётными записями с регистрацией таких попыток в журнале событий.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и каталогами (IdM, службы каталогов), средства защиты от несанкционированного доступа (СЗИ от НСД).
+Применимый класс средств — системы управления учётными записями и каталогами (IdM, службы каталогов), средства защиты от несанкционированного доступа (СЗИ от НСД).
 Иностранные: Microsoft Active Directory, Oracle Identity Manager, One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К, Avanpost IDM и др.
 Открытый код: FreeIPA, OpenLDAP и др.</t>
@@ -1249,13 +1280,13 @@
           <t>О-О-Т</t>
         </is>
       </c>
-      <c r="D6" s="127" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в периодическом сопоставлении перечня разблокированных (активных) учётных записей в информационных системах с перечнем легальных субъектов логического доступа — то есть работников, состоящих в трудовых отношениях с организацией, и представителей внешних (подрядных) организаций, имеющих действующие основания для доступа.
+      <c r="D6" s="146" t="inlineStr">
+        <is>
+          <t>Речь идёт о периодическом сопоставлении перечня разблокированных (активных) учётных записей в информационных системах с перечнем легальных субъектов логического доступа — то есть работников, состоящих в трудовых отношениях с организацией, и представителей внешних (подрядных) организаций, имеющих действующие основания для доступа.
 Главная цель меры — своевременно выявлять учётные записи, которые остаются разблокированными, хотя субъект, которому они принадлежат, уже утратил основания для логического доступа (уволен, переведён, истёк срок договора), и тем самым исключить возможность использования таких учётных записей для несанкционированного доступа.</t>
         </is>
       </c>
-      <c r="E6" s="128" t="inlineStr">
+      <c r="E6" s="147" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1266,7 +1297,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает проведение периодических сверок перечня активных учётных записей с кадровыми данными и данными о действующих договорах с внешними организациями. Для этого необходимо:
+На организационном уровне необходимо проводить периодические сверки перечня активных учётных записей с кадровыми данными и данными о действующих договорах с внешними организациями:
 1. Утвердить регламент, определяющий периодичность сверки (например, ежемесячно), источники данных о легальных субъектах (кадровая система, реестр договоров с подрядчиками) и ответственных за проведение сверки лиц;
 2. Проводить сверку выгрузки активных учётных записей с данными кадрового учёта и реестром действующих подрядных организаций;
 3. По фактам расхождений инициировать блокирование избыточных учётных записей и фиксировать результат сверки в акте.</t>
@@ -1281,21 +1312,10 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает автоматизацию процесса сверки за счёт интеграции системы управления учётными записями с источниками кадровых данных. Для этого используются:
+Технически процесс сверки можно и нужно автоматизировать за счёт интеграции системы управления учётными записями с источниками кадровых данных:
 1. Системы класса IdM, автоматически формирующие перечень легальных субъектов на основании данных кадровой системы (HRM) и реестра подрядчиков и сверяющие его с фактическим составом разблокированных учётных записей в подключённых информационных системах;
 2. Автоматизированные отчёты (скрипты, задания по расписанию), сопоставляющие выгрузку из каталога (AD/LDAP) с данными кадровой системы и формирующие список расхождений для передачи ответственным лицам.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM).
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM).
 Иностранные: Microsoft Identity Manager, SailPoint IdentityIQ, One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: FreeIPA, midPoint и др.</t>
@@ -1365,16 +1385,16 @@
           <t>О-О-Т</t>
         </is>
       </c>
-      <c r="D7" s="131" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в контроле отсутствия в информационных системах незаблокированных учётных записей следующих категорий субъектов, фактически утративших основания для логического доступа:
+      <c r="D7" s="148" t="inlineStr">
+        <is>
+          <t>Мера предполагает контроль отсутствия в информационных системах незаблокированных учётных записей следующих категорий субъектов, фактически утративших основания для логического доступа:
 1. Уволенных работников;
 2. Работников, отсутствующих на рабочем месте более 90 календарных дней (например, в связи с длительным отпуском, отпуском по уходу за ребёнком, длительной болезнью);
 3. Работников внешних (подрядных) организаций, прекративших свою деятельность в организации (истёк срок договора, договор расторгнут, завершены работы).
 Главная цель меры — исключить существование «мёртвых» учётных записей, формально всё ещё активных, но принадлежащих субъектам, у которых больше нет законных оснований для доступа, поскольку такие учётные записи представляют собой канал несанкционированного доступа, использование которого крайне сложно связать с конкретным нарушителем.</t>
         </is>
       </c>
-      <c r="E7" s="132" t="inlineStr">
+      <c r="E7" s="149" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1385,7 +1405,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка информирования подразделения, ответственного за управление учётными записями, о наступлении перечисленных событий. Для этого необходимо:
+Со стороны организационных мер требуется регламентировать порядок информирования подразделения, ответственного за управление учётными записями, о наступлении перечисленных событий:
 1. Утвердить регламент взаимодействия кадровой службы, подразделений — заказчиков услуг подрядных организаций и подразделения информационной безопасности, определяющий сроки и порядок передачи сведений об увольнении, длительном отсутствии работника или прекращении деятельности подрядной организации;
 2. Установить предельный срок блокирования учётной записи с момента наступления события (например, не позднее следующего рабочего дня);
 3. Проводить периодические контрольные сверки перечня активных учётных записей с кадровыми данными и данными о завершённых договорах.</t>
@@ -1400,22 +1420,11 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает автоматизацию блокирования учётных записей при наступлении контролируемых событий. Для этого используются:
+В части технических средств необходимо автоматизировать блокирование учётных записей при наступлении контролируемых событий:
 1. Интеграция системы управления учётными записями (IdM, каталог) с кадровой системой для автоматического блокирования учётной записи при регистрации в кадровой системе факта увольнения или длительного отсутствия работника;
 2. Автоматизированный контроль срока действия учётных записей подрядных организаций, привязанный к дате окончания действия договора, с автоматическим блокированием по её наступлении;
 3. Регулярные автоматизированные отчёты (задания по расписанию) о неразблокированных учётных записях уволенных и длительно отсутствующих работников для оперативного реагирования.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM).
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM).
 Иностранные: Microsoft Identity Manager, SailPoint IdentityIQ и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: FreeIPA, midPoint и др.</t>
@@ -1483,13 +1492,13 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D8" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в периодическом контроле того, что в информационных системах отсутствуют разблокированные учётные записи, назначение которых невозможно однозначно определить — то есть учётные записи, не привязанные к конкретному субъекту логического доступа (работнику, представителю подрядной организации) или к документированному технологическому процессу.
+      <c r="D8" s="144" t="inlineStr">
+        <is>
+          <t>Данная мера касается контроля отсутствия в информационных системах разблокированных учётных записей, назначение которых невозможно однозначно определить — то есть учётных записей, не привязанных к конкретному субъекту логического доступа (работнику, представителю подрядной организации) или к документированному технологическому процессу.
 Главная цель меры — исключить существование «бесхозных» учётных записей с неясной принадлежностью и назначением, поскольку такие учётные записи не позволяют установить ответственного за их использование и создают неконтролируемый канал доступа, привлекательный для нарушителя.</t>
         </is>
       </c>
-      <c r="E8" s="134" t="inlineStr">
+      <c r="E8" s="150" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1500,7 +1509,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает проведение периодической инвентаризации учётных записей с определением назначения каждой из них. Для этого необходимо:
+Организационно это выражается в проведении периодической инвентаризации учётных записей с определением назначения каждой из них:
 1. Утвердить регламент, определяющий периодичность и порядок инвентаризации учётных записей (например, ежеквартально);
 2. В ходе инвентаризации для каждой активной учётной записи установить, принадлежит ли она конкретному субъекту логического доступа либо документированному технологическому процессу (сервисная, техническая учётная запись), и кто является ответственным за её использование;
 3. По итогам инвентаризации учётные записи, назначение которых установить не удалось, блокировать до выяснения обстоятельств, а результаты инвентаризации и принятые решения фиксировать в акте.</t>
@@ -1567,13 +1576,13 @@
           <t>Н-О-О</t>
         </is>
       </c>
-      <c r="D10" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в разработке и утверждении внутреннего документа, устанавливающего правила предоставления, отзыва и блокирования логического доступа субъектов к ресурсам доступа финансовой организации.
+      <c r="D10" s="144" t="inlineStr">
+        <is>
+          <t>Мера сводится к разработке и утверждению внутреннего документа, устанавливающего правила предоставления, отзыва и блокирования логического доступа субъектов к ресурсам доступа финансовой организации.
 Главная цель меры — обеспечить, чтобы процессы управления логическим доступом выполнялись по единым, заранее определённым и утверждённым правилам, а не по усмотрению отдельных сотрудников, что делает управление доступом предсказуемым, воспроизводимым и проверяемым.</t>
         </is>
       </c>
-      <c r="E10" s="126" t="inlineStr">
+      <c r="E10" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1584,7 +1593,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Мера реализуется исключительно организационными методами и предполагает разработку и утверждение внутреннего нормативного документа (например, положения или регламента по управлению логическим доступом), в котором закрепляются:
+Поскольку мера реализуется только организационными методами, её внедрение предполагает разработку и утверждение внутреннего нормативного документа (например, положения или регламента по управлению логическим доступом), в котором закрепляются:
 1. Порядок и основания предоставления логического доступа (инициирование заявки, согласование распорядителем логического доступа, фактическое предоставление прав);
 2. Порядок и основания отзыва ранее предоставленных прав логического доступа;
 3. Порядок и основания блокирования учётных записей (плановое — при увольнении, истечении срока доступа; внеплановое — при выявлении инцидента);
@@ -1641,13 +1650,13 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D11" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в назначении для каждого ресурса доступа (информационной системы, базы данных, сетевого ресурса, отдельной функции автоматизированной системы (АС)) распорядителя логического доступа — должностного лица (владельца ресурса), уполномоченного принимать решения о предоставлении, изменении и отзыве прав логического доступа к данному ресурсу.
+      <c r="D11" s="144" t="inlineStr">
+        <is>
+          <t>Смысл меры — в назначении для каждого ресурса доступа (информационной системы, базы данных, сетевого ресурса, отдельной функции автоматизированной системы (АС)) распорядителя логического доступа — должностного лица (владельца ресурса), уполномоченного принимать решения о предоставлении, изменении и отзыве прав логического доступа к данному ресурсу.
 Главная цель меры — обеспечить персональную ответственность за принятие решений о доступе к каждому конкретному ресурсу, поскольку без явно определённого распорядителя решения о предоставлении доступа принимаются бессистемно (например, только силами IT-подразделения), без учёта реальной необходимости доступа для выполнения бизнес-функций.</t>
         </is>
       </c>
-      <c r="E11" s="126" t="inlineStr">
+      <c r="E11" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1658,7 +1667,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает документальное закрепление распорядителей логического доступа для всех ресурсов доступа. Для этого необходимо:
+Организационная составляющая сводится к документальному закреплению распорядителей логического доступа для всех ресурсов доступа:
 1. Составить и поддерживать в актуальном состоянии перечень ресурсов доступа организации;
 2. Для каждого ресурса доступа определить и документально закрепить (приказом, распоряжением либо в положении о ресурсе) распорядителя логического доступа из числа руководителей подразделений, в чьей зоне ответственности находится соответствующий ресурс;
 3. Довести до распорядителей логического доступа их обязанности и ответственность за принятие решений о предоставлении, изменении и отзыве прав доступа к закреплённому ресурсу;
@@ -1713,13 +1722,13 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D12" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в том, что предоставление прав логического доступа к ресурсу осуществляется только на основании решения распорядителя логического доступа (владельца соответствующего ресурса доступа), назначенного в рамках меры УЗП.6.
+      <c r="D12" s="144" t="inlineStr">
+        <is>
+          <t>Мера устанавливает, что предоставление прав логического доступа к ресурсу осуществляется только на основании решения распорядителя логического доступа (владельца соответствующего ресурса доступа), назначенного в рамках меры УЗП.6.
 Главная цель меры — исключить предоставление прав доступа в обход лица, ответственного за ресурс, поскольку только распорядитель обладает необходимыми знаниями о служебной необходимости доступа для конкретного субъекта, а предоставление прав без его санкции ведёт к избыточному и неконтролируемому расширению доступа.</t>
         </is>
       </c>
-      <c r="E12" s="126" t="inlineStr">
+      <c r="E12" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1730,7 +1739,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка согласования заявок на предоставление логического доступа с распорядителем логического доступа. Для этого необходимо:
+В организационном плане реализация включает регламентацию порядка согласования заявок на предоставление логического доступа с распорядителем логического доступа:
 1. Установить обязательный порядок, при котором любое предоставление (изменение) прав логического доступа к ресурсу инициируется заявкой и требует явного согласования (утверждения) со стороны распорядителя логического доступа, закреплённого за данным ресурсом;
 2. Определить форму и способ фиксации решения распорядителя (подпись на бумажном носителе, согласование в системе электронного документооборота или service desk);
 3. Установить запрет на предоставление прав логического доступа администратором (исполнителем) без документально зафиксированного решения распорядителя;
@@ -1786,13 +1795,13 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D13" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в ведении эталонного (авторитетного) источника информации о фактически предоставленных субъектам правах логического доступа, а также в обеспечении целостности этой информации — то есть её защищённости от несанкционированного или бесконтрольного изменения.
+      <c r="D13" s="144" t="inlineStr">
+        <is>
+          <t>В основе меры лежит ведение эталонного (авторитетного) источника информации о фактически предоставленных субъектам правах логического доступа, а также обеспечение целостности этой информации — то есть её защищённости от несанкционированного или бесконтрольного изменения.
 Главная цель меры — обеспечить наличие достоверного и защищённого от подмены источника данных о предоставленных правах доступа, поскольку без такого эталона невозможно достоверно контролировать соответствие фактических прав доступа санкционированным (мера УЗП.9), а искажение эталонных данных способно скрыть факт несанкционированного расширения прав.</t>
         </is>
       </c>
-      <c r="E13" s="126" t="inlineStr">
+      <c r="E13" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1803,7 +1812,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка ведения и защиты эталонной информации о предоставленных правах логического доступа. Для этого необходимо:
+Со стороны организационных мер требуется регламентировать порядок ведения и защиты эталонной информации о предоставленных правах логического доступа:
 1. Определить источник (систему), являющийся эталонным хранилищем информации о предоставленных правах логического доступа (например, система IdM, реестр заявок на доступ);
 2. Установить порядок внесения изменений в эталонную информацию исключительно на основании документально оформленных и согласованных решений распорядителей логического доступа;
 3. Ограничить круг лиц, имеющих право вносить изменения в эталонную информацию, минимально необходимым составом;
@@ -1819,22 +1828,11 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает применение технических средств для хранения эталонной информации и контроля её целостности. Для этого используются:
+Технически это обеспечивается применением средств хранения эталонной информации и контроля её целостности:
 1. Хранение эталонной информации о предоставленных правах в специализированной системе (IdM, система управления доступом) с разграничением прав доступа к самой этой информации на уровне операционной системы и приложения;
 2. Технические механизмы контроля целостности данных (контрольные суммы, электронная подпись записей, версионирование изменений) с автоматическим выявлением фактов несанкционированного изменения эталонной информации;
 3. Регистрация в журнале событий всех операций изменения эталонной информации о предоставленных правах доступа.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM) со встроенным контролем целостности.
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM) со встроенным контролем целостности.
 Иностранные: SailPoint IdentityIQ, One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: midPoint и др.</t>
@@ -1902,13 +1900,13 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D14" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в периодическом сопоставлении фактических прав логического доступа, действующих в информационных системах, с эталонной информацией о предоставленных правах, которая ведётся и защищается в рамках меры УЗП.8.
+      <c r="D14" s="144" t="inlineStr">
+        <is>
+          <t>Мера заключается в периодическом сопоставлении фактических прав логического доступа, действующих в информационных системах, с эталонной информацией о предоставленных правах, которая ведётся и защищается в рамках меры УЗП.8.
 Главная цель меры — своевременно выявлять расхождения между тем, какие права доступа должны быть предоставлены субъекту согласно эталонным (санкционированным) данным, и тем, какие права фактически действуют в информационных системах, поскольку такие расхождения могут свидетельствовать как об ошибках администрирования, так и о несанкционированном изменении прав доступа.</t>
         </is>
       </c>
-      <c r="E14" s="126" t="inlineStr">
+      <c r="E14" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1919,7 +1917,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает проведение периодических ручных сверок фактических прав доступа с эталонной информацией. Для этого необходимо:
+Организационно мера реализуется через периодические ручные сверки фактических прав доступа с эталонной информацией:
 1. Утвердить регламент проведения сверки с указанием периодичности, перечня проверяемых ресурсов доступа и ответственных лиц;
 2. Провести сверку выгрузки фактических прав доступа из информационных систем с эталонной информацией;
 3. По фактам выявленных расхождений инициировать служебное разбирательство и корректировку прав доступа до соответствия эталонным данным;
@@ -1935,21 +1933,10 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает автоматизацию сверки фактических прав доступа с эталонными данными. Для этого используются:
+На техническом уровне сверку целесообразно автоматизировать:
 1. Средства автоматической сверки (recertification, access review), формирующие отчёты о расхождениях между эталонными данными системы IdM и фактическими правами, действующими в подключённых информационных системах;
 2. Настройка регулярных автоматических заданий (скриптов, коннекторов), сравнивающих выгрузку прав доступа из целевых систем с эталонным источником и оповещающих ответственных лиц о выявленных расхождениях.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM) с функцией пересертификации доступа.
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM) с функцией пересертификации доступа.
 Иностранные: SailPoint IdentityIQ, Saviynt и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: midPoint и др.</t>
@@ -2016,13 +2003,13 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D15" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в исключении технической возможности для пользователей самостоятельно, без санкции распорядителя логического доступа, расширять предоставленные им права логического доступа — то есть предоставлять себе дополнительные полномочия, изменять состав ролей, повышать уровень привилегий.
+      <c r="D15" s="144" t="inlineStr">
+        <is>
+          <t>Мера исключает техническую возможность для пользователей самостоятельно, без санкции распорядителя логического доступа, расширять предоставленные им права логического доступа — то есть предоставлять себе дополнительные полномочия, изменять состав ролей, повышать уровень привилегий.
 Главная цель меры — не допустить ситуации, при которой пользователь фактически становится собственным распорядителем доступа, поскольку возможность бесконтрольного самостоятельного расширения прав полностью обесценивает всю систему санкционирования доступа, реализованную в рамках мер УЗП.6 и УЗП.7.</t>
         </is>
       </c>
-      <c r="E15" s="135" t="inlineStr">
+      <c r="E15" s="152" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2033,22 +2020,11 @@
           </r>
           <r>
             <t xml:space="preserve">
-Поскольку мера реализуется только техническими методами, её внедрение предполагает настройку технических средств таким образом, чтобы пользователи не имели возможности самостоятельно изменять состав предоставленных им прав. Основные направления реализации:
+Ввиду сугубо технического характера меры её внедрение сводится к настройке технических средств таким образом, чтобы пользователи не имели возможности самостоятельно изменять состав предоставленных им прав:
 1. Разграничение полномочий на уровне операционных систем, СУБД и прикладного ПО, при котором функции управления собственными правами доступа (назначение ролей, изменение членства в группах, предоставление привилегий) недоступны обычным пользователям и закреплены исключительно за администраторами и системами управления доступом;
 2. Технический запрет на изменение пользователем собственных атрибутов в системе управления учётными записями (каталоге, IdM), связанных с правами доступа;
 3. Контроль целостности и регистрация попыток изменения параметров прав доступа с оповещением администратора безопасности при выявлении попытки самостоятельного расширения прав пользователем.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — средства защиты от несанкционированного доступа (СЗИ от НСД), системы управления учётными записями и правами доступа (IdM).
+Применимый класс средств — средства защиты от несанкционированного доступа (СЗИ от НСД), системы управления учётными записями и правами доступа (IdM).
 Иностранные: Microsoft Active Directory (разграничение делегирования прав), One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К, Avanpost IDM и др.
 Открытый код: FreeIPA, midPoint и др.</t>
@@ -2098,15 +2074,15 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D16" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в исключении технической возможности для пользователей бесконтрольно, без санкции уполномоченных лиц, изменять:
+      <c r="D16" s="144" t="inlineStr">
+        <is>
+          <t>Речь идёт об исключении технической возможности для пользователей бесконтрольно, без санкции уполномоченных лиц, изменять:
 1. Параметры настроек средств и систем защиты информации;
 2. Параметры настроек автоматизированных систем (АС), связанные с защитой информации.
 Главная цель меры — обеспечить целостность и контролируемость конфигураций всех защищаемых компонентов информационной инфраструктуры, исключив ситуации, когда изменение критических параметров безопасности может быть выполнено неуполномоченным лицом как умышленно, так и по ошибке.</t>
         </is>
       </c>
-      <c r="E16" s="126" t="inlineStr">
+      <c r="E16" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2117,23 +2093,12 @@
           </r>
           <r>
             <t xml:space="preserve">
-Поскольку мера реализуется только техническими методами, её внедрение предполагает разграничение прав доступа к параметрам настроек средств защиты информации и АС и контроль их изменения. Основные направления реализации:
+Так как мера реализуется только техническими средствами, необходимо разграничить права доступа к параметрам настроек средств защиты информации и АС и наладить контроль их изменения:
 1. Выделение привилегированных учётных записей с минимально необходимыми правами на изменение параметров настроек СЗИ и АС, использование ролевых моделей доступа;
 2. Технический запрет на изменение защищаемых параметров настроек для учётных записей обычных пользователей на уровне операционной системы, приложений и самих средств защиты информации;
 3. Принудительное применение эталонных параметров настроек средствами централизованного управления конфигурациями (например, групповыми политиками) с автоматическим выявлением и блокированием отклонений;
 4. Регистрация всех попыток изменения защищаемых параметров настроек в журнале событий средства защиты информации или операционной системы.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — средства защиты от несанкционированного доступа (СЗИ от НСД), системы управления конфигурациями и контроля целостности.
+Применимый класс средств — средства защиты от несанкционированного доступа (СЗИ от НСД), системы управления конфигурациями и контроля целостности.
 Иностранные: Tripwire Enterprise, Microsoft Group Policy (AD GPO), Ivanti Endpoint Manager и пр.
 Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К, ViPNet Coordinator и др.
 Открытый код: Osquery, OSSEC и др.</t>
@@ -2181,13 +2146,13 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D17" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в контроле того, что при изменении должностных обязанностей субъекта логического доступа (перевод на другую должность, изменение зоны ответственности, временное исполнение обязанностей по другой должности) проводится анализ необходимости отзыва ранее предоставленных ему прав доступа, переставших соответствовать новым обязанностям.
+      <c r="D17" s="144" t="inlineStr">
+        <is>
+          <t>Мера обязывает контролировать необходимость отзыва прав субъекта логического доступа при изменении его должностных обязанностей (перевод на другую должность, изменение зоны ответственности, временное исполнение обязанностей по другой должности).
 Главная цель меры — не допустить накопления у субъекта избыточных прав доступа при должностных перемещениях внутри организации, поскольку без такого контроля права доступа со временем только добавляются, но не отзываются, что приводит к формированию у отдельных сотрудников чрезмерно широкого, несоответствующего текущим обязанностям набора полномочий.</t>
         </is>
       </c>
-      <c r="E17" s="126" t="inlineStr">
+      <c r="E17" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2198,7 +2163,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка контроля прав доступа при кадровых перемещениях. Для этого необходимо:
+Организационно это выражается в регламентации порядка контроля прав доступа при кадровых перемещениях:
 1. Установить обязанность подразделения, ответственного за управление учётными записями (или распорядителя логического доступа), проводить анализ ранее предоставленных прав доступа субъекта при получении сведений об изменении его должностных обязанностей;
 2. Определить порядок и сроки проведения такого анализа с момента получения кадровой информации об изменении должности (перевода);
 3. По результатам анализа инициировать отзыв прав доступа, не соответствующих новым должностным обязанностям, и предоставление новых прав при необходимости;
@@ -2253,13 +2218,13 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D18" s="137" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в контроле того, что логический доступ, предоставленный субъекту на определённый период (срок) — например, для выполнения временных задач, представителям подрядных организаций на срок действия договора, — фактически прекращается, а соответствующая учётная запись блокируется по истечении установленного срока.
+      <c r="D18" s="153" t="inlineStr">
+        <is>
+          <t>Суть меры — в контроле того, что логический доступ, предоставленный субъекту на определённый период (срок) — например, для выполнения временных задач, представителям подрядных организаций на срок действия договора, — фактически прекращается, а соответствующая учётная запись блокируется по истечении установленного срока.
 Главная цель меры — исключить продолжение действия прав логического доступа после истечения оснований, на которых эти права были предоставлены, поскольку доступ, предоставленный на ограниченный срок, но не прекращённый по его истечении, фактически превращается в бессрочный и бесконтрольный.</t>
         </is>
       </c>
-      <c r="E18" s="138" t="inlineStr">
+      <c r="E18" s="154" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2270,7 +2235,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка контроля сроков предоставленного доступа. Для этого необходимо:
+С организационной стороны мера реализуется через регламентацию порядка контроля сроков предоставленного доступа:
 1. Установить обязательное указание срока действия прав логического доступа в заявке на предоставление доступа для всех случаев срочного (временного) доступа;
 2. Определить ответственных за контроль соблюдения указанных сроков и порядок их действий по истечении срока (блокирование учётной записи, продление доступа по обоснованной заявке);
 3. Проводить периодические проверки перечня учётных записей с истёкшим сроком предоставленного доступа на предмет фактического блокирования.</t>
@@ -2285,22 +2250,11 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает автоматизацию контроля и применения ограничения сроков действия доступа. Для этого используются:
+Технически контроль сроков и применение ограничений реализуются так:
 1. Установка технического срока действия учётной записи (account expiration) или отдельных прав доступа непосредственно при их предоставлении в информационной системе или системе управления доступом (IdM, каталог);
 2. Автоматическое блокирование учётной записи или отзыв прав доступа средствами информационной системы по наступлении установленной даты без необходимости ручного вмешательства;
 3. Автоматизированные отчёты (оповещения) о приближающемся или наступившем истечении срока предоставленного доступа для ответственных лиц.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM), службы каталогов.
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM), службы каталогов.
 Иностранные: Microsoft Active Directory (срок действия учётной записи), One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: FreeIPA, midPoint и др.</t>
@@ -2375,7 +2329,7 @@
 Главная цель меры — своевременно выявлять «мёртвые» учётные записи и избыточные права доступа.</t>
         </is>
       </c>
-      <c r="E19" s="138" t="inlineStr">
+      <c r="E19" s="154" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2386,7 +2340,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает проведение периодических ручных проверок с использованием отчётов из систем учёта доступа. Для этого формируются протоколы (акты) о субъектах, которые не осуществляли логический доступ в течение 90 и более дней, по итогам которых распорядителями логического доступа принимается решение о целесообразности дальнейшего предоставления неиспользуемых прав (см. меру УЗП.16).</t>
+Организационно мера реализуется через периодические ручные проверки с использованием отчётов из систем учёта доступа: формируются протоколы (акты) о субъектах, которые не осуществляли логический доступ в течение 90 и более дней, по итогам которых распорядителями логического доступа принимается решение о целесообразности дальнейшего предоставления неиспользуемых прав (см. меру УЗП.16).</t>
           </r>
           <r>
             <rPr>
@@ -2398,19 +2352,8 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает настройку сбора и хранения событий аутентификации и авторизации (успешные и неудачные входы, использование прав доступа, запуск привилегированных команд) в системных журналах, базе данных Active Directory или специализированных системах управления доступом. Для автоматизированного выявления неиспользуемых прав применяются средства анализа журналов или SIEM-системы, формирующие отчёты по учётным записям с отсутствием активности за период, превышающий 90 дней.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM), средства анализа журналов и SIEM.
+На техническом уровне необходима настройка сбора и хранения событий аутентификации и авторизации (успешные и неудачные входы, использование прав доступа, запуск привилегированных команд) в системных журналах, базе данных Active Directory или специализированных системах управления доступом. Для автоматизированного выявления неиспользуемых прав применяются средства анализа журналов или SIEM-системы, формирующие отчёты по учётным записям с отсутствием активности за период, превышающий 90 дней.
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM), средства анализа журналов и SIEM.
 Иностранные: Microsoft Active Directory, ManageEngine ADManager Plus, SolarWinds Access Rights Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: Osquery, Graylog и др.</t>
@@ -2473,13 +2416,13 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D20" s="137" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в выявлении учётных записей и прав логического доступа, которые были предоставлены субъектам, но фактически не использовались ими на протяжении периода, превышающего 45 дней. Мера аналогична УЗП.14, но применяется к более короткому контрольному периоду и, в отличие от УЗП.14, требует исключительно технической (автоматизированной) реализации.
+      <c r="D20" s="153" t="inlineStr">
+        <is>
+          <t>Как и УЗП.14, данная мера направлена на выявление учётных записей и прав логического доступа, которые были предоставлены субъектам, но фактически не использовались ими — только контрольный период здесь короче (45, а не 90 дней), и, в отличие от УЗП.14, мера требует исключительно технической (автоматизированной) реализации.
 Главная цель меры — обеспечить более оперативное, чем в рамках УЗП.14, выявление неиспользуемых прав доступа для организаций (уровней защиты), где повышенные требования к оперативности контроля не позволяют полагаться на периодические ручные проверки.</t>
         </is>
       </c>
-      <c r="E20" s="138" t="inlineStr">
+      <c r="E20" s="154" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2490,22 +2433,11 @@
           </r>
           <r>
             <t xml:space="preserve">
-Поскольку мера реализуется только техническими методами, её внедрение предполагает автоматизированный, без участия оператора, контроль активности использования прав логического доступа. Основные направления реализации:
+Поскольку организационные меры здесь неприменимы, реализация строится исключительно на автоматизированном, без участия оператора, контроле активности использования прав логического доступа:
 1. Автоматизированный сбор и хранение событий аутентификации и авторизации (успешные и неудачные входы, использование прав доступа) в журналах информационных систем, каталоге (AD/LDAP) или системе управления доступом;
 2. Автоматическое формирование средствами анализа журналов или SIEM-системой перечня учётных записей, не проявлявших активности на протяжении более 45 дней, без необходимости запуска проверки вручную;
 3. Автоматическое оповещение ответственных лиц (администратора безопасности, распорядителя логического доступа) о выявленных фактах неиспользования прав для принятия решения в рамках меры УЗП.16.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM), средства анализа журналов и SIEM.
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM), средства анализа журналов и SIEM.
 Иностранные: Microsoft Active Directory, SolarWinds Access Rights Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: Osquery, Graylog и др.</t>
@@ -2559,13 +2491,13 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D21" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в том, что по фактам неиспользования прав логического доступа, выявленным в рамках мер УЗП.14 и УЗП.15, распорядитель логического доступа (владелец ресурса доступа) проводит анализ и принимает решение о целесообразности дальнейшего предоставления субъекту этих прав.
+      <c r="D21" s="144" t="inlineStr">
+        <is>
+          <t>Мера предусматривает, что по фактам неиспользования прав логического доступа, выявленным в рамках мер УЗП.14 и УЗП.15, распорядитель логического доступа (владелец ресурса доступа) проводит анализ и принимает решение о целесообразности дальнейшего предоставления субъекту этих прав.
 Главная цель меры — обеспечить, чтобы выявление неиспользуемых прав доступа не оставалось формальной процедурой без последствий, а завершалось содержательным решением лица, ответственного за ресурс: сохранить права за субъектом (при наличии обоснованной необходимости) либо отозвать их как избыточные.</t>
         </is>
       </c>
-      <c r="E21" s="126" t="inlineStr">
+      <c r="E21" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2576,7 +2508,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка рассмотрения распорядителем логического доступа фактов, выявленных в рамках мер УЗП.14 и УЗП.15. Для этого необходимо:
+Поскольку мера реализуется только организационными методами, требуется регламентировать порядок рассмотрения распорядителем логического доступа фактов, выявленных в рамках мер УЗП.14 и УЗП.15:
 1. Установить обязанность передачи распорядителю логического доступа перечня неиспользуемых прав, выявленных по конкретному ресурсу доступа, с определённой периодичностью;
 2. Установить срок, в течение которого распорядитель обязан рассмотреть полученные сведения и принять решение (сохранить права, отозвать права, запросить обоснование у субъекта);
 3. Зафиксировать порядок документального оформления принятого решения и передачи его для исполнения (отзыва прав) подразделению, ответственному за управление доступом;
@@ -2632,13 +2564,13 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D22" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в обеспечении технической и организационной возможности в любой момент времени однозначно определить полный состав субъектов и прав логического доступа, предоставленных к конкретному ресурсу доступа (информационной системе, базе данных, сетевому ресурсу).
+      <c r="D22" s="144" t="inlineStr">
+        <is>
+          <t>Мера обеспечивает техническую и организационную возможность в любой момент времени однозначно определить полный состав субъектов и прав логического доступа, предоставленных к конкретному ресурсу доступа (информационной системе, базе данных, сетевому ресурсу).
 Главная цель меры — дать распорядителю логического доступа, подразделению информационной безопасности и внешним проверяющим возможность оперативно получить достоверный ответ на вопрос «кто и какими правами обладает в отношении данного ресурса», без чего невозможны ни контроль соответствия прав эталонной информации (УЗП.9), ни расследование инцидентов, связанных с этим ресурсом.</t>
         </is>
       </c>
-      <c r="E22" s="126" t="inlineStr">
+      <c r="E22" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2649,7 +2581,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка получения сведений о составе предоставленных прав доступа к ресурсу. Для этого необходимо:
+Организационно это выражается в регламентации порядка получения сведений о составе предоставленных прав доступа к ресурсу:
 1. Определить порядок и сроки предоставления по запросу распорядителя логического доступа, подразделения информационной безопасности или проверяющих лиц выгрузки (отчёта) о составе субъектов и прав доступа к конкретному ресурсу;
 2. Закрепить ответственного (администратора ресурса или системы управления доступом) за формирование такой выгрузки.</t>
           </r>
@@ -2663,21 +2595,10 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает наличие в информационной системе или системе управления доступом функции формирования отчёта о правах доступа в разрезе ресурса. Для этого используются:
+Технически это требует наличия в информационной системе или системе управления доступом функции формирования отчёта о правах доступа в разрезе ресурса:
 1. Встроенные средства информационной системы (АС, СУБД) или системы управления учётными записями и правами доступа (IdM), позволяющие сформировать перечень субъектов и предоставленных им прав для выбранного ресурса доступа;
 2. Средства выгрузки списков контроля доступа (ACL) сетевого оборудования, файловых ресурсов и иных технических ресурсов доступа.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM), средства защиты от НСД со встроенной отчётностью.
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM), средства защиты от НСД со встроенной отчётностью.
 Иностранные: SailPoint IdentityIQ, Netwrix Access Analyzer и пр.
 Российские сертифицированные (ФСТЭК): Secret Net Studio, Avanpost IDM, Solar inRights и др.
 Открытый код: midPoint и др.</t>
@@ -2743,13 +2664,13 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D23" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в обеспечении технической и организационной возможности в любой момент времени однозначно определить полный состав ресурсов доступа и прав логического доступа, предоставленных конкретному субъекту (работнику, представителю эксплуатационного персонала).
+      <c r="D23" s="144" t="inlineStr">
+        <is>
+          <t>Зеркально мере УЗП.17, данная мера обеспечивает техническую и организационную возможность в любой момент времени однозначно определить полный состав ресурсов доступа и прав логического доступа, предоставленных конкретному субъекту (работнику, представителю эксплуатационного персонала).
 Главная цель меры — дать распорядителям логического доступа и подразделению информационной безопасности возможность оперативно получить достоверный ответ на вопрос «какими правами доступа в отношении каких ресурсов обладает данный субъект», что необходимо как для контроля обоснованности объёма прав (принцип минимально необходимых прав), так и для оперативного реагирования на инциденты, связанные с конкретным субъектом.</t>
         </is>
       </c>
-      <c r="E23" s="126" t="inlineStr">
+      <c r="E23" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2760,7 +2681,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает регламентацию порядка получения сведений о составе прав доступа субъекта. Для этого необходимо:
+С организационной стороны требуется регламентировать порядок получения сведений о составе прав доступа субъекта:
 1. Определить порядок и сроки предоставления по запросу руководителя субъекта, распорядителей логического доступа или подразделения информационной безопасности выгрузки (отчёта) о составе ресурсов доступа и прав, предоставленных конкретному субъекту;
 2. Закрепить ответственного (подразделение, отвечающее за управление учётными записями) за формирование такой выгрузки.</t>
           </r>
@@ -2774,21 +2695,10 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает наличие в системе управления учётными записями и правами доступа функции формирования сводного отчёта о правах конкретного субъекта. Для этого используются:
+На техническом уровне требуется наличие в системе управления учётными записями и правами доступа функции формирования сводного отчёта о правах конкретного субъекта:
 1. Система класса IdM, консолидирующая сведения о правах доступа субъекта во всех подключённых информационных системах и позволяющая сформировать единый («профильный») отчёт по конкретной учётной записи;
 2. При отсутствии централизованной системы IdM — совокупность встроенных средств формирования отчётов в каждой отдельной информационной системе.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM).
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM).
 Иностранные: SailPoint IdentityIQ, One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: midPoint и др.</t>
@@ -2854,16 +2764,16 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D24" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в:
-1. Определении состава ролей логического доступа, связанных с непосредственным выполнением операций (транзакций) в автоматизированных системах (АС), имеющих финансовые последствия для финансовой организации, её клиентов и контрагентов;
-2. Определении состава ролей, связанных с контролем выполнения указанных операций (транзакций);
-3. Установлении запрета на совмещение указанных ролей одним и тем же субъектом логического доступа.
+      <c r="D24" s="144" t="inlineStr">
+        <is>
+          <t>Мера охватывает сразу три взаимосвязанных требования:
+1. Определение состава ролей логического доступа, связанных с непосредственным выполнением операций (транзакций) в автоматизированных системах (АС), имеющих финансовые последствия для финансовой организации, её клиентов и контрагентов;
+2. Определение состава ролей, связанных с контролем выполнения указанных операций (транзакций);
+3. Установление запрета на совмещение указанных ролей одним и тем же субъектом логического доступа.
 Главная цель меры — реализовать принцип разделения обязанностей (segregation of duties) применительно к финансово значимым операциям: не допустить ситуации, при которой один и тот же субъект одновременно совершает операцию и контролирует её выполнение, поскольку совмещение этих ролей делает контроль фиктивным и создаёт условия для совершения и сокрытия мошеннических действий.</t>
         </is>
       </c>
-      <c r="E24" s="126" t="inlineStr">
+      <c r="E24" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2874,7 +2784,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает документальное определение состава ролей и закрепление запрета на их совмещение. Для этого необходимо:
+Организационно мера реализуется через документальное определение состава ролей и закрепление запрета на их совмещение:
 1. Совместно с владельцами бизнес-процессов и распорядителями логического доступа провести анализ автоматизированных систем и операций (транзакций), имеющих финансовые последствия для организации, клиентов и контрагентов;
 2. Сформировать и утвердить перечень ролей логического доступа, связанных с выполнением таких операций, и отдельно — перечень ролей, связанных с контролем их выполнения;
 3. Закрепить во внутреннем нормативном документе прямой запрет на предоставление одному субъекту логического доступа ролей из обеих категорий одновременно;
@@ -2890,21 +2800,10 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает применение технических средств для контроля состава ролей и недопущения их совмещения. Для этого используются:
+Технические средства применяются для контроля состава ролей и недопущения их совмещения:
 1. Ролевая модель управления доступом (RBAC), реализованная в АС или системе управления доступом (IdM), в которой роли, связанные с выполнением и с контролем финансово значимых операций, технически обособлены друг от друга;
 2. Функционал контроля разделения полномочий (Segregation of Duties, SoD), встроенный в систему IdM или GRC-платформу, автоматически выявляющий и блокирующий попытки предоставления субъекту конфликтующих ролей.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM) и GRC-платформы с функцией контроля разделения полномочий (SoD).
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM) и GRC-платформы с функцией контроля разделения полномочий (SoD).
 Иностранные: SAP GRC Access Control, SailPoint IdentityIQ и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights (с модулем контроля SoD) и др.
 Открытый код: midPoint и др.</t>
@@ -2972,13 +2871,13 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D25" s="124" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в практической реализации в процессах управления логическим доступом правил, обеспечивающих соблюдение запрета на совмещение одним субъектом ролей выполнения и контроля финансово значимых операций, состав которых определён в рамках меры УЗП.19.
-Главная цель меры — обеспечить, чтобы запрет на совмещение ролей, зафиксированный документально в рамках УЗП.19, реально соблюдался на всех этапах жизненного цикла прав доступа — при первичном предоставлении доступа, при последующих изменениях и при периодическом контроле, а не оставался декларацией, не подкреплённой действующими процедурами управления доступом.</t>
-        </is>
-      </c>
-      <c r="E25" s="126" t="inlineStr">
+      <c r="D25" s="144" t="inlineStr">
+        <is>
+          <t>Мера переводит в практическую плоскость запрет на совмещение одним субъектом ролей выполнения и контроля финансово значимых операций, состав которых определён в рамках меры УЗП.19.
+Главная цель меры — обеспечить, чтобы этот запрет реально соблюдался на всех этапах жизненного цикла прав доступа — при первичном предоставлении доступа, при последующих изменениях и при периодическом контроле, а не оставался декларацией, не подкреплённой действующими процедурами управления доступом.</t>
+        </is>
+      </c>
+      <c r="E25" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2989,7 +2888,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает встраивание проверки соблюдения запрета на совмещение ролей в процессы предоставления и изменения прав логического доступа. Для этого необходимо:
+С организационной стороны требуется встроить проверку соблюдения запрета на совмещение ролей в процессы предоставления и изменения прав логического доступа:
 1. Установить обязательную проверку заявки на предоставление (изменение) прав логического доступа на предмет потенциального конфликта с ролями, предусмотренными мерой УЗП.19, до её согласования распорядителем логического доступа;
 2. Определить порядок действий при выявлении конфликта ролей (отказ в предоставлении, требование обоснования и утверждения компенсирующей меры на уровне руководства);
 3. Периодически проводить ручные проверки фактического состава ролей субъектов на предмет соблюдения запрета совмещения.</t>
@@ -3004,21 +2903,10 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает автоматизацию проверки заявок и фактических прав доступа на предмет конфликта ролей. Для этого используются:
+Технически проверку заявок и фактических прав доступа на предмет конфликта ролей целесообразно автоматизировать:
 1. Автоматическая проверка каждой заявки на предоставление или изменение прав логического доступа на предмет конфликта с ролями, предусмотренными мерой УЗП.19, средствами системы IdM или GRC-платформы, с технической блокировкой предоставления конфликтующих прав;
 2. Периодические автоматизированные проверки (recertification) фактического состава прав всех субъектов на предмет выявления совмещения ролей, с формированием отчёта о выявленных конфликтах.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM) и GRC-платформы с функцией контроля разделения полномочий (SoD).
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM) и GRC-платформы с функцией контроля разделения полномочий (SoD).
 Иностранные: SAP GRC Access Control, SailPoint IdentityIQ и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights (с модулем контроля SoD) и др.
 Открытый код: midPoint и др.</t>
@@ -3090,9 +2978,9 @@
           <t>Н-О-Т</t>
         </is>
       </c>
-      <c r="D26" s="141" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в реализации правил управления правами логического доступа, обеспечивающих запрет на совмещение одним субъектом логического доступа следующих несовместимых функций:
+      <c r="D26" s="155" t="inlineStr">
+        <is>
+          <t>Мера закрепляет запрет на совмещение одним субъектом логического доступа следующих несовместимых функций:
 1. Эксплуатация и (или) контроль эксплуатации ресурса доступа, в том числе АС, одновременно с использованием этого же ресурса по назначению в рамках бизнес-процесса финансовой организации;
 2. Создание и (или) модернизация ресурса доступа, в том числе АС, одновременно с использованием этого же ресурса по назначению в рамках бизнес-процесса финансовой организации;
 3. Эксплуатация средств и систем защиты информации одновременно с контролем эксплуатации средств и систем защиты информации;
@@ -3100,7 +2988,7 @@
 Главная цель меры — реализовать принцип разделения обязанностей в отношении технического персонала и администраторов: не допустить сосредоточения в руках одного субъекта функций, взаимный контроль которых является необходимым элементом системы защиты информации, поскольку их совмещение позволяет субъекту скрыть собственные неправомерные действия.</t>
         </is>
       </c>
-      <c r="E26" s="126" t="inlineStr">
+      <c r="E26" s="151" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3111,7 +2999,7 @@
           </r>
           <r>
             <t xml:space="preserve">
-Организационная реализация предполагает документальное закрепление и соблюдение перечисленных запретов при формировании штатной структуры и распределении обязанностей. Для этого необходимо:
+Организационная составляющая сводится к документальному закреплению и соблюдению перечисленных запретов при формировании штатной структуры и распределении обязанностей:
 1. Закрепить во внутреннем нормативном документе перечень несовместимых функций, приведённый в описании меры;
 2. При формировании должностных инструкций и распределении обязанностей между сотрудниками (подразделениями) обеспечивать, чтобы ни один субъект не наделялся одновременно взаимоисключающими функциями;
 3. При предоставлении прав логического доступа проверять заявку на предмет соответствия установленным запретам до её согласования распорядителем логического доступа;
@@ -3127,23 +3015,12 @@
           </r>
           <r>
             <t xml:space="preserve">
-Техническая реализация предполагает разграничение прав логического доступа таким образом, чтобы техническая возможность совмещения перечисленных функций у одного субъекта отсутствовала. Для этого используются:
+Технически права логического доступа разграничиваются так, чтобы возможность совмещения перечисленных функций у одного субъекта отсутствовала:
 1. Ролевая модель управления доступом, в которой роли администрирования ресурсов доступа (АС) и роли их использования по назначению технически обособлены и не могут быть назначены одному субъекту;
 2. Ролевая модель, разделяющая права на эксплуатацию средств и систем защиты информации и права на контроль (аудит) их эксплуатации;
 3. Техническое разделение функций управления учётными записями (создание, блокирование) и функций управления правами доступа (назначение ролей, прав) между разными субъектами на уровне системы управления доступом (IdM);
 4. Функционал контроля разделения полномочий (SoD) в IdM/GRC-платформе, автоматически выявляющий и блокирующий попытки назначения субъекту несовместимых функций.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <t xml:space="preserve">
-Класс средств — системы управления учётными записями и правами доступа (IdM) и GRC-платформы с функцией контроля разделения полномочий (SoD).
+Применимый класс средств — системы управления учётными записями и правами доступа (IdM) и GRC-платформы с функцией контроля разделения полномочий (SoD).
 Иностранные: SAP GRC Access Control, One Identity Manager и пр.
 Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
 Открытый код: midPoint и др.</t>
@@ -22891,8 +22768,8 @@
     <mergeCell ref="A423:G423"/>
     <mergeCell ref="A174:G174"/>
     <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="A309:G309"/>
-    <mergeCell ref="A1:A2"/>
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A84:G84"/>
     <mergeCell ref="A286:G286"/>

</xml_diff>

<commit_message>
Fill РД.1-РД.29 (list «1. Описание мер», rows 37-66) per VIKI_measure_filling_rules.md
- 17 measures with all of D-G written from scratch: РД.1, РД.3-12,
  РД.17, РД.24, РД.26-29
- 10 measures with a pre-existing D kept, E/F/G added: РД.2, РД.13-15,
  РД.19-23, РД.25
- РД.16, РД.18: fixed defects in the pre-existing D (stray trailing
  period; a grammar error that also silently dropped the measure's
  second requirement — передача аутентификационных данных куда-либо,
  кроме средств аутентификации) before adding E/F/G
- D/E opening phrasing varied per measure (not a fixed template) per
  house-style feedback; technical examples name the tool class before
  listing products
- H flagged on РД.5 (PKI/СКЗИ certification is FSB's, not FSTEC's,
  domain)
- All filled/rewritten cells shaded pale yellow for review; untouched
  cells keep their existing formatting
</commit_message>
<xml_diff>
--- a/docs/WIKI GOST R 57580.1.xlsx
+++ b/docs/WIKI GOST R 57580.1.xlsx
@@ -334,7 +334,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -793,6 +793,10 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -3767,10 +3771,60 @@
           <t>Т-Т-Н</t>
         </is>
       </c>
-      <c r="D37" s="21" t="n"/>
-      <c r="E37" s="31" t="n"/>
-      <c r="F37" s="31" t="n"/>
-      <c r="G37" s="31" t="n"/>
+      <c r="D37" s="144" t="inlineStr">
+        <is>
+          <t>Мера устанавливает базовое требование: перед предоставлением логического доступа пользователь должен пройти идентификацию (предъявление уникального идентификатора — логина, номера учётной записи) и однофакторную аутентификацию (подтверждение подлинности с использованием одного фактора — как правило, пароля).
+Главная цель меры — исключить анонимный или неаутентифицированный доступ к ресурсам финансовой организации: без этой базовой процедуры невозможно связать действия в системе с конкретным субъектом, а любые более сложные меры защиты логического доступа (в том числе разграничение прав) теряют смысл.</t>
+        </is>
+      </c>
+      <c r="E37" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера носит сугубо технический характер, её внедрение сводится к настройке штатных механизмов идентификации и аутентификации:
+1. Настройка операционных систем, СУБД, прикладного программного обеспечения (ПО) и сетевого оборудования таким образом, чтобы вход в систему был невозможен без предъявления уникального идентификатора и прохождения проверки подлинности (пароля);
+2. Централизованное управление учётными данными через каталог (Active Directory, LDAP) либо локальные механизмы аутентификации для систем, не подключённых к каталогу;
+3. Технический запрет анонимного доступа и доступа без прохождения процедуры аутентификации.
+Применимый класс средств — операционные системы и прикладное ПО со встроенными механизмами идентификации и аутентификации, службы каталогов, средства защиты от несанкционированного доступа (СЗИ от НСД).
+Иностранные: Microsoft Active Directory, Cisco ISE (для сетевого доступа) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К и др.
+Открытый код: FreeIPA, OpenLDAP и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F37" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек, подтверждающие обязательность идентификации и аутентификации при входе в информационные системы;
+3. Результаты тестирования (попытка входа без учётных данных или под неизвестным идентификатором), подтверждающие невозможность анонимного доступа;
+4. Журналы событий, подтверждающие регистрацию фактов идентификации и аутентификации пользователей.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G37" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные информационные системы или сервисы допускают вход без идентификации и аутентификации (например, тестовые или устаревшие системы);
+2. Идентификация не является уникальной — несколько пользователей используют один и тот же идентификатор;
+3. Настройки, требующие обязательной аутентификации, применены не на всех точках входа (например, отсутствуют на резервных или альтернативных интерфейсах доступа);
+4. Отсутствует регистрация фактов идентификации и аутентификации, что не позволяет подтвердить соблюдение меры.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="213.75" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
@@ -3794,9 +3848,55 @@
 Главная цель меры — значительно повысить уровень защищённости процесса аутентификации по сравнению с однофакторными методами (например, только паролем). Даже если один из факторов будет скомпрометирован (например, пароль украден), злоумышленник не сможет получить доступ, так как ему потребуется предъявить второй (и/или третий) независимый фактор.</t>
         </is>
       </c>
-      <c r="E38" s="31" t="n"/>
-      <c r="F38" s="31" t="n"/>
-      <c r="G38" s="31" t="n"/>
+      <c r="E38" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит чисто технический характер и включает:
+1. Настройку систем многофакторной аутентификации (МФА), требующих последовательного предъявления как минимум двух независимых факторов (например, пароль и одноразовый код, пароль и аппаратный токен, пароль и биометрия);
+2. Интеграцию средств МФА со всеми информационными системами контура безопасности, к которым пользователи осуществляют логический доступ, включая удалённый доступ (VPN, терминальные сессии);
+3. Технический запрет входа в систему при успешном прохождении только одного из факторов;
+4. Регистрацию событий прохождения (и неуспешных попыток прохождения) многофакторной аутентификации.
+Класс используемых средств — средства многофакторной аутентификации (МФА).
+Иностранные: RSA SecurID, Duo Security и пр.
+Российские сертифицированные (ФСТЭК): «Мультифактор», JaCarta (программные компоненты), Рутокен (в связке с ПО аутентификации) и др.
+Открытый код: privacyIDEA и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F38" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами систем аутентификации;
+2. Скриншоты настроек систем МФА, подтверждающие требование не менее двух факторов для входа пользователей;
+3. Результаты тестирования (попытка входа с предъявлением только одного фактора), подтверждающие блокирование такого входа;
+4. Журналы событий, подтверждающие успешные и неуспешные попытки многофакторной аутентификации пользователей.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G38" s="151" t="inlineStr">
+        <is>
+          <t>1. МФА подключена не ко всем информационным системам, к которым пользователи осуществляют логический доступ (например, отсутствует для удалённого доступа);
+2. Отдельные категории пользователей исключены из периметра действия МФА без документированного обоснования;
+3. В качестве второго фактора используется метод, не являющийся независимым от первого (например, код приходит на то же устройство, с которого вводится пароль, без дополнительной защиты канала);
+4. Технически возможен обход МФА через альтернативные точки входа (legacy-интерфейсы, API), не охваченные требованием.</t>
+        </is>
+      </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -3819,10 +3919,60 @@
           <t>Т-Н-Н</t>
         </is>
       </c>
-      <c r="D39" s="21" t="n"/>
-      <c r="E39" s="31" t="n"/>
-      <c r="F39" s="31" t="n"/>
-      <c r="G39" s="31" t="n"/>
+      <c r="D39" s="144" t="inlineStr">
+        <is>
+          <t>Мера — зеркальное отражение РД.1, но применительно к эксплуатационному персоналу: перед предоставлением логического доступа представитель эксплуатационного персонала (администратор) должен пройти идентификацию и однофакторную аутентификацию.
+Главная цель меры — обеспечить минимально необходимый уровень контроля доступа для технического персонала на тех уровнях защиты, где многофакторная аутентификация для этой категории субъектов (мера РД.4) ещё не требуется, не допуская анонимного администрирования систем.</t>
+        </is>
+      </c>
+      <c r="E39" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера подразумевает исключительно технические меры защиты, а именно:
+1. Настройку операционных систем, СУБД, средств виртуализации, сетевого оборудования и средств защиты информации таким образом, чтобы административный доступ был невозможен без предъявления уникального идентификатора и прохождения проверки подлинности;
+2. Использование персональных привилегированных учётных записей для каждого представителя эксплуатационного персонала (без общих административных учётных записей — см. также меру РД.10);
+3. Технический запрет анонимного или неаутентифицированного административного доступа ко всем управляемым компонентам инфраструктуры.
+Класс используемых средств — операционные системы, средства виртуализации и сетевое оборудование со встроенными механизмами идентификации и аутентификации, системы управления привилегированным доступом (PAM).
+Иностранные: Microsoft Active Directory, CyberArk PAM и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Indeed Privileged Access Manager и др.
+Открытый код: FreeIPA, Teleport и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F39" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем и подразделением информационной безопасности;
+2. Скриншоты настроек, подтверждающие обязательность идентификации и аутентификации при административном доступе;
+3. Выгрузка перечня учётных записей эксплуатационного персонала, подтверждающая их персональный (не групповой) характер;
+4. Журналы событий, подтверждающие регистрацию фактов идентификации и аутентификации эксплуатационного персонала.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G39" s="151" t="inlineStr">
+        <is>
+          <t>1. Часть оборудования (сетевые устройства, гипервизоры, встроенные консоли управления) администрируется без персональной идентификации, через общую учётную запись производителя по умолчанию;
+2. Для отдельных унаследованных систем аутентификация технически не реализована и компенсируется только организационными мерами;
+3. Журналы идентификации и аутентификации эксплуатационного персонала не собираются централизованно;
+4. Отсутствует контроль за тем, что все административные интерфейсы (включая консольный и физический доступ) охвачены требованием аутентификации.</t>
+        </is>
+      </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -3845,10 +3995,61 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D40" s="21" t="n"/>
-      <c r="E40" s="31" t="n"/>
-      <c r="F40" s="31" t="n"/>
-      <c r="G40" s="31" t="n"/>
+      <c r="D40" s="144" t="inlineStr">
+        <is>
+          <t>Мера аналогична РД.2, но распространяется на эксплуатационный персонал: администраторы и иные представители эксплуатационного персонала обязаны проходить многофакторную аутентификацию для получения логического доступа к управляемым ими системам.
+Главная цель меры — усилить защиту административного доступа, поскольку компрометация учётных данных эксплуатационного персонала (обладающего расширенными, зачастую критичными правами) несёт существенно больший риск, чем компрометация учётной записи рядового пользователя, а однофакторной аутентификации для этой категории субъектов недостаточно.</t>
+        </is>
+      </c>
+      <c r="E40" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Внедрение и настройку средств многофакторной аутентификации для всех административных интерфейсов доступа (консоли управления, средства удалённого администрирования, системы виртуализации, PAM-системы);
+2. Обязательное прохождение МФА для доступа к средствам и системам защиты информации, сетевому оборудованию, СУБД и иным критичным компонентам инфраструктуры;
+3. Технический запрет административного доступа при прохождении только одного фактора аутентификации;
+4. Регистрацию событий успешного и неуспешного прохождения многофакторной аутентификации эксплуатационным персоналом.
+Класс используемых средств — средства многофакторной аутентификации (МФА), системы контроля действий привилегированных пользователей (PAM).
+Иностранные: RSA SecurID, CyberArk PAM (со встроенной МФА) и пр.
+Российские сертифицированные (ФСТЭК): «Мультифактор», Indeed Privileged Access Manager и др.
+Открытый код: privacyIDEA, Teleport и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F40" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами систем аутентификации и представителями эксплуатационного персонала;
+2. Скриншоты настроек, подтверждающие требование МФА для всех административных интерфейсов;
+3. Результаты тестирования (попытка административного входа с предъявлением только одного фактора), подтверждающие блокирование такого входа;
+4. Журналы событий, подтверждающие успешные и неуспешные попытки многофакторной аутентификации эксплуатационного персонала.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G40" s="151" t="inlineStr">
+        <is>
+          <t>1. МФА для эксплуатационного персонала подключена не ко всем административным интерфейсам (например, отсутствует для консольного или физического доступа к оборудованию);
+2. Встроенные (сервисные) учётные записи производителей оборудования не охвачены требованием МФА;
+3. Резервные («аварийные») способы административного доступа позволяют обойти требование многофакторной аутентификации;
+4. Журналы прохождения МФА эксплуатационным персоналом не анализируются на предмет аномалий (например, множественных неуспешных попыток).</t>
+        </is>
+      </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -3871,10 +4072,66 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D41" s="21" t="n"/>
-      <c r="E41" s="31" t="n"/>
-      <c r="F41" s="31" t="n"/>
-      <c r="G41" s="31" t="n"/>
+      <c r="D41" s="144" t="inlineStr">
+        <is>
+          <t>Речь идёт об обязательной аутентификации программных сервисов (служб, приложений, скриптов автоматизации), которые осуществляют логический доступ к информационным ресурсам от имени технических (сервисных) учётных записей, а не от имени конкретного физического пользователя.
+Главная цель меры — исключить возможность взаимодействия с информационными ресурсами со стороны неаутентифицированных или подменённых программных компонентов, поскольку технические учётные записи зачастую обладают широкими правами доступа и представляют собой привлекательную цель для компрометации, если аутентификация не контролируется так же строго, как для обычных пользователей.</t>
+        </is>
+      </c>
+      <c r="E41" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационный компонент в этой мере отсутствует, поэтому применяются технические средства:
+1. Настройка обязательной аутентификации технических учётных записей при каждом обращении программного сервиса к информационному ресурсу (по паролю, сертификату, ключу API или иному аутентификационному признаку);
+2. Использование строгих методов аутентификации сервисов — сертификатов (PKI), ключей доступа с ограниченным сроком действия, токенов OAuth и аналогичных механизмов, минимизирующих риск компрометации;
+3. Технический запрет обращения к ресурсам доступа от имени технической учётной записи без предъявления соответствующих аутентификационных данных;
+4. Регистрация событий аутентификации технических учётных записей, включая неуспешные попытки.
+Класс используемых средств — средства управления секретами и сертификатами (Secrets Management, PKI), встроенные механизмы аутентификации СУБД и промежуточного ПО.
+Иностранные: HashiCorp Vault, Microsoft Active Directory Certificate Services и пр.
+Российские сертифицированные (ФСТЭК): ViPNet PKI, «КриптоПро PKI» (программные компоненты) и др.
+Открытый код: HashiCorp Vault (Community Edition), EJBCA и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F41" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с разработчиками и администраторами интеграционных сервисов;
+2. Скриншоты (конфигурации) настроек аутентификации технических учётных записей в подключаемых сервисах;
+3. Результаты тестирования (попытка обращения к ресурсу от имени технической учётной записи без аутентификационных данных), подтверждающие блокирование такого обращения;
+4. Журналы событий, подтверждающие регистрацию аутентификации программных сервисов.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G41" s="151" t="inlineStr">
+        <is>
+          <t>1. Часть программных сервисов обращается к ресурсам доступа с использованием технических учётных записей без аутентификации (например, по доверенному сетевому адресу без проверки подлинности);
+2. Аутентификационные данные технических учётных записей (пароли, ключи) хранятся в открытом виде в конфигурационных файлах или коде интеграции;
+3. Сроки действия сертификатов или ключей технических учётных записей не контролируются и не обновляются регулярно;
+4. Инвентаризация технических учётных записей и используемых ими методов аутентификации не ведётся, часть таких записей может быть не выявлена.</t>
+        </is>
+      </c>
+      <c r="H41" s="156" t="inlineStr">
+        <is>
+          <t>Средства криптографической защиты информации и компоненты PKI в Российской Федерации сертифицируются преимущественно ФСБ России, а не ФСТЭК России. При подборе конкретного продукта для реализации меры необходимо сверяться также с реестром сертифицированных ФСБ России СКЗИ, а не только с реестром ФСТЭК.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="28.5" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
@@ -3892,10 +4149,60 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D42" s="21" t="n"/>
-      <c r="E42" s="31" t="n"/>
-      <c r="F42" s="31" t="n"/>
-      <c r="G42" s="31" t="n"/>
+      <c r="D42" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует аутентификации не только субъекта (представителя эксплуатационного персонала), но и самого автоматизированного рабочего места (АРМ), с которого осуществляется логический доступ, — то есть подтверждения того, что доступ выполняется именно с доверенного, легитимного устройства.
+Главная цель меры — исключить возможность администрирования информационной инфраструктуры с посторонних, неучтённых или скомпрометированных устройств, даже если аутентификационные данные самого сотрудника были предъявлены корректно: без аутентификации устройства кража или подбор пароля администратора позволили бы выполнить вход с любого компьютера.</t>
+        </is>
+      </c>
+      <c r="E42" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как организационных мер здесь не предусмотрено, всё сводится к техническим настройкам:
+1. Использование сертификатов устройств (машинных сертификатов, выпущенных внутренним удостоверяющим центром) или иных технических признаков (например, привязки по MAC-адресу совместно с сертификатом, доменного членства АРМ), подтверждающих легитимность АРМ эксплуатационного персонала;
+2. Настройка средств сетевого доступа (VPN-шлюзов, систем контроля доступа к сети — NAC) таким образом, чтобы административный доступ предоставлялся только с АРМ, прошедших аутентификацию устройства;
+3. Технический запрет административного доступа с устройств, не прошедших аутентификацию (в том числе с личных и неучтённых устройств).
+Класс используемых средств — средства контроля доступа к сети (NAC), инфраструктура открытых ключей (PKI) для аутентификации устройств, VPN-шлюзы с проверкой сертификата устройства.
+Иностранные: Cisco ISE, Palo Alto GlobalProtect и пр.
+Российские сертифицированные (ФСТЭК): «С-Терра Шлюз», ViPNet Coordinator и др.
+Открытый код: FreeRADIUS (совместно с PKI) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F42" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Скриншоты настроек NAC/VPN, подтверждающие проверку сертификата (иного признака) АРМ перед предоставлением административного доступа;
+3. Результаты тестирования (попытка административного подключения с непривязанного устройства), подтверждающие блокирование такого подключения;
+4. Журналы событий аутентификации устройств.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G42" s="151" t="inlineStr">
+        <is>
+          <t>1. Аутентификация АРМ эксплуатационного персонала не охватывает все каналы административного доступа (например, отсутствует для локального/консольного подключения);
+2. Сертификаты устройств выпускаются без строгой проверки принадлежности АРМ конкретному сотруднику или подразделению;
+3. Просроченные или отозванные сертификаты устройств не блокируются автоматически;
+4. Допускается административный доступ с личных устройств при условии установки VPN-клиента, без полноценной проверки соответствия корпоративным требованиям (compliance-проверки).</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="28.5" customHeight="1">
       <c r="A43" s="20" t="inlineStr">
@@ -3913,10 +4220,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D43" s="21" t="n"/>
-      <c r="E43" s="31" t="n"/>
-      <c r="F43" s="31" t="n"/>
-      <c r="G43" s="31" t="n"/>
+      <c r="D43" s="144" t="inlineStr">
+        <is>
+          <t>Мера аналогична РД.6, но распространяется на рабочие места рядовых пользователей: логический доступ должен предоставляться только с АРМ, прошедшего аутентификацию как доверенное устройство, а не с произвольного компьютера.
+Главная цель меры — снизить риск доступа к информационным ресурсам с непроверенных, личных или скомпрометированных устройств, даже при наличии у пользователя корректных аутентификационных данных.</t>
+        </is>
+      </c>
+      <c r="E43" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Здесь требуются только технические решения:
+1. Использование сертификатов устройств или доменного членства АРМ пользователей как условия для предоставления логического доступа к информационным ресурсам;
+2. Настройка средств контроля доступа к сети (NAC) или VPN-шлюзов таким образом, чтобы доступ предоставлялся только с АРМ, прошедших проверку принадлежности к корпоративному парку устройств;
+3. Технический запрет доступа с личных, неучтённых или не прошедших проверку устройств.
+Класс используемых средств — средства контроля доступа к сети (NAC), инфраструктура открытых ключей (PKI) для аутентификации устройств, службы каталогов с привязкой устройств к домену.
+Иностранные: Microsoft Active Directory (доменное членство), Cisco ISE и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, ViPNet Coordinator и др.
+Открытый код: FreeRADIUS, FreeIPA и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F43" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры и рабочих мест;
+2. Скриншоты настроек, подтверждающие проверку принадлежности АРМ пользователя к корпоративному парку устройств перед предоставлением доступа;
+3. Результаты тестирования (попытка входа с непривязанного устройства), подтверждающие блокирование доступа;
+4. Журналы событий аутентификации АРМ пользователей.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G43" s="151" t="inlineStr">
+        <is>
+          <t>1. Аутентификация АРМ пользователей реализована не для всех способов подключения (например, отсутствует для доступа через мобильные приложения или веб-интерфейс);
+2. Часть пользователей работает с личных устройств (BYOD) без применения к ним требований аутентификации устройства;
+3. Учёт (инвентаризация) АРМ пользователей неполон, часть устройств не привязана к домену или системе NAC;
+4. Компрометация сертификата устройства не приводит к его оперативному отзыву.</t>
+        </is>
+      </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -3939,10 +4296,56 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D44" s="21" t="n"/>
-      <c r="E44" s="31" t="n"/>
-      <c r="F44" s="31" t="n"/>
-      <c r="G44" s="31" t="n"/>
+      <c r="D44" s="144" t="inlineStr">
+        <is>
+          <t>Мера устанавливает техническое требование: при вводе пароля (и иных аутентификационных данных) символы не должны отображаться на экране в открытом виде — вместо них показываются символы-заменители (точки, звёздочки) либо поле ввода вовсе не отображает введённые символы.
+Главная цель меры — исключить возможность визуального подглядывания пароля (так называемый shoulder surfing) посторонними лицами, находящимися рядом с субъектом доступа в момент ввода аутентификационных данных.</t>
+        </is>
+      </c>
+      <c r="E44" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера не имеет организационной составляющей — её выполнение обеспечивается техническими средствами:
+1. Использование штатных элементов интерфейса операционных систем, прикладного программного обеспечения (ПО) и веб-приложений, которые маскируют вводимые символы пароля (отображают точки, звёздочки или пустое поле вместо самих символов);
+2. Контроль того, что это требование распространяется на все точки ввода аутентификационных данных — локальный вход в систему, удалённый доступ, веб-интерфейсы, мобильные приложения, консоли администрирования;
+3. Технический запрет на использование или кастомизацию форм ввода, в которых пароль отображается в открытом (незамаскированном) виде.
+Поскольку сокрытие вводимых символов пароля — базовая функция подавляющего большинства современных операционных систем, СУБД, веб-фреймворков и прикладного ПО, отдельного специализированного средства защиты для реализации меры, как правило, не требуется: задача сводится к контролю того, что данная штатная функция не отключена и не обойдена в кастомных интерфейсах.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F44" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем и разработчиками внутренних приложений;
+2. Скриншоты экранов ввода пароля в различных информационных системах и интерфейсах, подтверждающие маскирование вводимых символов;
+3. Результаты выборочной проверки нестандартных (самописных) интерфейсов входа на предмет корректного сокрытия пароля при вводе.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G44" s="151" t="inlineStr">
+        <is>
+          <t>1. В отдельных самописных или устаревших приложениях пароль при вводе отображается в открытом виде;
+2. Требование не распространяется на консоли администрирования специализированного оборудования (например, интерфейсы управления через последовательный порт);
+3. Мобильные приложения временно отображают последний введённый символ пароля дольше, чем это оправдано с точки зрения безопасности, без возможности отключения такого поведения;
+4. Проверка соблюдения требования на нестандартных интерфейсах не проводится.</t>
+        </is>
+      </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -3965,10 +4368,56 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D45" s="21" t="n"/>
-      <c r="E45" s="31" t="n"/>
-      <c r="F45" s="31" t="n"/>
-      <c r="G45" s="31" t="n"/>
+      <c r="D45" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает эксплуатацию учётных записей, для которых аутентификационные данные (пароли) либо вовсе не заданы, либо оставлены такими, какими их установил производитель (разработчик) ресурса доступа или автоматизированной системы (АС) «по умолчанию» — то есть широко известными или предсказуемыми значениями (admin/admin, admin/password и подобными).
+Главная цель меры — устранить один из самых распространённых и легко эксплуатируемых векторов атаки: учётные данные «по умолчанию» известны из документации производителя, находятся в открытом доступе и, как правило, являются первым, что пробует злоумышленник или автоматизированный сканер уязвимостей.</t>
+        </is>
+      </c>
+      <c r="E45" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная составляющая сводится к следующим шагам:
+1. Включить в регламент ввода в эксплуатацию информационных систем и оборудования обязательный этап смены (или первичного задания) аутентификационных данных, отличных от заводских (заданных по умолчанию), до подключения ресурса к рабочей среде;
+2. Закрепить ответственность за выполнение данного этапа за конкретным подразделением (администраторами, инженерами по внедрению);
+3. Проводить периодические проверки (инвентаризацию) эксплуатируемых ресурсов доступа и АС на предмет использования заводских или незаданных аутентификационных данных;
+4. Фиксировать факт смены аутентификационных данных по умолчанию в акте ввода в эксплуатацию или ином документе.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F45" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент ввода в эксплуатацию, содержащий обязательный этап смены аутентификационных данных по умолчанию;
+2. Акты ввода в эксплуатацию информационных систем и оборудования с отметкой о выполнении данного этапа;
+3. Акты (отчёты) периодических проверок на предмет использования заводских или незаданных аутентификационных данных.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G45" s="151" t="inlineStr">
+        <is>
+          <t>1. Регламент ввода в эксплуатацию не содержит явного требования о смене аутентификационных данных по умолчанию;
+2. Проверки на предмет использования заводских учётных данных охватывают не все классы оборудования и ПО (например, забывают про сетевое оборудование, IoT-устройства, встраиваемые системы);
+3. Тестовые или демонстрационные учётные записи, поставляемые с ресурсом «по умолчанию», не отключаются и не удаляются при вводе в эксплуатацию;
+4. Периодическая проверка отсутствия заводских учётных данных не проводится, факт их использования выявляется только по результатам инцидента или внешнего аудита.</t>
+        </is>
+      </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -3991,10 +4440,55 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D46" s="21" t="n"/>
-      <c r="E46" s="31" t="n"/>
-      <c r="F46" s="31" t="n"/>
-      <c r="G46" s="31" t="n"/>
+      <c r="D46" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает использование групповых (используемых несколькими субъектами одновременно), общих и стандартных учётных записей и паролей, а также любых иных методов идентификации и аутентификации, которые не позволяют однозначно определить, какой именно конкретный субъект осуществил логический доступ.
+Главная цель меры — обеспечить персональную идентифицируемость каждого субъекта доступа на уровне самого процесса аутентификации: мера дополняет требование УЗП.1 (уникальные персонифицированные учётные записи), явно запрещая типичные обходные пути — совместное использование одной учётной записи несколькими людьми, стандартные («сервисные») учётные записи для интерактивного входа и подобные практики.</t>
+        </is>
+      </c>
+      <c r="E46" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит организационный характер и включает:
+1. Закрепление во внутреннем нормативном документе прямого запрета на создание и использование групповых, общих и стандартных учётных записей и паролей для интерактивного логического доступа субъектов;
+2. Проведение периодической инвентаризации учётных записей на предмет выявления групповых, общих или стандартных учётных записей, используемых в нарушение установленного запрета;
+3. При выявлении нарушений — инициирование их устранения (замены на персональные учётные записи) и, при необходимости, служебного разбирательства.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F46" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний нормативный документ, содержащий запрет на использование групповых, общих и стандартных учётных записей и паролей;
+2. Акты (отчёты) инвентаризации учётных записей на предмет выявления нарушений установленного запрета;
+3. Свидетельства устранения выявленных нарушений (замены групповых учётных записей на персональные).</t>
+          </r>
+        </is>
+      </c>
+      <c r="G46" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные технологические процессы (например, эксплуатация унаследованных систем) продолжают использовать групповые учётные записи в нарушение запрета, без документированного компенсирующего решения;
+2. Инвентаризация учётных записей на предмет выявления групповых и общих учётных записей не проводится или проводится формально;
+3. Запрет закреплён документально, но не доводится до сведения сотрудников, ответственных за создание учётных записей;
+4. Выявленные нарушения не устраняются в разумный срок.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="42.75" customHeight="1">
       <c r="A47" s="20" t="inlineStr">
@@ -4012,10 +4506,61 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D47" s="21" t="n"/>
-      <c r="E47" s="31" t="n"/>
-      <c r="F47" s="31" t="n"/>
-      <c r="G47" s="31" t="n"/>
+      <c r="D47" s="144" t="inlineStr">
+        <is>
+          <t>Мера устанавливает техническое требование к автоматической временной блокировке учётной записи пользователя после определённого числа последовательных неуспешных попыток аутентификации, причём период такой блокировки должен составлять не менее 30 минут.
+Главная цель меры — противодействовать атакам подбора пароля (brute-force, перебор по словарю): ограничение числа попыток и введение задержки перед следующей возможной попыткой делает подбор пароля вычислительно нецелесообразным для злоумышленника, при этом сохраняя для легитимного пользователя возможность восстановить доступ по истечении установленного времени.</t>
+        </is>
+      </c>
+      <c r="E47" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация меры лежит полностью в технической плоскости и включает:
+1. Настройку политики блокировки учётных записей в операционной системе, каталоге (Active Directory, LDAP) или ином средстве аутентификации: задание порогового числа неуспешных последовательных попыток аутентификации, после которого учётная запись автоматически блокируется;
+2. Установку длительности временной блокировки не менее 30 минут (либо снятие блокировки только по обращению к администратору — при более строгих требованиях к безопасности);
+3. Применение данной политики единообразно ко всем информационным системам, где осуществляется аутентификация пользователей, включая веб-интерфейсы и удалённый доступ;
+4. Регистрацию событий блокировки учётной записи в журнале для последующего анализа (в том числе на предмет выявления попыток подбора пароля).
+Класс используемых средств — службы каталогов и системы управления учётными записями (IdM) со встроенной политикой блокировки, средства защиты от несанкционированного доступа (СЗИ от НСД).
+Иностранные: Microsoft Active Directory (Account Lockout Policy) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К и др.
+Открытый код: FreeIPA и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F47" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек политики блокировки учётных записей (пороговое число попыток, длительность блокировки);
+3. Результаты тестирования (несколько последовательных неуспешных попыток входа), подтверждающие фактическую блокировку учётной записи на период не менее 30 минут;
+4. Журналы событий, подтверждающие регистрацию фактов блокировки учётных записей.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G47" s="151" t="inlineStr">
+        <is>
+          <t>1. Пороговое число неуспешных попыток аутентификации либо длительность блокировки не настроены или не соответствуют установленным требованиям (блокировка короче 30 минут);
+2. Политика блокировки применена не ко всем информационным системам (например, отсутствует для веб-интерфейсов или устаревших приложений);
+3. Механизм блокировки технически реализован, но фактическое тестирование его срабатывания не проводится;
+4. События блокировки учётных записей не анализируются на предмет выявления целенаправленных попыток подбора паролей.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="57" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
@@ -4033,10 +4578,60 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D48" s="21" t="n"/>
-      <c r="E48" s="31" t="n"/>
-      <c r="F48" s="31" t="n"/>
-      <c r="G48" s="31" t="n"/>
+      <c r="D48" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает одновременное открытие нескольких параллельных сессий логического доступа под одной и той же учётной записью с разных автоматизированных рабочих мест (АРМ), включая виртуальные машины.
+Главная цель меры — исключить ситуацию, при которой скомпрометированная учётная запись используется злоумышленником параллельно с легитимным пользователем (что затрудняет своевременное обнаружение компрометации), а также предотвратить намеренное совместное использование одной учётной записи несколькими сотрудниками одновременно.</t>
+        </is>
+      </c>
+      <c r="E48" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера реализуется только техническими средствами, необходимо:
+1. Настройку информационных систем и служб каталогов таким образом, чтобы при попытке открытия новой сессии под учётной записью, уже имеющей активную сессию с другого АРМ, происходил отказ в доступе либо принудительное завершение предыдущей сессии;
+2. Централизованный контроль активных сессий (Single Session Enforcement) через систему управления доступом или средства терминального доступа;
+3. Регистрацию попыток открытия параллельных сессий под одной учётной записью для последующего анализа на предмет возможной компрометации.
+Класс используемых средств — средства терминального доступа и виртуализации рабочих столов (VDI), системы контроля сессий, службы каталогов с политикой ограничения одновременных сеансов.
+Иностранные: Citrix Virtual Apps and Desktops, Microsoft Remote Desktop Services (ограничение сессий) и пр.
+Российские сертифицированные (ФСТЭК): «Термидеск», Astra Linux (совместно со средствами разграничения сессий) и др.
+Открытый код: FreeRDP (с ограничениями на стороне сервера) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F48" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек, ограничивающих количество одновременных сессий под одной учётной записью;
+3. Результаты тестирования (попытка одновременного входа под одной учётной записью с двух разных АРМ), подтверждающие срабатывание запрета;
+4. Журналы событий, подтверждающие регистрацию попыток открытия параллельных сессий.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G48" s="151" t="inlineStr">
+        <is>
+          <t>1. Ограничение параллельных сессий настроено не для всех информационных систем (например, отсутствует для веб-приложений или мобильного доступа);
+2. Технические учётные записи и учётные записи для автоматизированных процессов исключены из-под действия запрета без документированного обоснования;
+3. При обнаружении попытки открытия параллельной сессии система не уведомляет администратора безопасности;
+4. Виртуальные АРМ (в инфраструктуре VDI) не учитываются при определении количества активных сессий наравне с физическими.</t>
+        </is>
+      </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4065,9 +4660,50 @@
 Главная цель меры — защита информации от несанкционированного доступа в ситуациях, когда сотрудник временно покидает рабочее место, но не хочет или не может завершить все текущие операции. Возможность быстро заблокировать экран или завершить сессию позволяет предотвратить доступ посторонних лиц к конфиденциальной информации.</t>
         </is>
       </c>
-      <c r="E49" s="31" t="n"/>
-      <c r="F49" s="31" t="n"/>
-      <c r="G49" s="31" t="n"/>
+      <c r="E49" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Технический характер меры предполагает следующий набор действий:
+1. Настройку операционных систем и прикладного ПО таким образом, чтобы субъект логического доступа мог самостоятельно инициировать блокировку экрана (приостановку сессии) сочетанием клавиш или соответствующим элементом интерфейса;
+2. Настройку возможности принудительного завершения сессии логического доступа (выхода из системы) по инициативе пользователя, с корректным закрытием всех активных приложений и соединений;
+3. Обеспечение того, что при блокировке экрана прекращается отображение любой информации, полученной в рамках сессии, до момента повторной аутентификации (см. меру РД.15).
+Отдельное специализированное средство защиты для реализации этой меры, как правило, не требуется — функция блокировки экрана и завершения сессии входит в базовую поставку современных операционных систем и прикладного ПО.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F49" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с пользователями и администраторами АРМ;
+2. Результаты тестирования (инициирование блокировки экрана и завершения сессии пользователем), подтверждающие корректную работу функции;
+3. Скриншоты настроек операционной системы (прикладного ПО), подтверждающие доступность данной функции пользователю.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G49" s="151" t="inlineStr">
+        <is>
+          <t>1. Функция принудительной блокировки экрана недоступна пользователю на части АРМ (например, отключена локальными настройками);
+2. При блокировке экрана часть информации (уведомления, превью писем) продолжает отображаться поверх экрана блокировки;
+3. Пользователи не осведомлены о наличии и способе использования данной функции, что снижает практическую эффективность меры;
+4. Функция реализована не для всех типов АРМ (например, отсутствует в терминальных сессиях или на тонких клиентах).</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="199.5" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
@@ -4091,9 +4727,55 @@
 Главная цель меры — исключить возможность несанкционированного доступа к информационным ресурсам в случае, когда пользователь оставил рабочее место без присмотра, забыв заблокировать экран. Автоматическая блокировка предотвращает доступ посторонних лиц к открытым сессиям и выполнение любых операций от имени авторизованного пользователя в его отсутствие.</t>
         </is>
       </c>
-      <c r="E50" s="31" t="n"/>
-      <c r="F50" s="31" t="n"/>
-      <c r="G50" s="31" t="n"/>
+      <c r="E50" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно техническими средствами:
+1. Настройку операционных систем и (или) средств защиты информации на автоматическое включение блокировки экрана (приостановку сессии) по истечении периода бездействия пользователя, не превышающего 15 минут;
+2. Обеспечение прекращения отображения информации, полученной в рамках сессии, сразу после срабатывания автоматической блокировки;
+3. Единообразное применение данной настройки ко всем АРМ пользователей и эксплуатационного персонала, включая терминальные и удалённые сессии;
+4. Технический запрет на изменение пользователем установленного времени бездействия в сторону увеличения (см. также меру УЗП.11).
+Класс используемых средств — операционные системы с политиками блокировки экрана (screen lock), средства централизованного управления конфигурациями (групповые политики).
+Иностранные: Microsoft Group Policy (Interactive logon: Machine inactivity limit) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К и др.
+Открытый код: настройки экранной заставки (блокировки) дистрибутивов Linux (gsettings, loginctl) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F50" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами АРМ;
+2. Скриншоты (выгрузки) групповых политик или иных настроек, подтверждающие установленное время бездействия не более 15 минут;
+3. Результаты тестирования (оставление сессии без активности) на выборке АРМ, подтверждающие фактическое срабатывание автоматической блокировки в установленное время;
+4. Результаты выборочной проверки, подтверждающие, что пользователи технически не могут увеличить установленное время бездействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G50" s="151" t="inlineStr">
+        <is>
+          <t>1. Время автоматической блокировки экрана превышает установленные 15 минут на части АРМ;
+2. Настройка применена не ко всем категориям устройств (например, отсутствует для терминальных серверов, серверов приложений с интерактивным входом);
+3. Пользователи технически имеют возможность изменить (увеличить или отключить) установленное время бездействия;
+4. Фактическое тестирование срабатывания автоматической блокировки не проводится, контроль ограничивается проверкой конфигурации.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="228" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
@@ -4117,9 +4799,48 @@
 Главная цель меры — исключить возможность несанкционированного доступа к информационным ресурсам в ситуациях, когда сессия была прервана (автоматически или по инициативе пользователя), но рабочая станция осталась физически доступной для посторонних лиц. Повторная аутентификация гарантирует, что продолжить работу сможет только тот пользователь, который знает (или имеет) соответствующие аутентификационные данные.</t>
         </is>
       </c>
-      <c r="E51" s="31" t="n"/>
-      <c r="F51" s="31" t="n"/>
-      <c r="G51" s="31" t="n"/>
+      <c r="E51" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера выполняется силами технических средств защиты информации, а именно:
+1. Настройку операционных систем и прикладного ПО таким образом, чтобы после принудительного (мера РД.13) или автоматического (мера РД.14) прерывания сессии продолжение работы было технически невозможно без повторного прохождения процедуры аутентификации;
+2. Обеспечение того, что повторная аутентификация выполняется с той же строгостью, что и первичная (в том числе с соблюдением требования многофакторности, если оно применимо к соответствующей категории субъектов);
+3. Технический запрет на автоматическое (без участия пользователя) возобновление сессии в обход процедуры аутентификации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F51" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами АРМ и информационных систем;
+2. Результаты тестирования (попытка продолжить работу после блокировки экрана без ввода аутентификационных данных), подтверждающие невозможность такого продолжения;
+3. Скриншоты настроек, подтверждающие обязательность повторной аутентификации после прерывания сессии.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G51" s="151" t="inlineStr">
+        <is>
+          <t>1. На части АРМ возможно продолжение работы после блокировки экрана без повторной аутентификации (например, из-за настроек энергосбережения, отключающих экран без блокировки сессии);
+2. Повторная аутентификация после прерывания сессии не требует того же уровня строгости, что и первичная (например, не запрашивается второй фактор МФА);
+3. Тестирование фактической невозможности обхода повторной аутентификации не проводится.</t>
+        </is>
+      </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4142,17 +4863,57 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D52" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Суть меры заключается в использовании на автоматизированных рабочих местах (АРМ) субъектов логического доступа встроенных механизмов контроля изменения базовой конфигурации оборудования. Таким механизмом является пароль на изменение параметров конфигурации системы, хранящихся в энергонезависимой памяти.
+      <c r="D52" s="153" t="inlineStr">
+        <is>
+          <t>Суть меры заключается в использовании на автоматизированных рабочих местах (АРМ) субъектов логического доступа встроенных механизмов контроля изменения базовой конфигурации оборудования. Таким механизмом является пароль на изменение параметров конфигурации системы, хранящихся в энергонезависимой памяти.
 Под «базовой конфигурацией оборудования» понимаются настройки, хранящиеся в энергонезависимой памяти (например, BIOS/UEFI), которые определяют параметры загрузки системы, порядок загрузки устройств, включение/отключение интерфейсов и портов, настройки безопасности процессора и другие низкоуровневые параметры оборудования.
-Главная цель меры — защитить базовые настройки оборудования от несанкционированного изменения со стороны пользователей или злоумышленников. .
-</t>
-        </is>
-      </c>
-      <c r="E52" s="31" t="n"/>
-      <c r="F52" s="31" t="n"/>
-      <c r="G52" s="31" t="n"/>
+Главная цель меры — защитить базовые настройки оборудования от несанкционированного изменения со стороны пользователей или злоумышленников.</t>
+        </is>
+      </c>
+      <c r="E52" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационные меры для данного требования не предусмотрены — реализация строится на технических решениях:
+1. Использование встроенных в BIOS/UEFI механизмов защиты паролем изменения параметров базовой конфигурации оборудования (порядка загрузки устройств, включения/отключения портов и интерфейсов, параметров безопасности процессора);
+2. Установку уникальных паролей BIOS/UEFI на каждом АРМ силами эксплуатационного персонала при вводе оборудования в эксплуатацию;
+3. Технический запрет на сброс пароля BIOS/UEFI пользователем без физического вмешательства эксплуатационного персонала (например, без вскрытия корпуса и работы с перемычками на материнской плате);
+4. Периодическую проверку того, что защита BIOS/UEFI паролем не отключена и не обойдена.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F52" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами АРМ и эксплуатационным персоналом, отвечающим за настройку оборудования;
+2. Результаты выборочной проверки настроек BIOS/UEFI на предмет наличия установленного пароля на изменение конфигурации;
+3. Акты ввода в эксплуатацию АРМ с отметкой о выполнении настройки защиты BIOS/UEFI паролем.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G52" s="151" t="inlineStr">
+        <is>
+          <t>1. Пароль BIOS/UEFI установлен не на всех АРМ, часть оборудования эксплуатируется с заводскими настройками;
+2. Используется единый (одинаковый) пароль BIOS/UEFI для всего парка оборудования, что снижает эффективность меры при компрометации одного устройства;
+3. Периодическая проверка наличия и действия пароля BIOS/UEFI не проводится;
+4. Пароль BIOS/UEFI известен широкому кругу лиц, включая пользователей АРМ, что обесценивает ограничение.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
@@ -4183,10 +4944,59 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D54" s="21" t="n"/>
-      <c r="E54" s="53" t="n"/>
-      <c r="F54" s="53" t="n"/>
-      <c r="G54" s="53" t="n"/>
+      <c r="D54" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает применение технологий аутентификации, при которых аутентификационные данные (пароли) сохраняются в средствах вычислительной техники (СВТ) — операционных системах, базах данных, конфигурационных файлах приложений — в открытом (незашифрованном, нехешированном) виде.
+Главная цель меры — исключить возможность непосредственного хищения паролей в случае получения злоумышленником доступа к файловой системе, базе данных или памяти СВТ: при правильном хранении (хеширование с солью либо шифрование) компрометация носителя данных сама по себе не раскрывает пароли субъектов доступа.</t>
+        </is>
+      </c>
+      <c r="E54" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Ввиду того, что мера реализуется только технически, необходимо:
+1. Использование операционных систем, СУБД и прикладного ПО, хранящих аутентификационные данные исключительно в виде криптографических хешей (с применением «соли» и стойких алгоритмов хеширования), либо в зашифрованном виде с использованием сертифицированных средств криптографической защиты информации (СКЗИ);
+2. Технический запрет на применение устаревших или заведомо небезопасных механизмов хранения паролей (обратимое шифрование слабыми алгоритмами, хранение в открытом виде в конфигурационных файлах, базах данных или реестре);
+3. Периодический технический контроль (сканирование конфигураций и хранилищ данных) на предмет выявления аутентификационных данных, сохранённых в открытом виде.
+Класс используемых средств — средства сканирования конфигураций и анализа уязвимостей, встроенные механизмы хранения учётных данных операционных систем и СУБД.
+Иностранные: Microsoft Active Directory (хранение хешей паролей), Tenable Nessus (для выявления небезопасного хранения) и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol (сканер защищённости), Secret Net Studio и др.
+Открытый код: OpenLDAP (с современными схемами хеширования), OpenVAS и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F54" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем и разработчиками внутренних приложений;
+2. Результаты сканирования (анализа конфигураций) информационных систем на предмет выявления аутентификационных данных, хранящихся в открытом виде;
+3. Выгрузки настроек СУБД и прикладного ПО, подтверждающие применение хеширования (шифрования) для хранения аутентификационных данных.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G54" s="157" t="inlineStr">
+        <is>
+          <t>1. Отдельные (как правило, устаревшие или самописные) приложения хранят пароли в открытом виде в конфигурационных файлах или базе данных;
+2. Используются слабые или устаревшие алгоритмы хеширования, не обеспечивающие достаточной криптографической стойкости;
+3. Периодическое сканирование на предмет небезопасного хранения аутентификационных данных не проводится;
+4. Резервные копии баз данных и конфигурационных файлов, содержащие аутентификационные данные, не защищены так же строго, как основные системы хранения.</t>
+        </is>
+      </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4209,15 +5019,63 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D55" s="44" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в том, что чтобы при любой передаче по сети идентификаторов и паролей (аутентификационных данных) использовались только защищённые протоколы, исключающие возможность их перехвата в незашифрованном виде, что исключает компрометацию учётных данных при перехвате трафика или в результате ошибочной настройки приложений. 
-Главная цель меры — предотвратить перехват и компрометацию аутентификационных данных злоумышленниками при их передаче по сетям, а также исключить случаи, когда аутентификационные данные оказываются в системах, не имеющих отношения к аутентификации, и становятся доступными для несанкционированного ознакомления.</t>
-        </is>
-      </c>
-      <c r="E55" s="53" t="n"/>
-      <c r="F55" s="53" t="n"/>
-      <c r="G55" s="53" t="n"/>
+      <c r="D55" s="153" t="inlineStr">
+        <is>
+          <t>Мера объединяет два взаимосвязанных запрета:
+1. Запрет на передачу аутентификационных данных (паролей, идентификаторов) по каналам и линиям связи в открытом (незашифрованном) виде — для этого должны использоваться только защищённые протоколы;
+2. Запрет на передачу (направление, копирование) аутентификационных данных куда-либо, кроме непосредственно средств или систем аутентификации, — то есть исключение ситуаций, при которых пароли попадают в журналы приложений, системы мониторинга, аналитические системы или иные хранилища, не предназначенные для хранения аутентификационных данных.
+Главная цель меры — предотвратить перехват и компрометацию аутентификационных данных при их передаче по сети, а также исключить их «утечку» в системы, не имеющие отношения к процессу аутентификации и не обеспечивающие для этого надлежащей защиты.</t>
+        </is>
+      </c>
+      <c r="E55" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация меры лежит полностью в технической плоскости и включает:
+1. Использование защищённых (шифрованных) протоколов передачи данных (TLS/SSL, SSH и аналогичных) для всех каналов, по которым передаются аутентификационные данные, включая внутреннюю сетевую инфраструктуру;
+2. Технический запрет на применение протоколов, передающих аутентификационные данные в открытом виде (устаревшие версии Telnet, FTP, HTTP без TLS, ранние версии протоколов аутентификации);
+3. Настройку систем логирования и мониторинга таким образом, чтобы аутентификационные данные не попадали в журналы событий, системы аналитики и иные хранилища, не относящиеся непосредственно к средствам аутентификации (маскирование или исключение полей с паролями при логировании);
+4. Периодический технический контроль (анализ сетевого трафика, аудит конфигураций) на предмет использования незащищённых протоколов или утечки аутентификационных данных в посторонние системы.
+Класс используемых средств — средства криптографической защиты каналов связи (VPN, TLS-терминаторы), средства анализа сетевого трафика и выявления утечек данных (DLP).
+Иностранные: F5 BIG-IP (TLS-терминация), Wireshark (для контрольного анализа трафика) и пр.
+Российские сертифицированные (ФСТЭК): «С-Терра Шлюз», ViPNet Coordinator, InfoWatch Traffic Monitor и др.
+Открытый код: OpenSSL/OpenVPN, Wireshark и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F55" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры и разработчиками внутренних приложений;
+2. Результаты анализа сетевого трафика (или конфигураций протоколов), подтверждающие отсутствие передачи аутентификационных данных в открытом виде;
+3. Выгрузки настроек систем логирования, подтверждающие маскирование или исключение аутентификационных данных из журналов событий;
+4. Результаты выборочной проверки (аудита) конфигураций информационных систем на предмет использования незащищённых протоколов.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G55" s="157" t="inlineStr">
+        <is>
+          <t>1. Отдельные внутренние сервисы или устаревшее оборудование продолжают использовать незащищённые протоколы передачи данных (Telnet, HTTP без TLS);
+2. Пароли или их фрагменты попадают в журналы событий приложений или систем мониторинга без маскирования;
+3. Анализ сетевого трафика и конфигураций на предмет утечки аутентификационных данных не проводится на регулярной основе;
+4. Аутентификационные данные передаются по электронной почте или в мессенджерах при первичной выдаче пользователю без последующей обязательной смены.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="99.75" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
@@ -4241,9 +5099,55 @@
 Главная цель меры — снизить риски компрометации паролей за счёт ограничения времени их использования.</t>
         </is>
       </c>
-      <c r="E56" s="31" t="n"/>
-      <c r="F56" s="31" t="n"/>
-      <c r="G56" s="31" t="n"/>
+      <c r="E56" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера подразумевает исключительно технические меры защиты, а именно:
+1. Настройку в операционных системах, каталогах (Active Directory, LDAP) и прикладных информационных системах политики максимального срока действия пароля пользователя, не превышающего 365 дней;
+2. Автоматическое информирование пользователя (уведомление) о приближающемся истечении срока действия пароля;
+3. Технический запрет на продолжение работы под учётной записью с истёкшим сроком действия пароля без его обязательной смены;
+4. Технический запрет на установку пользователем нового пароля, совпадающего с одним из ранее использовавшихся (история паролей).
+Класс используемых средств — службы каталогов и системы управления учётными записями (IdM) со встроенной политикой паролей.
+Иностранные: Microsoft Active Directory (Password Policy) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Avanpost IDM и др.
+Открытый код: FreeIPA, OpenLDAP (совместно с модулями контроля срока действия пароля) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F56" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты (выгрузки) настроек политики паролей, подтверждающие максимальный срок действия пароля не более 365 дней;
+3. Выгрузка отчёта о датах последней смены паролей пользователей, подтверждающая соблюдение установленной периодичности;
+4. Результаты тестирования (попытка входа под учётной записью с истёкшим сроком действия пароля без его смены), подтверждающие срабатывание требования.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G56" s="151" t="inlineStr">
+        <is>
+          <t>1. Политика максимального срока действия пароля настроена не для всех информационных систем, к которым пользователи осуществляют логический доступ;
+2. Отдельные учётные записи (например, технические или редко используемые) исключены из-под действия политики без документированного обоснования;
+3. Пользователи обходят требование, меняя пароль формально (на очень похожий) при отсутствии контроля истории паролей;
+4. Отчётность о соблюдении срока действия паролей не формируется, нарушения выявляются только по факту инцидента.</t>
+        </is>
+      </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4272,9 +5176,55 @@
 Главная цель меры — снизить риски компрометации паролей эксплуатационного персонала за счёт более частой (по сравнению с рядовыми пользователями) смены паролей. Эксплуатационный персонал обладает привилегированными правами доступа, и компрометация их учётных данных может привести к наиболее серьёзным последствиям для организации.</t>
         </is>
       </c>
-      <c r="E57" s="31" t="n"/>
-      <c r="F57" s="31" t="n"/>
-      <c r="G57" s="31" t="n"/>
+      <c r="E57" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как речь идёт о чисто технической мере, реализация включает:
+1. Настройку в системах управления привилегированным доступом, службах каталогов и на управляемом оборудовании политики максимального срока действия пароля эксплуатационного персонала, не превышающего 90 дней;
+2. Применение более строгого контроля соблюдения данной политики по сравнению с учётными записями рядовых пользователей — с учётом повышенной критичности привилегированных прав доступа;
+3. Технический запрет на продолжение административной работы под учётной записью с истёкшим сроком действия пароля;
+4. Технический запрет на повторное использование ранее применявшихся паролей (история паролей) для привилегированных учётных записей.
+Класс используемых средств — системы управления привилегированным доступом (PAM), службы каталогов с политикой паролей.
+Иностранные: CyberArk PAM, Microsoft Active Directory (Fine-Grained Password Policy) и пр.
+Российские сертифицированные (ФСТЭК): Indeed Privileged Access Manager, «Система контроля привилегированных пользователей SafeInspect» и др.
+Открытый код: Teleport и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F57" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с эксплуатационным персоналом и подразделением информационной безопасности;
+2. Скриншоты (выгрузки) настроек политики паролей для привилегированных учётных записей, подтверждающие максимальный срок действия не более 90 дней;
+3. Выгрузка отчёта о датах последней смены паролей эксплуатационного персонала;
+4. Результаты тестирования (попытка административного входа под учётной записью с истёкшим сроком действия пароля), подтверждающие срабатывание требования.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G57" s="151" t="inlineStr">
+        <is>
+          <t>1. Политика срока действия пароля для эксплуатационного персонала не отличается от политики для рядовых пользователей (не учитывает более строгий квартальный порог);
+2. Встроенные (сервисные) учётные записи оборудования не охвачены политикой смены паролей;
+3. Смена паролей выполняется формально, без фактического изменения сложности пароля;
+4. Контроль соблюдения квартальной периодичности не формализован, нарушения выявляются несистемно.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="128.25" customHeight="1">
       <c r="A58" s="20" t="inlineStr">
@@ -4298,9 +5248,52 @@
 Главная цель меры — повысить устойчивость паролей к подбору (методами перебора, атаками по словарю и т.п.) за счёт увеличения их длины. Чем длиннее пароль, тем больше возможных комбинаций и тем сложнее его подобрать злоумышленнику.</t>
         </is>
       </c>
-      <c r="E58" s="31" t="n"/>
-      <c r="F58" s="31" t="n"/>
-      <c r="G58" s="31" t="n"/>
+      <c r="E58" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется на техническом уровне без организационной составляющей:
+1. Настройку в операционных системах, каталогах и прикладных информационных системах политики минимальной длины пароля пользователей — не менее восьми символов;
+2. Технический запрет на установку (сохранение) пользователем пароля короче установленного минимума;
+3. Распространение данной настройки на все информационные системы, к которым пользователи осуществляют логический доступ.
+Класс используемых средств — службы каталогов и системы управления учётными записями (IdM) со встроенной политикой паролей.
+Иностранные: Microsoft Active Directory (Minimum Password Length) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Avanpost IDM и др.
+Открытый код: FreeIPA, OpenLDAP и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F58" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты (выгрузки) настроек политики паролей, подтверждающие минимальную длину не менее восьми символов;
+3. Результаты тестирования (попытка установки пароля короче восьми символов), подтверждающие блокирование такой попытки.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G58" s="151" t="inlineStr">
+        <is>
+          <t>1. Политика минимальной длины пароля настроена не для всех информационных систем;
+2. Требование к длине пароля установлено на уровне регламента, но технически не контролируется (пользователь фактически может задать более короткий пароль);
+3. Отдельные унаследованные системы технически не поддерживают установку минимальной длины пароля восемь и более символов, компенсирующие меры не приняты.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="256.5" customHeight="1">
       <c r="A59" s="20" t="inlineStr">
@@ -4324,9 +5317,52 @@
 Главная цель меры — существенно повысить устойчивость паролей эксплуатационного персонала к подбору (методами перебора, атаками по словарю и т.п.) за счёт значительного увеличения их длины. Пароль длиной 16 символов экспоненциально сложнее подобрать, чем 8-символьный, что критически важно для защиты привилегированных учётных записей.</t>
         </is>
       </c>
-      <c r="E59" s="31" t="n"/>
-      <c r="F59" s="31" t="n"/>
-      <c r="G59" s="31" t="n"/>
+      <c r="E59" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационные меры для данного требования не предусмотрены — реализация строится на технических решениях:
+1. Настройку отдельной (более строгой) политики паролей для привилегированных (административных) учётных записей — минимальная длина пароля не менее шестнадцати символов;
+2. Технический запрет на установку эксплуатационным персоналом пароля короче установленного минимума;
+3. Распространение данной настройки на все административные интерфейсы и системы, к которым эксплуатационный персонал осуществляет логический доступ, включая сетевое оборудование и средства защиты информации.
+Класс используемых средств — системы управления привилегированным доступом (PAM), службы каталогов с раздельными политиками паролей (Fine-Grained Password Policy).
+Иностранные: CyberArk PAM, Microsoft Active Directory (Fine-Grained Password Policy) и пр.
+Российские сертифицированные (ФСТЭК): Indeed Privileged Access Manager, Secret Net Studio и др.
+Открытый код: Teleport и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F59" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с эксплуатационным персоналом и подразделением информационной безопасности;
+2. Скриншоты (выгрузки) настроек политики паролей для привилегированных учётных записей, подтверждающие минимальную длину не менее шестнадцати символов;
+3. Результаты тестирования (попытка установки административного пароля короче шестнадцати символов), подтверждающие блокирование такой попытки.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G59" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельная (более строгая) политика длины пароля для эксплуатационного персонала не настроена, применяется общая политика для рядовых пользователей;
+2. Требование распространяется не на все административные интерфейсы (например, отсутствует для встроенных консолей управления сетевым оборудованием);
+3. Встроенные (сервисные) учётные записи производителей оборудования используют пароли короче установленного минимума.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="199.5" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
@@ -4350,9 +5386,52 @@
 Главная цель меры — существенно повысить устойчивость паролей к подбору (методами перебора, атаками по словарю и т.п.) за счёт увеличения их сложности. Пароль, состоящий только из букв одного регистра, значительно легче подобрать, чем пароль, содержащий буквы разных регистров и цифры. Использование символов из разных групп расширяет пространство возможных комбинаций, что делает перебор паролей вычислительно трудоёмким для злоумышленника.</t>
         </is>
       </c>
-      <c r="E60" s="31" t="n"/>
-      <c r="F60" s="31" t="n"/>
-      <c r="G60" s="31" t="n"/>
+      <c r="E60" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера выполняется силами технических средств защиты информации, а именно:
+1. Настройку в операционных системах, каталогах и прикладных информационных системах политики сложности пароля, требующей одновременного использования заглавных и строчных букв, а также цифр;
+2. Технический запрет на установку пароля, не соответствующего установленным требованиям сложности;
+3. Распространение данной настройки на все информационные системы, к которым субъекты логического доступа осуществляют вход.
+Класс используемых средств — службы каталогов и системы управления учётными записями (IdM) со встроенной политикой сложности паролей.
+Иностранные: Microsoft Active Directory (Password must meet complexity requirements) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Avanpost IDM и др.
+Открытый код: FreeIPA, pam_pwquality (Linux) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F60" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты (выгрузки) настроек политики сложности паролей;
+3. Результаты тестирования (попытка установки пароля без цифр или без букв разных регистров), подтверждающие блокирование такой попытки.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G60" s="151" t="inlineStr">
+        <is>
+          <t>1. Политика сложности пароля настроена не для всех информационных систем;
+2. Требование к сложности пароля декларировано в регламенте, но технически не контролируется;
+3. Отдельные унаследованные системы не поддерживают проверку сложности пароля, компенсирующие меры не приняты.</t>
+        </is>
+      </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4375,10 +5454,55 @@
           <t>Н-О-О</t>
         </is>
       </c>
-      <c r="D61" s="21" t="n"/>
-      <c r="E61" s="31" t="n"/>
-      <c r="F61" s="31" t="n"/>
-      <c r="G61" s="31" t="n"/>
+      <c r="D61" s="144" t="inlineStr">
+        <is>
+          <t>Мера дополняет требования к длине и сложности паролей (РД.21—РД.23) запретом на использование легко вычисляемых (предсказуемых) комбинаций — личных данных субъекта (имени, фамилии, даты рождения), наименований организации или её подразделений, общепринятых сокращений и иных сочетаний, которые злоумышленник может подобрать не перебором, а логическим предположением или методами социальной инженерии.
+Главная цель меры — исключить класс паролей, формально соответствующих требованиям длины и сложности, но фактически легко угадываемых, поскольку такие пароли сводят на нет эффект от остальных парольных требований.</t>
+        </is>
+      </c>
+      <c r="E61" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно организационными методами и предполагает:
+1. Закрепление во внутреннем нормативном документе (парольной политике) прямого запрета на использование в паролях личных данных субъекта, наименований организации, общепринятых сокращений и иных легко вычисляемых сочетаний, с приведением показательных примеров недопустимых паролей;
+2. Информирование (инструктаж) субъектов логического доступа об этом требовании при первичном допуске к работе и периодически в рамках повышения осведомлённости по вопросам информационной безопасности;
+3. Включение данного требования в памятки и инструкции по формированию надёжных паролей, доводимые до сведения пользователей и эксплуатационного персонала.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F61" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний нормативный документ (парольная политика), содержащий запрет на использование легко вычисляемых сочетаний в паролях;
+2. Листы ознакомления субъектов логического доступа с требованиями к формированию паролей;
+3. Материалы инструктажа (памятки) по формированию надёжных паролей.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G61" s="151" t="inlineStr">
+        <is>
+          <t>1. Запрет декларирован в документе, но не проверяется на практике — технические средства контроля «слабых» паролей на основе словарей и типовых шаблонов не используются;
+2. Субъекты логического доступа не информируются о данном требовании при первичном допуске;
+3. Инструктаж проводится формально, без разъяснения конкретных примеров недопустимых паролей;
+4. Требование не пересматривается и не актуализируется с учётом современных методов подбора паролей (атаки по маскам, использование утёкших баз данных).</t>
+        </is>
+      </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4407,9 +5531,54 @@
 Главная цель меры — снизить нагрузку на административный персонал и повысить оперативность смены паролей пользователями (например, при подозрении на компрометацию, по требованию политики безопасности, при забывании пароля с использованием механизмов самовосстановления или по истечении срока действия). Это также способствует повышению безопасности, так как пользователи могут незамедлительно сменить пароль при возникновении подозрений на его компрометацию, не дожидаясь администратора.</t>
         </is>
       </c>
-      <c r="E62" s="31" t="n"/>
-      <c r="F62" s="31" t="n"/>
-      <c r="G62" s="31" t="n"/>
+      <c r="E62" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Предоставление субъектам логического доступа штатной технической возможности самостоятельно изменить свой пароль без обращения к администратору (стандартная функция смены пароля в операционной системе, каталоге или портале самообслуживания);
+2. Реализацию механизма самостоятельного восстановления доступа при утрате (забывании) пароля — с обязательным подтверждением личности субъекта дополнительным способом (секретные вопросы, одноразовый код, обращение к service desk);
+3. Применение к самостоятельно устанавливаемому пользователем паролю тех же требований сложности, длины и истории паролей, что предусмотрены мерами РД.19—РД.23.
+Класс используемых средств — службы каталогов и системы управления учётными записями (IdM) с функцией самообслуживания пользователей (self-service password reset).
+Иностранные: Microsoft Identity Manager (Self-Service Password Reset), Okta и пр.
+Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
+Открытый код: FreeIPA (портал самообслуживания) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F62" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с пользователями и администраторами информационных систем;
+2. Результаты тестирования (самостоятельная смена пароля пользователем), подтверждающие доступность и корректную работу функции;
+3. Скриншоты интерфейса самостоятельной смены (восстановления) пароля;
+4. Результаты выборочной проверки, подтверждающие применение к самостоятельно устанавливаемому паролю требований сложности, длины и истории паролей.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G62" s="151" t="inlineStr">
+        <is>
+          <t>1. Функция самостоятельной смены пароля доступна не для всех информационных систем, к части систем пароль меняет только администратор;
+2. Механизм восстановления пароля при его утрате не предусматривает достаточного подтверждения личности субъекта, что создаёт риск социальной инженерии;
+3. При самостоятельной смене пароля не проверяется его соответствие требованиям сложности и истории паролей;
+4. Пользователи не осведомлены о наличии функции самостоятельной смены пароля и продолжают обращаться к администраторам.</t>
+        </is>
+      </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4432,10 +5601,56 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D63" s="21" t="n"/>
-      <c r="E63" s="31" t="n"/>
-      <c r="F63" s="31" t="n"/>
-      <c r="G63" s="31" t="n"/>
+      <c r="D63" s="144" t="inlineStr">
+        <is>
+          <t>Мера предполагает создание и хранение резервных копий аутентификационных данных эксплуатационного персонала (в первую очередь — паролей от критичных привилегированных учётных записей, в том числе аварийных «break-glass» учётных записей) на выделенных машинных носителях информации (МНИ) либо на бумажных носителях, отдельно от систем, в которых эти данные используются.
+Главная цель меры — обеспечить возможность восстановления доступа к критичным системам в аварийной ситуации (например, при недоступности эксплуатационного персонала, владеющего паролем, или при отказе средств централизованного управления доступом), не полагаясь исключительно на память конкретных сотрудников или на системы, которые сами могут быть недоступны в момент аварии.</t>
+        </is>
+      </c>
+      <c r="E63" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационно это выражается в следующем:
+1. Определение перечня критичных привилегированных учётных записей, аутентификационные данные которых подлежат резервному хранению (аварийные учётные записи, учётные записи с полномочиями восстановления систем управления доступом);
+2. Утверждение порядка формирования, хранения и обновления резервных копий аутентификационных данных на выделенных МНИ или бумажных носителях (конвертах с печатью, сейф-пакетах);
+3. Определение места хранения (сейф, иное защищённое хранилище) и круга лиц, имеющих право доступа к резервным копиям аутентификационных данных;
+4. Установление порядка обновления резервных копий при плановой смене аутентификационных данных (см. также меры РД.19—РД.20, РД.29).</t>
+          </r>
+        </is>
+      </c>
+      <c r="F63" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент (порядок) формирования, хранения и обновления резервных копий аутентификационных данных эксплуатационного персонала;
+2. Перечень критичных привилегированных учётных записей, аутентификационные данные которых подлежат резервному хранению;
+3. Акты закладки (обновления) резервных копий аутентификационных данных на МНИ или бумажных носителях.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G63" s="151" t="inlineStr">
+        <is>
+          <t>1. Перечень критичных учётных записей, подлежащих резервному хранению аутентификационных данных, не определён или неполон;
+2. Резервные копии аутентификационных данных не обновляются при плановой или внеплановой смене паролей, что делает их фактически бесполезными;
+3. Место хранения резервных копий не защищено надлежащим образом (общедоступный сейф, отсутствие контроля доступа);
+4. Факты обращения к резервным копиям (в аварийных ситуациях) не фиксируются документально.</t>
+        </is>
+      </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4458,10 +5673,58 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D64" s="21" t="n"/>
-      <c r="E64" s="31" t="n"/>
-      <c r="F64" s="31" t="n"/>
-      <c r="G64" s="31" t="n"/>
+      <c r="D64" s="144" t="inlineStr">
+        <is>
+          <t>Мера дополняет требование РД.26 и устанавливает необходимость защиты самих резервных копий аутентификационных данных эксплуатационного персонала от несанкционированного доступа (НСД) в процессе их хранения на машинных носителях информации (МНИ) или бумажных носителях.
+Главная цель меры — исключить ситуацию, при которой резервные копии критичных паролей, созданные во исполнение меры РД.26 для аварийных случаев, сами становятся уязвимым звеном — то есть хранятся без надлежащей защиты и могут быть скомпрометированы лицом, не имеющим полномочий на доступ к ним.</t>
+        </is>
+      </c>
+      <c r="E64" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Со стороны организационных мер требуется:
+1. Определение требований к физической защите места хранения резервных копий аутентификационных данных (сейф с ограниченным кругом лиц, имеющих доступ, помещение с контролем доступа);
+2. Использование для бумажных носителей опечатанных конвертов (сейф-пакетов) с индикацией вскрытия, позволяющих визуально определить факт несанкционированного доступа;
+3. Для машинных носителей информации — применение шифрования содержимого носителя с ограничением круга лиц, обладающих ключом расшифрования;
+4. Ведение учёта (журнала) доступа к резервным копиям аутентификационных данных с фиксацией даты, времени, лица и цели обращения;
+5. Периодический контроль целостности хранения (проверка сохранности пломб (печатей), инвентаризация МНИ).</t>
+          </r>
+        </is>
+      </c>
+      <c r="F64" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент, устанавливающий требования к защите резервных копий аутентификационных данных от несанкционированного доступа;
+2. Акты проверки состояния мест хранения (сейфов), опечатанных конвертов и сейф-пакетов;
+3. Журнал учёта доступа к резервным копиям аутентификационных данных;
+4. Свидетельства применения шифрования для машинных носителей информации, содержащих резервные копии аутентификационных данных.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G64" s="151" t="inlineStr">
+        <is>
+          <t>1. Резервные копии аутентификационных данных хранятся в местах с широким кругом доступа (незапираемый шкаф, общий сейф без разграничения доступа);
+2. Бумажные носители не опечатываются способом, позволяющим выявить факт вскрытия;
+3. Машинные носители информации с резервными копиями аутентификационных данных не зашифрованы;
+4. Журнал учёта доступа к резервным копиям не ведётся или ведётся формально, не позволяя восстановить историю обращений.</t>
+        </is>
+      </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -4484,10 +5747,57 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D65" s="21" t="n"/>
-      <c r="E65" s="31" t="n"/>
-      <c r="F65" s="31" t="n"/>
-      <c r="G65" s="31" t="n"/>
+      <c r="D65" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует ведения учёта (регистрации) всего жизненного цикла персональных технических устройств аутентификации, используемых для многофакторной аутентификации (аппаратных токенов, смарт-карт, USB-ключей и подобных устройств): их персонализации (привязки к конкретному субъекту), выдачи (передачи) субъекту и последующего уничтожения (вывода из эксплуатации).
+Главная цель меры — обеспечить полную прослеживаемость обращения физических устройств аутентификации, поскольку без такого учёта невозможно достоверно установить, какому субъекту принадлежит конкретное устройство, находится ли оно у него на руках либо утрачено или не возвращено при увольнении, а также подтвердить факт надлежащего уничтожения выведенных из эксплуатации устройств.</t>
+        </is>
+      </c>
+      <c r="E65" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно организационными методами и предполагает:
+1. Ведение реестра (журнала) персональных технических устройств аутентификации с указанием серийного (уникального) номера устройства, субъекта, за которым оно закреплено, и статуса устройства (выдано, возвращено, уничтожено);
+2. Оформление факта выдачи (передачи) устройства субъекту актом или иным документом с подписью получателя;
+3. Оформление факта возврата устройства (при увольнении, замене, окончании срока действия) и его последующего уничтожения актом с участием комиссии или ответственного лица;
+4. Периодическую сверку данных реестра с фактическим наличием устройств у субъектов и фактическим статусом многофакторной аутентификации в соответствующих системах.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F65" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент (порядок) регистрации персонификации, выдачи и уничтожения персональных технических устройств аутентификации;
+2. Реестр (журнал) персональных технических устройств аутентификации;
+3. Акты выдачи (передачи) устройств субъектам;
+4. Акты уничтожения (списания) устройств, выведенных из эксплуатации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G65" s="151" t="inlineStr">
+        <is>
+          <t>1. Реестр устройств аутентификации ведётся не по всем выданным устройствам либо содержит устаревшие данные;
+2. Факт выдачи устройства субъекту не оформляется документально (акт отсутствует);
+3. При увольнении сотрудника устройство аутентификации не изымается и не деактивируется своевременно;
+4. Уничтожение выведенных из эксплуатации устройств не оформляется актом, что не позволяет подтвердить их фактическую утилизацию.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="20" t="inlineStr">
@@ -4505,10 +5815,56 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D66" s="21" t="n"/>
-      <c r="E66" s="31" t="n"/>
-      <c r="F66" s="31" t="n"/>
-      <c r="G66" s="31" t="n"/>
+      <c r="D66" s="144" t="inlineStr">
+        <is>
+          <t>Мера обязывает незамедлительно менять аутентификационные данные (пароли, а для устройств многофакторной аутентификации — переоформлять либо блокировать устройство) при выявлении факта их компрометации — то есть в случаях, когда есть основания полагать, что аутентификационные данные стали известны или могли стать известны лицу, не имеющему на это полномочий.
+Главная цель меры — минимизировать время, в течение которого скомпрометированные аутентификационные данные остаются действующими и потенциально могут использоваться злоумышленником, независимо от того, наступил ли для этого плановый срок смены пароля по мерам РД.19—РД.20.</t>
+        </is>
+      </c>
+      <c r="E66" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит организационный характер и включает:
+1. Определение во внутреннем нормативном документе признаков (событий), при которых аутентификационные данные считаются скомпрометированными или потенциально скомпрометированными (утеря устройства аутентификации, подозрение на фишинг, ввод пароля на постороннем ресурсе, инцидент информационной безопасности);
+2. Установление обязанности субъекта логического доступа немедленно сообщать о подозрении на компрометацию своих аутентификационных данных в подразделение информационной безопасности или service desk;
+3. Установление порядка и предельного срока внеплановой смены аутентификационных данных (или блокирования/переоформления устройства аутентификации) при получении сигнала о компрометации;
+4. Фиксацию факта компрометации и принятых мер в журнале инцидентов информационной безопасности.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F66" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний нормативный документ, определяющий признаки компрометации аутентификационных данных и порядок реагирования;
+2. Журнал (реестр) инцидентов, связанных с компрометацией аутентификационных данных, с указанием принятых мер;
+3. Свидетельства внеплановой смены аутентификационных данных (журналы смены паролей, акты переоформления устройств аутентификации) по зафиксированным случаям компрометации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G66" s="151" t="inlineStr">
+        <is>
+          <t>1. Субъекты логического доступа не осведомлены о необходимости и порядке сообщения о подозрении на компрометацию своих аутентификационных данных;
+2. Сроки внеплановой смены аутентификационных данных при подтверждённой компрометации не соблюдаются;
+3. Факты компрометации не фиксируются в едином журнале (реестре) инцидентов, что не позволяет оценить масштаб и повторяемость таких случаев;
+4. При компрометации пароля не проводится анализ возможных последствий (например, не проверяется, использовался ли этот же пароль для доступа к другим ресурсам).</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="13" t="inlineStr">
@@ -22768,8 +24124,8 @@
     <mergeCell ref="A423:G423"/>
     <mergeCell ref="A174:G174"/>
     <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A84:G84"/>
     <mergeCell ref="A286:G286"/>

</xml_diff>

<commit_message>
Fill РД.30-РД.44 (list «1. Описание мер», rows 68-83) per VIKI_measure_filling_rules.md
- 8 measures with all of D-G written from scratch: РД.30-35, РД.38,
  РД.44
- 7 measures with a pre-existing D kept, E/F/G added: РД.36, РД.37,
  РД.39-43
- РД.39: fixed a duplicated-letter typo in D
- РД.40, РД.41: fixed a garbled clause in D (nonsensical claim about
  what session/login logging 'reduces') while keeping the rest of the
  text
- РД.43: fixed dash-list punctuation in D (mid-list items were ending
  with '.' instead of ';')
- All filled/rewritten cells shaded pale yellow for review
</commit_message>
<xml_diff>
--- a/docs/WIKI GOST R 57580.1.xlsx
+++ b/docs/WIKI GOST R 57580.1.xlsx
@@ -334,7 +334,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -797,6 +797,9 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -5895,10 +5898,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D68" s="21" t="n"/>
-      <c r="E68" s="31" t="n"/>
-      <c r="F68" s="31" t="n"/>
-      <c r="G68" s="31" t="n"/>
+      <c r="D68" s="144" t="inlineStr">
+        <is>
+          <t>Мера устанавливает базовое техническое требование: любое обращение субъекта логического доступа к ресурсу доступа (в том числе к автоматизированной системе (АС)) должно сопровождаться процедурой авторизации — проверкой того, что данному субъекту действительно предоставлены права на запрашиваемое действие.
+Главная цель меры — гарантировать, что успешного прохождения идентификации и аутентификации (мер РД.1—РД.7) недостаточно для получения доступа к конкретному ресурсу: должна выполняться отдельная проверка полномочий, без которой любой аутентифицированный субъект мог бы обращаться к любым ресурсам вне зависимости от предоставленных ему прав.</t>
+        </is>
+      </c>
+      <c r="E68" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется на техническом уровне без организационной составляющей:
+1. Настройку операционных систем, СУБД, прикладного ПО и сетевого оборудования таким образом, чтобы каждое обращение к ресурсу доступа проверялось на соответствие фактически предоставленным правам, независимо от факта успешной аутентификации;
+2. Использование встроенных механизмов авторизации ресурсов доступа (списки контроля доступа — ACL, ролевые модели, политики доступа) в каждой информационной системе;
+3. Технический запрет на выполнение операций, не охваченных явно предоставленными правами субъекта («запрет по умолчанию» — default deny).
+Класс используемых средств — встроенные механизмы авторизации операционных систем, СУБД и прикладного ПО, средства защиты от несанкционированного доступа (СЗИ от НСД).
+Иностранные: Microsoft Active Directory (списки контроля доступа), Oracle Database (Fine-Grained Access Control) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К и др.
+Открытый код: SELinux, PostgreSQL (Row-Level Security) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F68" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек авторизации (списков контроля доступа, ролевых моделей) в информационных системах;
+3. Результаты тестирования (попытка обращения аутентифицированного, но не авторизованного субъекта к ресурсу), подтверждающие срабатывание запрета;
+4. Журналы событий, подтверждающие регистрацию решений об авторизации (разрешении/отказе в доступе).</t>
+          </r>
+        </is>
+      </c>
+      <c r="G68" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные ресурсы доступа (в том числе АС) не проверяют права субъекта при обращении, полагаясь только на факт успешной аутентификации;
+2. Модель авторизации построена по принципу «разрешено по умолчанию», а не «запрещено по умолчанию», что создаёт риск избыточного доступа к неучтённым функциям;
+3. Настройки авторизации не покрывают все точки доступа к ресурсу (например, отсутствуют для программных интерфейсов — API);
+4. Тестирование фактического срабатывания механизма авторизации не проводится.</t>
+        </is>
+      </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -5921,10 +5974,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D69" s="21" t="n"/>
-      <c r="E69" s="31" t="n"/>
-      <c r="F69" s="31" t="n"/>
-      <c r="G69" s="31" t="n"/>
+      <c r="D69" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы в каждом ресурсе доступа применялся метод разграничения логического доступа, соответствующий характеру обрабатываемой информации и уровню защиты, — дискреционный (управление доступом на основе прав, назначаемых владельцем ресурса), мандатный (управление доступом на основе меток конфиденциальности) или ролевой (управление доступом на основе ролей субъектов), либо иной обоснованный метод.
+Главная цель меры — обеспечить осознанный и соответствующий специфике ресурса выбор модели разграничения доступа, а не бессистемное предоставление прав, поскольку выбор неподходящего или отсутствие какого-либо формализованного метода делает управление доступом непрозрачным и труднопроверяемым.</t>
+        </is>
+      </c>
+      <c r="E69" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера реализуется только техническими средствами, необходимо:
+1. Определение для каждого ресурса доступа (АС, СУБД, файлового ресурса и т. д.) применимого метода разграничения доступа исходя из специфики обрабатываемой информации и архитектуры ресурса;
+2. Настройку выбранного метода средствами самого ресурса доступа (дискреционные списки контроля доступа, мандатные метки конфиденциальности, ролевые модели);
+3. Технический контроль того, что разграничение доступа выполняется именно выбранным методом, а не в обход него (например, через прямой доступ к данным на уровне файловой системы или СУБД, минуя прикладную логику авторизации).
+Класс используемых средств — встроенные механизмы разграничения доступа операционных систем и СУБД, средства защиты от несанкционированного доступа (СЗИ от НСД) с поддержкой мандатного управления доступом.
+Иностранные: Microsoft Active Directory (дискреционная модель), Oracle Label Security (мандатная модель) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Astra Linux Special Edition (мандатное управление доступом) и др.
+Открытый код: SELinux (мандатное управление доступом) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F69" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Проектная (эксплуатационная) документация ресурсов доступа, содержащая описание применяемого метода разграничения доступа;
+3. Скриншоты настроек, подтверждающие фактическую реализацию выбранного метода;
+4. Результаты тестирования, подтверждающие невозможность обхода выбранного метода разграничения доступа.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G69" s="151" t="inlineStr">
+        <is>
+          <t>1. Метод разграничения доступа не определён и не обоснован документально для части ресурсов доступа;
+2. Заявленный метод (например, мандатный) реализован не в полном объёме, фактически используется упрощённая дискреционная модель;
+3. Существуют технические пути обхода установленного метода разграничения доступа (прямой доступ к данным в обход прикладной логики);
+4. Настройки метода разграничения доступа не пересматриваются при изменении состава обрабатываемой информации.</t>
+        </is>
+      </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -5947,10 +6050,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D70" s="21" t="n"/>
-      <c r="E70" s="31" t="n"/>
-      <c r="F70" s="31" t="n"/>
-      <c r="G70" s="31" t="n"/>
+      <c r="D70" s="144" t="inlineStr">
+        <is>
+          <t>Мера конкретизирует РД.31 применительно к автоматизированным системам (АС): в них должен применяться именно ролевой метод разграничения доступа (Role-Based Access Control, RBAC), при котором для каждой роли заранее определён чётко зафиксированный набор прав доступа, а субъектам права предоставляются через назначение соответствующей роли, а не по отдельности.
+Главная цель меры — упростить и сделать прозрачным управление правами доступа в АС за счёт группировки прав в типовые роли, соответствующие производственным функциям субъектов, что снижает риск ошибок при назначении прав и облегчает последующий контроль (в том числе в рамках мер УЗП.8—УЗП.9).</t>
+        </is>
+      </c>
+      <c r="E70" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера подразумевает исключительно технические меры защиты, а именно:
+1. Разработку и настройку в АС ролевой модели: определение перечня ролей, соответствующих производственным функциям субъектов, и фиксацию для каждой роли конкретного набора прав доступа к функциям и данным АС;
+2. Настройку АС таким образом, чтобы предоставление прав доступа субъекту выполнялось исключительно через назначение ему одной или нескольких ролей, без возможности точечного (вне ролевой модели) назначения отдельных прав;
+3. Технический контроль соответствия фактически предоставленных прав заявленному составу прав для назначенных субъекту ролей.
+Класс используемых средств — встроенные механизмы ролевого управления доступом (RBAC) прикладного ПО и АС, системы управления учётными записями и правами доступа (IdM) с поддержкой ролевых моделей.
+Иностранные: SAP (ролевая модель авторизаций), Microsoft Dynamics (RBAC) и пр.
+Российские сертифицированные (ФСТЭК): Avanpost IDM, Solar inRights и др.
+Открытый код: Keycloak (Role-Based Access Control) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F70" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами АС;
+2. Проектная документация АС, содержащая описание ролевой модели и состава прав каждой роли;
+3. Скриншоты настроек ролевой модели в АС;
+4. Результаты тестирования (сопоставление фактических прав субъекта с заявленным составом прав его роли (ролей)).</t>
+          </r>
+        </is>
+      </c>
+      <c r="G70" s="151" t="inlineStr">
+        <is>
+          <t>1. Ролевая модель в АС не охватывает все функции и данные, часть прав предоставляется точечно, в обход ролей;
+2. Роли определены нечётко, их состав пересекается, что затрудняет контроль фактически предоставленных прав;
+3. Роли не пересматриваются при изменении функциональности АС, актуальность состава прав каждой роли не подтверждается;
+4. Одному субъекту назначено избыточное количество ролей без документированного обоснования служебной необходимости.</t>
+        </is>
+      </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -5973,10 +6126,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D71" s="21" t="n"/>
-      <c r="E71" s="31" t="n"/>
-      <c r="F71" s="31" t="n"/>
-      <c r="G71" s="31" t="n"/>
+      <c r="D71" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы разграничение логического доступа выполнялось не только на уровне «есть доступ / нет доступа» к ресурсу в целом, но и по конкретным типам операций — чтению, записи, выполнению или иным применимым типам, — с определением правил, по которым тот или иной тип доступа предоставляется субъекту.
+Главная цель меры — реализовать принцип минимально необходимых прав на уровне операций: субъект должен получать только те типы доступа к ресурсу, которые действительно необходимы ему для выполнения служебных обязанностей (например, право только на чтение данных без права их изменения), а не полный доступ ко всем операциям с ресурсом.</t>
+        </is>
+      </c>
+      <c r="E71" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Ввиду того, что мера реализуется только технически, необходимо:
+1. Настройку ресурсов доступа (файловых систем, СУБД, прикладного ПО) таким образом, чтобы для субъекта можно было раздельно предоставлять права на чтение, запись, выполнение и иные применимые операции;
+2. Определение и документальное закрепление правил, по которым субъектам предоставляется тот или иной тип доступа (например, право на запись предоставляется только субъектам, ответственным за ввод и изменение данных, право на чтение — более широкому кругу субъектов);
+3. Технический контроль того, что субъекту не предоставлен более широкий тип доступа, чем это предусмотрено установленными правилами (например, исключение случаев, когда право на чтение фактически сопровождается и правом на запись).
+Класс используемых средств — встроенные механизмы разграничения доступа операционных систем, файловых систем и СУБД (списки контроля доступа — ACL, права на уровне объектов).
+Иностранные: Microsoft NTFS (права на уровне файлов и папок), Oracle Database (системные и объектные привилегии) и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Astra Linux Special Edition и др.
+Открытый код: файловые права POSIX (ACL), PostgreSQL (GRANT/REVOKE) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F71" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Внутренний документ, определяющий правила предоставления субъектам различных типов доступа (чтение, запись, выполнение);
+3. Скриншоты настроек, подтверждающие раздельное разграничение типов доступа к ресурсу;
+4. Результаты тестирования (проверка фактического типа доступа субъекта к ресурсу на соответствие установленным правилам).</t>
+          </r>
+        </is>
+      </c>
+      <c r="G71" s="151" t="inlineStr">
+        <is>
+          <t>1. Правила предоставления различных типов доступа не формализованы документально;
+2. Субъектам систематически предоставляется более широкий тип доступа, чем необходимо (например, право на запись вместо права только на чтение);
+3. Отдельные ресурсы доступа не поддерживают раздельное разграничение по типам операций, что вынуждает предоставлять полный доступ;
+4. Соответствие фактически предоставленных типов доступа установленным правилам не проверяется на регулярной основе.</t>
+        </is>
+      </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -5999,10 +6202,89 @@
           <t>О-Т-Т</t>
         </is>
       </c>
-      <c r="D72" s="21" t="n"/>
-      <c r="E72" s="31" t="n"/>
-      <c r="F72" s="31" t="n"/>
-      <c r="G72" s="31" t="n"/>
+      <c r="D72" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает пользователям выполнять бизнес-процессы и технологические процессы (то есть их обычную рабочую деятельность) под учётными записями эксплуатационного персонала — привилегированными административными учётными записями, предназначенными для эксплуатации и администрирования систем, а не для выполнения повседневных операций.
+Главная цель меры — предотвратить смешение ролей пользователя и администратора: использование привилегированной учётной записи для рутинных операций резко увеличивает потенциальный ущерб от компрометации такой учётной записи или от ошибки пользователя, а также обесценивает разграничение прав, установленное мерами УЗП.19—УЗП.21.</t>
+        </is>
+      </c>
+      <c r="E72" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная составляющая сводится к следующим шагам:
+1. Закрепление во внутреннем нормативном документе прямого запрета на использование учётных записей эксплуатационного персонала для выполнения бизнес-процессов и технологических процессов, не относящихся к эксплуатации и администрированию систем;
+2. Информирование эксплуатационного персонала о данном запрете и о необходимости использования отдельной персональной пользовательской учётной записи для непроизводственных (не связанных с администрированием) операций;
+3. Периодический контроль (анализ журналов, выборочные проверки) фактического использования привилегированных учётных записей на предмет выполнения под ними операций бизнес- и технологических процессов.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Технически права логического доступа разграничиваются так:
+1. Предоставление эксплуатационному персоналу двух раздельных учётных записей — привилегированной (административной) для задач эксплуатации и обычной пользовательской для выполнения непроизводственных операций (при их наличии у данного сотрудника);
+2. Технический запрет использования привилегированных учётных записей для входа в АС и выполнения в них функций, относящихся к бизнес-процессам и технологическим процессам (например, ограничение состава ролей, доступных привилегированной учётной записи, только административными функциями);
+3. Регистрацию и автоматизированный анализ фактов выполнения под привилегированными учётными записями операций, типичных для бизнес-процессов, с оповещением подразделения информационной безопасности при выявлении таких фактов.
+Класс используемых средств — системы управления привилегированным доступом (PAM), системы управления событиями информационной безопасности (SIEM).
+Иностранные: CyberArk PAM, Splunk (для анализа журналов) и пр.
+Российские сертифицированные (ФСТЭК): Indeed Privileged Access Manager, MaxPatrol SIEM и др.
+Открытый код: Teleport, Wazuh и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F72" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний нормативный документ, содержащий запрет на использование учётных записей эксплуатационного персонала для выполнения бизнес- и технологических процессов;
+2. Материалы информирования (инструктажа) эксплуатационного персонала о данном запрете;
+3. Акты (отчёты) периодического контроля фактического использования привилегированных учётных записей.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Выгрузка перечня учётных записей эксплуатационного персонала, подтверждающая наличие раздельных привилегированной и пользовательской учётных записей;
+3. Скриншоты настроек, ограничивающих состав ролей, доступных привилегированной учётной записи, административными функциями;
+4. Журналы событий (отчёты SIEM), подтверждающие анализ фактов выполнения бизнес-операций под привилегированными учётными записями.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G72" s="151" t="inlineStr">
+        <is>
+          <t>1. Эксплуатационному персоналу не выделяется отдельная пользовательская учётная запись, вся деятельность (включая непроизводственную) выполняется под привилегированной учётной записью;
+2. Технический запрет на выполнение бизнес-операций под привилегированными учётными записями не реализован, ограничение носит только организационный (декларативный) характер;
+3. Анализ журналов на предмет выполнения бизнес-операций под привилегированными учётными записями не проводится;
+4. Запрет не доведён до сведения эксплуатационного персонала.</t>
+        </is>
+      </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6025,10 +6307,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D73" s="21" t="n"/>
-      <c r="E73" s="31" t="n"/>
-      <c r="F73" s="31" t="n"/>
-      <c r="G73" s="31" t="n"/>
+      <c r="D73" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает пользователям выполнять бизнес-процессы, обладая привилегированными правами логического доступа, — в частности, запрещает повседневную работу пользователя на автоматизированном рабочем месте (АРМ) под учётной записью с правами локального администратора.
+Главная цель меры — минимизировать потенциальный ущерб от компрометации рабочей станции пользователя (например, в результате заражения вредоносным ПО или фишинговой атаки): если пользователь работает без привилегированных прав, вредоносный код, запущенный от его имени, также не получает административных полномочий на АРМ, что существенно ограничивает возможности злоумышленника закрепиться в системе или распространиться на другие ресурсы.</t>
+        </is>
+      </c>
+      <c r="E73" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Настройку учётных записей пользователей таким образом, чтобы для повседневной работы (выполнения бизнес-процессов) использовалась учётная запись без прав локального администратора и без иных привилегированных прав логического доступа;
+2. Реализацию отдельного, контролируемого механизма временного повышения привилегий для случаев, когда пользователю действительно необходимо выполнить операцию, требующую административных прав (запрос повышения привилегий с санкционированием и регистрацией);
+3. Технический контроль (аудит состава локальных администраторов АРМ), выявляющий и устраняющий случаи, когда обычные пользователи фактически обладают правами локального администратора.
+Класс используемых средств — средства управления привилегиями на конечных точках (Endpoint Privilege Management), системы управления конфигурациями.
+Иностранные: Microsoft Defender for Endpoint (совместно с политиками ограничения прав), CyberArk Endpoint Privilege Manager и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К и др.
+Открытый код: групповые политики Linux/Windows без выделенных общепринятых открытых аналогов и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F73" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами АРМ;
+2. Выгрузка перечня локальных администраторов АРМ, подтверждающая отсутствие среди них рядовых пользователей;
+3. Скриншоты настроек механизма временного повышения привилегий (при его наличии);
+4. Результаты аудита (сканирования) АРМ на предмет фактического состава локальных администраторов.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G73" s="151" t="inlineStr">
+        <is>
+          <t>1. Часть пользователей продолжает работать с правами локального администратора АРМ по факту исторически сложившейся практики;
+2. Механизм временного контролируемого повышения привилегий отсутствует, что вынуждает администраторов постоянно предоставлять пользователям административные права «про запас»;
+3. Аудит фактического состава локальных администраторов АРМ не проводится на регулярной основе;
+4. Выявленные случаи наличия у пользователя прав локального администратора не устраняются в разумный срок.</t>
+        </is>
+      </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6057,9 +6389,50 @@
 Главная цель меры — снижение риска несанкционированного доступа и своевременное выявление факта компрометации учётной записи. Если пользователь видит, что его предыдущий вход был совершён в то время, когда он точно не работал в системе, это является явным признаком того, что его учётные данные были использованы злоумышленником. Пользователь может оперативно среагировать: сменить пароль и сообщить о случившемся в службу информационной безопасности.</t>
         </is>
       </c>
-      <c r="E74" s="31" t="n"/>
-      <c r="F74" s="31" t="n"/>
-      <c r="G74" s="31" t="n"/>
+      <c r="E74" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит чисто технический характер и включает:
+1. Настройку АС таким образом, чтобы после успешной авторизации субъекту отображалось информационное сообщение с датой и временем его предыдущего успешного входа в данную АС;
+2. Хранение в системе сведений о дате и времени предыдущих успешных авторизаций каждого субъекта в объёме, достаточном для формирования такого уведомления;
+3. Обеспечение того, что данное уведомление не может быть отключено или скрыто самим пользователем.
+Отдельного специализированного средства защиты для реализации меры, как правило, не требуется: функция реализуется на уровне логики самой АС и её встроенных механизмов идентификации и аутентификации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F74" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с пользователями и разработчиками (администраторами) АС;
+2. Скриншоты интерфейса АС, подтверждающие отображение уведомления о дате и времени предыдущей авторизации;
+3. Результаты тестирования (последовательный вход под одной учётной записью), подтверждающие корректность отображаемых даты и времени.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G74" s="151" t="inlineStr">
+        <is>
+          <t>1. Функция реализована не во всех АС, к которым субъекты осуществляют логический доступ;
+2. Отображаемые дата и время предыдущей авторизации не соответствуют фактическим (ошибка логики учёта);
+3. Уведомление отображается слишком кратковременно или в неприметном месте интерфейса, из-за чего пользователи его не замечают;
+4. Пользователи не проинформированы о значении данного уведомления и о необходимых действиях в случае обнаружения несоответствия.</t>
+        </is>
+      </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6088,9 +6461,48 @@
 Главная цель меры — минимизировать риски несанкционированных действий и атак на этапе, когда личность пользователя ещё не подтверждена. Это предотвращает возможность получения доступа к защищённым ресурсам, выполнения операций или сбора информации о системе до прохождения аутентификации.</t>
         </is>
       </c>
-      <c r="E75" s="31" t="n"/>
-      <c r="F75" s="31" t="n"/>
-      <c r="G75" s="31" t="n"/>
+      <c r="E75" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера выполняется силами технических средств защиты информации, а именно:
+1. Настройку АС таким образом, чтобы до прохождения идентификации и аутентификации субъекту были доступны исключительно минимально необходимые функции (например, отображение формы входа, общая информация об организации без раскрытия структуры системы);
+2. Технический запрет на получение до аутентификации какой-либо информации о внутренней архитектуре АС, версиях используемого ПО, структуре базы данных и иных технических деталях, которые могут быть использованы для подготовки атаки;
+3. Настройку обработки ошибок таким образом, чтобы сообщения об ошибках на этапе входа не раскрывали избыточные технические подробности (например, обобщённое сообщение «неверный логин или пароль» вместо детализации, какая именно часть учётных данных неверна).</t>
+          </r>
+        </is>
+      </c>
+      <c r="F75" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с разработчиками и администраторами АС;
+2. Результаты тестирования (попытка получить доступ к функциям или информации АС до прохождения аутентификации), подтверждающие ограничение состава доступных действий;
+3. Скриншоты сообщений об ошибках на этапе входа, подтверждающие отсутствие избыточной технической детализации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G75" s="151" t="inlineStr">
+        <is>
+          <t>1. До прохождения аутентификации пользователю доступны отдельные функции АС сверх необходимого минимума (например, часть справочной информации, раскрывающей структуру системы);
+2. Сообщения об ошибках на этапе входа раскрывают избыточные технические подробности (версии ПО, структуру базы данных, стек трассировки);
+3. Тестирование состава действий, доступных до аутентификации, не проводится на регулярной основе.</t>
+        </is>
+      </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6113,10 +6525,56 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D76" s="21" t="n"/>
-      <c r="E76" s="53" t="n"/>
-      <c r="F76" s="53" t="n"/>
-      <c r="G76" s="53" t="n"/>
+      <c r="D76" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует такого физического размещения устройств вывода (отображения) информации — мониторов, экранов, панелей — при котором исключается возможность несанкционированного просмотра отображаемой на них защищаемой информации посторонними лицами (так называемый visual hacking, shoulder surfing).
+Главная цель меры — исключить утечку защищаемой информации через простое визуальное наблюдение за экраном, поскольку такой канал утечки не требует от нарушителя никаких технических средств или специальных знаний — достаточно оказаться в поле зрения экрана.</t>
+        </is>
+      </c>
+      <c r="E76" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационно это выражается в следующем:
+1. Определение требований к размещению устройств вывода информации, исключающих просмотр экрана с мест, доступных посторонним лицам (например, разворот мониторов от окон, дверных проёмов, зон обслуживания клиентов);
+2. Учёт данных требований при планировке рабочих мест, на которых обрабатывается защищаемая информация, а также при организации рабочих мест эксплуатационного персонала;
+3. Применение дополнительных организационных мер там, где оптимальное размещение технически невозможно (например, временное затемнение, использование перегородок);
+4. Периодический контроль соблюдения установленных требований к размещению устройств вывода информации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F76" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний документ, определяющий требования к размещению устройств вывода информации;
+2. Результаты выборочного визуального осмотра рабочих мест на предмет соблюдения установленных требований;
+3. Акты (отчёты) периодического контроля соблюдения требований к размещению устройств вывода информации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G76" s="157" t="inlineStr">
+        <is>
+          <t>1. Требования к размещению устройств вывода информации не формализованы документально;
+2. Мониторы отдельных рабочих мест обращены в сторону зон, доступных клиентам или посторонним лицам (зоны обслуживания, коридоры, окна первого этажа);
+3. Периодический контроль соблюдения требований не проводится;
+4. Требования не учитываются при организации новых рабочих мест или при перепланировке помещений.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
@@ -6147,17 +6605,62 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D78" s="44" t="inlineStr">
+      <c r="D78" s="153" t="inlineStr">
         <is>
           <t>Суть меры заключается в обязательной фиксации в журналах событий всех случаев, когда субъект логического доступа (пользователь, эксплуатационный персонал или программный сервис) совершает ряд неуспешных последовательных попыток аутентификации.
 Главная цель меры — создание доказательной базы для:
-- cсвоевременного выявления атак на подбор паролей и иных попыток несанкционированного доступа;
+- своевременного выявления атак на подбор паролей и иных попыток несанкционированного доступа;
 - расследования инцидентов безопасности, связанных с компрометацией учётных записей.</t>
         </is>
       </c>
-      <c r="E78" s="31" t="n"/>
-      <c r="F78" s="31" t="n"/>
-      <c r="G78" s="31" t="n"/>
+      <c r="E78" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как речь идёт о чисто технической мере, реализация включает:
+1. Настройку операционных систем, каталогов (Active Directory, LDAP) и прикладных информационных систем на регистрацию событий каждой неуспешной попытки аутентификации субъекта;
+2. Настройку правил (например, в SIEM-системе) для выявления последовательных неуспешных попыток аутентификации, указывающих на возможную атаку подбора пароля;
+3. Обеспечение достаточного срока хранения журналов регистрации таких событий для последующего анализа и расследования инцидентов.
+Класс используемых средств — системы управления событиями информационной безопасности (SIEM), встроенные средства аудита операционных систем и служб каталогов.
+Иностранные: Splunk, Microsoft Active Directory (Audit Logon Events) и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, RuSIEM и др.
+Открытый код: Wazuh, ELK Stack (Elasticsearch, Logstash, Kibana) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F78" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем и подразделением информационной безопасности;
+2. Скриншоты настроек, подтверждающие регистрацию неуспешных попыток аутентификации;
+3. Выгрузка журналов событий с зафиксированными неуспешными попытками аутентификации за проверяемый период;
+4. Правила корреляции SIEM-системы (при наличии), настроенные на выявление последовательных неуспешных попыток аутентификации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G78" s="151" t="inlineStr">
+        <is>
+          <t>1. Регистрация неуспешных попыток аутентификации включена не для всех информационных систем;
+2. События неуспешных попыток аутентификации собираются, но не анализируются на предмет выявления атак подбора пароля;
+3. Журналы событий хранятся менее срока, необходимого для расследования инцидентов;
+4. Отсутствуют настроенные оповещения о превышении порогового числа неуспешных попыток аутентификации в единицу времени.</t>
+        </is>
+      </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6180,18 +6683,62 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D79" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует фиксирования в журналах регистрации событий всех фактов идентификации и аутентификации (логина и пароля) при входе в ресурс доступа (СУБД, АС и т.п.) пользователями логического доступа, что снижает возможность фильтрации нелегитимных действий в нерабочее время. 
+      <c r="D79" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует фиксирования в журналах регистрации событий всех фактов идентификации и аутентификации (логина и пароля) при входе субъектов логического доступа в ресурс доступа (СУБД, АС и т. п.), что позволяет впоследствии выявлять факты входа в систему в нехарактерное для субъекта время (например, в нерабочие часы).
 Главная цель меры — создание доказательной базы для:
 - подтверждения факта входа конкретного субъекта в систему в определённое время;
 - расследования инцидентов безопасности;
 - обеспечения прозрачности и подотчётности всех действий субъектов логического доступа.</t>
         </is>
       </c>
-      <c r="E79" s="31" t="n"/>
-      <c r="F79" s="31" t="n"/>
-      <c r="G79" s="31" t="n"/>
+      <c r="E79" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера не имеет организационной составляющей — её выполнение обеспечивается техническими средствами:
+1. Настройку встроенных механизмов аудита операционных систем, СУБД, АС и служб каталогов на регистрацию каждого факта успешной идентификации и аутентификации субъекта;
+2. Фиксацию в журнале как минимум даты и времени события, идентификатора субъекта и результата (успешно/неуспешно);
+3. Централизованный сбор данных журналов идентификации и аутентификации из различных источников для последующего анализа.
+Класс используемых средств — системы управления событиями информационной безопасности (SIEM), встроенные средства аудита операционных систем, СУБД и служб каталогов.
+Иностранные: Splunk, Microsoft Active Directory (Audit Logon Events) и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, RuSIEM и др.
+Открытый код: Wazuh, ELK Stack и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F79" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек аудита, подтверждающие регистрацию фактов идентификации и аутентификации;
+3. Выгрузка журналов событий идентификации и аутентификации за проверяемый период.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G79" s="151" t="inlineStr">
+        <is>
+          <t>1. Регистрация фактов идентификации и аутентификации включена не для всех информационных систем;
+2. Журналы не содержат достаточного набора атрибутов (например, отсутствует точное время события);
+3. Журналы событий разных систем не собираются централизованно, что затрудняет их анализ;
+4. Журналы хранятся менее установленного срока, что не позволяет предоставить свидетельства за требуемый период.</t>
+        </is>
+      </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6214,15 +6761,59 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D80" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует фиксирования в журналах регистрации событий всех событий, связанных с предоставлением доступа (авторизацией), с завершением или принудительным прерыванием сеанса работы пользователей и эксплуатационного персонала в ресурс доступа (СУБД, АС и т.п.), что снижает риск создания полной цепочки событий в рамках сессии логического доступа нелегитимным пользователем.
+      <c r="D80" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует фиксирования в журналах регистрации событий всех событий, связанных с предоставлением доступа (авторизацией), с завершением или принудительным прерыванием сеанса работы пользователей и эксплуатационного персонала в ресурсе доступа (СУБД, АС и т. п.), что позволяет восстановить полную и непрерывную цепочку событий в рамках каждой сессии логического доступа.
 Главная цель меры — создание полной и непрерывной доказательной базы всех этапов сессии логического доступа: от предоставления прав (авторизация) до её завершения или прерывания.</t>
         </is>
       </c>
-      <c r="E80" s="31" t="n"/>
-      <c r="F80" s="31" t="n"/>
-      <c r="G80" s="31" t="n"/>
+      <c r="E80" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит организационно необременительный, полностью технический характер:
+1. Настройку АС и иных ресурсов доступа на регистрацию события авторизации сессии (момента предоставления доступа после успешной идентификации и аутентификации);
+2. Настройку регистрации события завершения сессии — как штатного (выход пользователя), так и принудительного или автоматического прерывания (в том числе в рамках мер РД.13—РД.14);
+3. Обеспечение возможности сопоставления событий начала и завершения сессии по единому идентификатору (идентификатору сессии), позволяющего восстановить полную хронологию сессии.
+Класс используемых средств — системы управления событиями информационной безопасности (SIEM), встроенные средства аудита АС и служб каталогов.
+Иностранные: Splunk, Microsoft Active Directory (Audit Logon/Logoff Events) и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, RuSIEM и др.
+Открытый код: Wazuh, ELK Stack и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F80" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами АС;
+2. Скриншоты настроек, подтверждающие регистрацию событий авторизации, завершения и прерывания сессии;
+3. Выгрузка журналов событий, подтверждающая возможность сопоставления начала и завершения одной и той же сессии.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G80" s="151" t="inlineStr">
+        <is>
+          <t>1. Регистрация событий завершения (прерывания) сессии реализована не для всех АС, где регистрируется её начало;
+2. События начала и завершения сессии невозможно сопоставить между собой (отсутствует единый идентификатор сессии);
+3. Принудительное или аварийное прерывание сессии (например, при сбое) не регистрируется;
+4. Журналы событий сессий разных систем не собираются централизованно.</t>
+        </is>
+      </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6251,9 +6842,53 @@
 Главная цель меры — обеспечить прозрачность и подотчётность всех автоматизированных процессов, которые взаимодействуют с информационными системами. Это критически важно, так как программные сервисы, как правило, обладают высокими привилегиями и их деятельность часто остаётся вне поля зрения администраторов.</t>
         </is>
       </c>
-      <c r="E81" s="31" t="n"/>
-      <c r="F81" s="31" t="n"/>
-      <c r="G81" s="31" t="n"/>
+      <c r="E81" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как организационных мер здесь не предусмотрено, всё сводится к техническим настройкам:
+1. Настройку регистрации события запуска каждого программного сервиса (службы, приложения, скрипта автоматизации), осуществляющего логический доступ к информационным ресурсам от имени технической учётной записи;
+2. Фиксацию в журнале как минимум даты и времени запуска, идентификатора сервиса и технической учётной записи, от имени которой он запущен;
+3. Централизованный сбор данных о запуске программных сервисов для последующего анализа на предмет выявления несанкционированного или аномального запуска.
+Класс используемых средств — системы управления событиями информационной безопасности (SIEM), средства мониторинга процессов и служб операционных систем.
+Иностранные: Splunk, Microsoft Sysmon (мониторинг запуска процессов) и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, RuSIEM и др.
+Открытый код: Wazuh, osquery и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F81" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек, подтверждающие регистрацию событий запуска программных сервисов;
+3. Выгрузка журналов событий запуска программных сервисов за проверяемый период.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G81" s="151" t="inlineStr">
+        <is>
+          <t>1. Регистрация запуска программных сервисов включена не для всех технических учётных записей;
+2. Журналы запуска сервисов не анализируются на предмет выявления аномального (незапланированного) запуска;
+3. Запуск сервисов с непредусмотренными правами (эскалация привилегий при старте) не выявляется;
+4. Журналы запуска программных сервисов хранятся менее установленного срока.</t>
+        </is>
+      </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6276,18 +6911,62 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D82" s="56" t="inlineStr">
+      <c r="D82" s="158" t="inlineStr">
         <is>
           <t>Суть меры заключается в обязательной фиксации в журналах событий всех случаев изменения аутентификационных данных, используемых субъектами логического доступа для входа в информационные системы.
 Главная цель меры — создание полной и непрерывной доказательной базы всех изменений аутентификационных данных для:
-- расследования инцидентов безопасности, связанных с компрометацией учётных записей.
-- выявления аномалий (например, массовая смена паролей, смена пароля администратором без ведома пользователя).
+- расследования инцидентов безопасности, связанных с компрометацией учётных записей;
+- выявления аномалий (например, массовая смена паролей, смена пароля администратором без ведома пользователя);
 - подтверждения факта выполнения регламентных процедур смены аутентификационных данных.</t>
         </is>
       </c>
-      <c r="E82" s="31" t="n"/>
-      <c r="F82" s="31" t="n"/>
-      <c r="G82" s="31" t="n"/>
+      <c r="E82" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно техническими средствами:
+1. Настройку операционных систем, каталогов, СУБД и прикладных информационных систем на регистрацию каждого факта изменения аутентификационных данных субъекта (смены пароля, перевыпуска сертификата, привязки/отвязки фактора МФА);
+2. Фиксацию в журнале как минимум даты и времени изменения, идентификатора субъекта, инициатора изменения (сам субъект или администратор) и результата операции;
+3. Централизованный сбор данных об изменениях аутентификационных данных для последующего анализа на предмет аномалий.
+Класс используемых средств — системы управления событиями информационной безопасности (SIEM), службы каталогов и системы управления учётными записями (IdM) со встроенным аудитом.
+Иностранные: Splunk, Microsoft Active Directory (Audit Credential Validation) и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, Avanpost IDM и др.
+Открытый код: Wazuh, ELK Stack и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F82" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами информационных систем;
+2. Скриншоты настроек, подтверждающие регистрацию событий изменения аутентификационных данных;
+3. Выгрузка журналов событий изменения аутентификационных данных за проверяемый период.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G82" s="151" t="inlineStr">
+        <is>
+          <t>1. Регистрация изменений аутентификационных данных включена не для всех информационных систем;
+2. Журналы не позволяют определить, кто инициировал изменение — сам субъект или администратор от его имени;
+3. Массовые (аномальные) изменения аутентификационных данных не выявляются автоматически;
+4. Журналы событий изменения аутентификационных данных хранятся менее установленного срока.</t>
+        </is>
+      </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -6310,10 +6989,53 @@
           <t>Н-О-О</t>
         </is>
       </c>
-      <c r="D83" s="21" t="n"/>
-      <c r="E83" s="31" t="n"/>
-      <c r="F83" s="31" t="n"/>
-      <c r="G83" s="31" t="n"/>
+      <c r="D83" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует регистрации (документальной фиксации) действий, которые субъект логического доступа и вовлечённые сотрудники обязаны выполнить в случае компрометации его аутентификационных данных, — то есть действий, предусмотренных мерой РД.29 (сообщение о компрометации, внеплановая смена аутентификационных данных, иные реагирующие мероприятия).
+Главная цель меры — обеспечить документальное подтверждение того, что при каждом зафиксированном случае компрометации аутентификационных данных предусмотренные действия были выполнены фактически, а не только формально предписаны регламентом (мера РД.29).</t>
+        </is>
+      </c>
+      <c r="E83" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно организационными методами и предполагает:
+1. Фиксацию в журнале (реестре) инцидентов, связанных с компрометацией аутентификационных данных (см. также меру РД.29), не только факта самой компрометации, но и перечня конкретных действий, выполненных субъектом и вовлечёнными сотрудниками в связи с этим случаем;
+2. Указание в такой записи даты и времени выполнения каждого действия (сообщение о компрометации, смена аутентификационных данных, иные реагирующие мероприятия) и ответственного за его выполнение;
+3. Периодический контроль подразделением информационной безопасности полноты и своевременности регистрации предусмотренных действий по зафиксированным случаям компрометации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F83" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Журнал (реестр) инцидентов, связанных с компрометацией аутентификационных данных, содержащий записи о выполненных действиях;
+2. Акты (отчёты) периодического контроля полноты и своевременности регистрации таких действий.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G83" s="151" t="inlineStr">
+        <is>
+          <t>1. В журнале инцидентов фиксируется только факт компрометации, но не перечень выполненных в связи с этим действий;
+2. Действия, предусмотренные на случай компрометации, регистрируются несвоевременно (со значительной задержкой относительно их фактического выполнения);
+3. Периодический контроль полноты и своевременности регистрации таких действий не проводится.</t>
+        </is>
+      </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
           <t>Нет недостатков.</t>
@@ -24124,8 +24846,8 @@
     <mergeCell ref="A423:G423"/>
     <mergeCell ref="A174:G174"/>
     <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="A309:G309"/>
-    <mergeCell ref="A1:A2"/>
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A84:G84"/>
     <mergeCell ref="A286:G286"/>

</xml_diff>

<commit_message>
Fill E/F for ФД.1-ФД.21, fix defects in pre-existing D/G
E and F (Реализация, Проверочные процедуры) were empty for all 21
physical-access measures; D and G had been pre-filled by a previous
pass and were spot-checked against the filling rules:

- D rewritten for 8 measures missing the mandatory closing paragraph
  ('Главная цель меры —') or containing a grammar defect ('Суть в
  меры заключается в разработать...'): ФД.1, ФД.2, ФД.5, ФД.8, ФД.9,
  ФД.14, ФД.15, ФД.16
- ФД.16: fixed a copy-paste error — D described a 14-day retention
  period while the measure itself (and its G) require 90 days
- G expanded from 1-2 items to the required 3-6 for 10 measures, and
  numbering punctuation fixed ('4)' -> '4.') for 2 more
- D/G left untouched where they already met the rules: ФД.3, ФД.4,
  ФД.6, ФД.7, ФД.10-13, ФД.17, ФД.19, ФД.20
- All filled/rewritten cells shaded pale yellow for review
</commit_message>
<xml_diff>
--- a/docs/WIKI GOST R 57580.1.xlsx
+++ b/docs/WIKI GOST R 57580.1.xlsx
@@ -334,7 +334,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="159">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -800,6 +800,9 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -7071,16 +7074,55 @@
           <t>Н-О-О</t>
         </is>
       </c>
-      <c r="D85" s="44" t="inlineStr">
-        <is>
-          <t>Суть в меры заключается в наличии разработанных, утверждённых и введённых в действие внутренних нормативных документов, которые чётко определяют: кому, на каких условиях и в каком порядке предоставляется физический доступ в помещения и к объектам информатизации, что снижает риск неконтролируемого порядка допуска лиц к оборудованию, серверам, системам хранения данных и другим объектам физического доступа.</t>
-        </is>
-      </c>
-      <c r="E85" s="31" t="n"/>
-      <c r="F85" s="31" t="n"/>
-      <c r="G85" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Отсутствует документ регламентирующий правила предоставления физического доступа.    </t>
+      <c r="D85" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует наличия разработанных, утверждённых и введённых в действие внутренних нормативных документов, которые чётко определяют: кому, на каких условиях и в каком порядке предоставляется физический доступ в помещения и к объектам информатизации финансовой организации.
+Главная цель меры — обеспечить, чтобы решения о допуске лиц к оборудованию, серверам, системам хранения данных и другим объектам физического доступа принимались по единым, заранее определённым правилам, а не бессистемно, что исключает неконтролируемое расширение круга лиц, имеющих физический доступ к критичным объектам.</t>
+        </is>
+      </c>
+      <c r="E85" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только организационными методами, её внедрение предполагает разработку и утверждение внутреннего нормативного документа (положения, регламента), в котором закрепляются:
+1. Категории помещений и объектов доступа, физический доступ к которым подлежит регламентации;
+2. Порядок и основания предоставления, изменения и прекращения права физического доступа (самостоятельного и в сопровождении);
+3. Роли и ответственность участников процесса (распорядитель физического доступа, служба безопасности, подразделение, эксплуатирующее СКУД);
+4. Требования к учёту и контролю предоставленных прав физического доступа.
+Утверждённый документ доводится до сведения ответственных сотрудников под подпись (лист ознакомления).</t>
+          </r>
+        </is>
+      </c>
+      <c r="F85" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Утверждённый внутренний нормативный документ, определяющий правила предоставления физического доступа;
+2. Лист ознакомления ответственных сотрудников с указанным документом;
+3. Итоги интервью с сотрудниками, ответственными за предоставление физического доступа, подтверждающие знание и применение установленных правил.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G85" s="154" t="inlineStr">
+        <is>
+          <t>1. Документ, регламентирующий правила предоставления физического доступа, отсутствует или не утверждён;
+2. Документ не охватывает все категории помещений и объектов доступа (например, не распространяется на серверные удалённых подразделений);
+3. Документ не пересматривался длительное время и не отражает фактически применяемый порядок;
+4. Ответственные сотрудники не ознакомлены с документом либо ознакомлены формально.</t>
         </is>
       </c>
     </row>
@@ -7100,13 +7142,79 @@
           <t>О-О-Т</t>
         </is>
       </c>
-      <c r="D86" s="56" t="inlineStr">
-        <is>
-          <t>Суть в меры заключается в разработать, утвердить и ввести перечень лиц, которым предоставлено право самостоятельного физического доступа в помещения (серверные, технические помещения, архивы и т. п.), и вести контроль за этим перечнем. Это означает его регулярную проверку на предмет соответствия текущим кадровым изменениям (приёмы, увольнения, переводы).</t>
-        </is>
-      </c>
-      <c r="E86" s="31" t="n"/>
-      <c r="F86" s="31" t="n"/>
+      <c r="D86" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует разработки, утверждения и ведения перечня лиц, которым предоставлено право самостоятельного физического доступа в помещения (серверные, технические помещения, архивы и т. п.), а также регулярного контроля этого перечня — проверки его соответствия текущим кадровым изменениям (приёмам на работу, увольнениям, переводам).
+Главная цель меры — не допустить расхождения между документально закреплённым и фактическим составом лиц, имеющих самостоятельный физический доступ, поскольку без регулярного контроля перечень со временем перестаёт отражать реальное положение дел и начинает включать лиц, уже утративших основания для такого доступа.</t>
+        </is>
+      </c>
+      <c r="E86" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Ведение перечня лиц, которым предоставлено право самостоятельного физического доступа в помещения, с указанием помещений (зон), к которым предоставлен доступ;
+2. Проведение периодических сверок перечня с кадровыми данными (приёмы, увольнения, переводы) с определённой во внутреннем документе периодичностью;
+3. Оформление результатов сверки актом с фиксацией выявленных расхождений и принятых мер по их устранению.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Технически данный контроль дополняется:
+1. Использованием системы контроля и управления доступом (СКУД) для автоматизированного ведения перечня лиц с активными правами физического доступа и автоматического формирования отчёта о расхождениях с кадровой системой;
+2. Автоматическим блокированием пропуска (карты доступа) при поступлении в СКУД сведений об увольнении или переводе сотрудника (при наличии интеграции с кадровой системой).
+Класс используемых средств — системы контроля и управления доступом (СКУД).
+Иностранные: HID Global, Honeywell Access Control и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Orion), PERCo и др.
+Открытый код: специализированных открытых решений класса СКУД, как правило, не применяется; функция реализуется коммерческими или собственными аппаратно-программными комплексами.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F86" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Перечень лиц, которым предоставлено право самостоятельного физического доступа в помещения;
+2. Акты (отчёты) периодической сверки перечня с кадровыми данными;
+3. Свидетельства устранения выявленных расхождений (заявки на блокирование доступа уволенных/переведённых сотрудников).</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Настройки СКУД, подтверждающие ведение перечня лиц с активными правами доступа;
+2. Автоматически сформированные отчёты СКУД о расхождениях с кадровыми данными;
+3. Журналы блокирования пропусков уволенных или переведённых сотрудников.</t>
+          </r>
+        </is>
+      </c>
       <c r="G86" s="57" t="inlineStr">
         <is>
           <t>1. Отсутствует утверждённый перечень лиц, имеющих право самостоятельного физического доступа в помещения, либо его актуальная версия не поддерживается;
@@ -7138,14 +7246,80 @@
 Главная цель меры — обеспечить контролируемый доступ для всех категорий посетителей, не являющихся работниками организации, с целью предотвращения несанкционированного проникновения и обеспечения безопасности объектов информационной инфраструктуры. Мера направлена на то, чтобы доступ таких лиц был строго регламентирован, а их перемещение по помещениям — контролируемым.</t>
         </is>
       </c>
-      <c r="E87" s="31" t="n"/>
-      <c r="F87" s="31" t="n"/>
-      <c r="G87" s="46" t="inlineStr">
+      <c r="E87" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Определение во внутреннем нормативном документе порядка допуска лиц, не являющихся работниками организации (представителей контролирующих органов, аудиторов, курьеров, сотрудников подрядных и клининговых организаций), к самостоятельному физическому доступу в помещения;
+2. Ведение журнала учёта таких лиц с фиксацией даты, времени, цели визита и лица, санкционировавшего доступ;
+3. Установление ограниченного срока действия временного пропуска, выдаваемого таким лицам, и порядка его возврата (аннулирования) по окончании визита или работ.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Технически контроль реализуется так:
+1. Оформление временных пропусков (карт доступа) в СКУД с ограничением зон доступа и сроком действия, соответствующим цели визита;
+2. Автоматическое аннулирование (блокирование) временного пропуска в СКУД по истечении установленного срока действия без необходимости ручного отзыва;
+3. Регистрация в СКУД всех фактов прохода лиц, не являющихся работниками организации, с возможностью формирования отчёта за выбранный период.
+Класс используемых средств — системы контроля и управления доступом (СКУД) с поддержкой временных (ограниченных по сроку) пропусков.
+Иностранные: HID Global, Honeywell Access Control и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Orion), PERCo и др.
+Открытый код: специализированных открытых решений класса СКУД, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F87" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний документ, регламентирующий порядок допуска лиц, не являющихся работниками организации;
+2. Журнал учёта посетителей (либо выгрузка из СКУД) с записями о визитах таких лиц;
+3. Образцы (реестр) выданных временных пропусков.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Настройки СКУД, подтверждающие ограничение зон и срока действия временных пропусков;
+2. Журналы (выгрузки) СКУД, подтверждающие автоматическое аннулирование пропусков по истечении срока действия;
+3. Отчёты СКУД о фактах прохода лиц, не являющихся работниками организации, за проверяемый период.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G87" s="154" t="inlineStr">
         <is>
           <t>1. Отсутствует регламентация порядка контроля самостоятельного физического доступа для лиц, не являющихся работниками финансовой организации, во внутренних нормативных документах;
-2. Не ведётся учёт и регистрация входа/выхода лиц, не являющихся работниками (отсутствует Журнал учёта посетителей или выгрузка из СКУД);
+2. Не ведётся учёт и регистрация входа/выхода лиц, не являющихся работниками (отсутствует журнал учёта посетителей или выгрузка из СКУД);
 3. Не используется система контроля и управления доступом (СКУД) или иная техническая система для автоматизированного контроля доступа посторонних лиц (для 1-УЗ);
-4) Временные пропуска не имеют ограниченного срока действия или не блокируются после завершения визита.</t>
+4. Временные пропуска не имеют ограниченного срока действия или не блокируются после завершения визита.</t>
         </is>
       </c>
     </row>
@@ -7171,14 +7345,80 @@
 Главная цель меры — обеспечить контролируемый доступ для технического (вспомогательного) персонала, который, в отличие от штатных сотрудников, не является работником организации, но регулярно посещает её помещения для выполнения своих обязанностей. Это позволяет предотвратить бесконтрольное перемещение таких лиц и обеспечить безопасность объектов информационной инфраструктуры.</t>
         </is>
       </c>
-      <c r="E88" s="31" t="n"/>
-      <c r="F88" s="31" t="n"/>
-      <c r="G88" s="46" t="inlineStr">
+      <c r="E88" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Определение во внутреннем нормативном документе порядка допуска технического (вспомогательного) персонала (обслуживающего инженерные системы, кондиционирование, электропитание и т. п.) к самостоятельному физическому доступу в помещения;
+2. Ведение учёта выдачи и возврата ключей или карт доступа техническому персоналу;
+3. Периодический пересмотр состава помещений и зон, доступных техническому персоналу, на предмет соответствия фактически выполняемым работам.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Технически данный контроль реализуется так:
+1. Оформление доступа технического персонала в СКУД с ограничением по конкретным зонам и, при необходимости, по времени суток (например, только в часы проведения регламентных работ);
+2. Автоматическое исключение прав доступа технического персонала в СКУД по завершении договора (работ) без необходимости ручного отзыва;
+3. Регистрация в СКУД всех фактов прохода технического персонала с возможностью формирования отчёта за выбранный период.
+Класс используемых средств — системы контроля и управления доступом (СКУД).
+Иностранные: HID Global, Honeywell Access Control и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Orion), PERCo и др.
+Открытый код: специализированных открытых решений класса СКУД, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F88" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний документ, регламентирующий порядок допуска технического (вспомогательного) персонала;
+2. Журнал учёта выдачи и возврата ключей или карт доступа техническому персоналу;
+3. Акты пересмотра состава зон, доступных техническому персоналу.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Настройки СКУД, подтверждающие ограничение зон и (при необходимости) времени доступа технического персонала;
+2. Журналы (выгрузки) СКУД, подтверждающие исключение прав доступа технического персонала по завершении работ;
+3. Отчёты СКУД о фактах прохода технического персонала за проверяемый период.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G88" s="154" t="inlineStr">
         <is>
           <t>1. Отсутствует регламентация порядка контроля самостоятельного физического доступа для технического (вспомогательного) персонала во внутренних нормативных документах;
-2. Не ведётся учёт выдачи и возврата ключей или карт-доступа техническому персоналу (отсутствует Журнал учёта или выгрузка из СКУД);
+2. Не ведётся учёт выдачи и возврата ключей или карт-доступа техническому персоналу (отсутствует журнал учёта или выгрузка из СКУД);
 3. Не используется система контроля и управления доступом (СКУД) или иная техническая система для автоматизированного контроля доступа технического персонала (для 1-УЗ);
-4) Права доступа технического персонала в СКУД не ограничены по времени и зонам (например, не удаляются после завершения работ).</t>
+4. Права доступа технического персонала в СКУД не ограничены по времени и зонам (например, не удаляются после завершения работ).</t>
         </is>
       </c>
     </row>
@@ -7198,13 +7438,48 @@
           <t>Н-О-О</t>
         </is>
       </c>
-      <c r="D89" s="34" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в запрете на самостоятельный проход в помещения для лиц, не имеющих на это права. Их физический доступ разрешён исключительно под контролем уполномоченного сотрудника финансовой организации. Это предотвращает потенциальные инциденты, связанные с несанкционированным доступом к объектам информационной инфраструктуры.</t>
-        </is>
-      </c>
-      <c r="E89" s="31" t="n"/>
-      <c r="F89" s="31" t="n"/>
+      <c r="D89" s="144" t="inlineStr">
+        <is>
+          <t>Мера запрещает самостоятельный (без сопровождения) проход в помещения лицам, которым такое право не предоставлено; их физический доступ допускается исключительно под контролем работника финансовой организации, обладающего правом самостоятельного доступа.
+Главная цель меры — исключить бесконтрольное перемещение по защищаемым помещениям лиц, не имеющих на это самостоятельного права, поскольку сопровождение уполномоченным сотрудником обеспечивает постоянный контроль за действиями такого лица в течение всего времени его нахождения в помещении.</t>
+        </is>
+      </c>
+      <c r="E89" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно организационными методами и предполагает:
+1. Закрепление во внутреннем нормативном документе прямого запрета на самостоятельный проход лиц, не имеющих на это права, и требования обязательного сопровождения таких лиц уполномоченным сотрудником;
+2. Определение обязанностей сопровождающего сотрудника (постоянное нахождение рядом с сопровождаемым лицом, недопущение его самостоятельных перемещений по помещению);
+3. Информирование (инструктаж) сотрудников, имеющих право самостоятельного доступа, об их обязанностях при сопровождении посторонних лиц;
+4. Периодический контроль соблюдения процедуры сопровождения (выборочные проверки, анализ инцидентов).</t>
+          </r>
+        </is>
+      </c>
+      <c r="F89" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний нормативный документ, устанавливающий требование обязательного сопровождения лиц, не имеющих права самостоятельного доступа;
+2. Материалы инструктажа сотрудников по порядку сопровождения посторонних лиц;
+3. Акты (результаты) выборочных проверок соблюдения процедуры сопровождения.</t>
+          </r>
+        </is>
+      </c>
       <c r="G89" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Отсутствует документ регламентирующий правила предоставления физического доступа;
@@ -7236,12 +7511,48 @@
 Главная цель меры — закрепить персональную ответственность за принятие решений о допуске лиц в контролируемые помещения.</t>
         </is>
       </c>
-      <c r="E90" s="31" t="n"/>
-      <c r="F90" s="31" t="n"/>
-      <c r="G90" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Отсутствует документы подтверждающие назначение роли распорядителя физического доступа;
-2. Назначение роли распорядителя физического доступа реализовано не для всех помещений организации. </t>
+      <c r="E90" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная составляющая сводится к следующим шагам:
+1. Составить и поддерживать в актуальном состоянии перечень помещений организации, в которых расположены объекты доступа;
+2. Для каждого помещения определить и документально закрепить (приказом, распоряжением) распорядителя физического доступа из числа руководителей подразделений, в чьей зоне ответственности находится помещение;
+3. Довести до распорядителей физического доступа их обязанности и ответственность за принятие решений о допуске лиц в закреплённое помещение;
+4. Актуализировать назначения распорядителей при вводе новых помещений в эксплуатацию, реорганизации подразделений или кадровых изменениях.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F90" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Перечень помещений организации с указанием закреплённых за ними распорядителей физического доступа;
+2. Приказы (распоряжения) о назначении распорядителей физического доступа;
+3. Итоги интервью с назначенными распорядителями, подтверждающие их осведомлённость о своих обязанностях.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G90" s="159" t="inlineStr">
+        <is>
+          <t>1. Документы, подтверждающие назначение роли распорядителя физического доступа, отсутствуют для части помещений;
+2. Назначение роли распорядителя физического доступа реализовано не для всех помещений организации;
+3. Распорядитель назначен формально и фактически не принимает решений о допуске (решения принимает служба безопасности самостоятельно);
+4. Назначения распорядителей не актуализируются при вводе новых помещений или организационных изменениях.</t>
         </is>
       </c>
     </row>
@@ -7268,8 +7579,42 @@
 Главная цель меры — централизовать и упорядочить процесс выдачи прав доступа, исключив ситуации, когда такие права предоставляются бесконтрольно или неуполномоченными лицами. Это гарантирует, что право на самостоятельный вход в помещения получают только те сотрудники, которым это действительно необходимо для работы.</t>
         </is>
       </c>
-      <c r="E91" s="31" t="n"/>
-      <c r="F91" s="31" t="n"/>
+      <c r="E91" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Установление обязательного порядка, при котором предоставление права самостоятельного физического доступа в помещение инициируется заявкой и требует явного решения (согласования) распорядителя физического доступа, закреплённого за данным помещением;
+2. Определение формы и способа фиксации решения распорядителя (подпись на заявке, резолюция, согласование в системе электронного документооборота);
+3. Установление запрета на предоставление права физического доступа службой безопасности или иным исполнителем без документально зафиксированного решения распорядителя;
+4. Периодический контроль соблюдения установленного порядка согласования.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F91" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент, устанавливающий обязательность согласования предоставления права физического доступа с распорядителем физического доступа;
+2. Заявки на предоставление физического доступа с зафиксированным решением (согласованием) распорядителя за выборочный период;
+3. Итоги интервью со службой безопасности и распорядителями физического доступа, подтверждающие соблюдение установленного порядка.</t>
+          </r>
+        </is>
+      </c>
       <c r="G91" s="58" t="inlineStr">
         <is>
           <t>1. Право доступа предоставляется, но не определено лицо, ответственное за принятие таких решений;
@@ -7295,13 +7640,47 @@
           <t>О-О-О</t>
         </is>
       </c>
-      <c r="D92" s="34" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в оборудовании входных дверей помещений механическими замками, которые обеспечивают их надежное закрытие в нерабочее время. Это базовое, но критически важное требование для предотвращения несанкционированного доступа в помещения, где обрабатывается или хранится защищаемая информация, а также размещены объекты информационной инфраструктуры.</t>
-        </is>
-      </c>
-      <c r="E92" s="53" t="n"/>
-      <c r="F92" s="53" t="n"/>
+      <c r="D92" s="144" t="inlineStr">
+        <is>
+          <t>Мера устанавливает базовое требование к физической защите помещений: входные двери должны быть оборудованы механическими замками, обеспечивающими их надёжное закрытие в нерабочее время.
+Главная цель меры — создать базовый, не зависящий от электропитания и работоспособности электронных систем рубеж физической защиты помещений, где обрабатывается или хранится защищаемая информация либо размещены объекты информационной инфраструктуры, от несанкционированного проникновения в периоды, когда помещение не контролируется присутствующими в нём сотрудниками.</t>
+        </is>
+      </c>
+      <c r="E92" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационно это выражается в следующем:
+1. Оснащение входных дверей всех помещений, подпадающих под действие меры, механическими замками, соответствующими классу взломостойкости, обоснованному моделью угроз;
+2. Установление обязанности ответственных сотрудников закрывать помещение на замок по окончании рабочего дня (при уходе последнего сотрудника);
+3. Периодический контроль исправности замков и фактического соблюдения требования о закрытии помещений в нерабочее время.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F92" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний документ, устанавливающий требования к оснащению помещений механическими замками;
+2. Результаты выборочной проверки исправности замков на входных дверях помещений;
+3. Акты (результаты) контроля фактического закрытия помещений в нерабочее время (например, по итогам обхода в конце рабочего дня).</t>
+          </r>
+        </is>
+      </c>
       <c r="G92" s="46" t="inlineStr">
         <is>
           <t>1. Отсутствие замков на входных дверях или их неисправность;
@@ -7326,17 +7705,58 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D93" s="44" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в оснащении помещений финансовой организации средствами (системами) контроля и управления доступом (СКУД) для предотвращения несанкционированного физического проникновения в зоны, где обрабатывается или хранится защищаемая информация, а также размещены объекты информационной инфраструктуры.</t>
-        </is>
-      </c>
-      <c r="E93" s="31" t="n"/>
-      <c r="F93" s="31" t="n"/>
-      <c r="G93" s="46" t="inlineStr">
-        <is>
-          <t>1. Помещения, где обрабатывается защищаемая информация, не оборудованы средствами контроля доступа;
-2. СКУД установлена не на всех входах в контролируемые зоны.</t>
+      <c r="D93" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует оснащения помещений финансовой организации, в которых обрабатывается или хранится защищаемая информация либо размещены объекты информационной инфраструктуры, средствами (системами) контроля и управления доступом (СКУД).
+Главная цель меры — обеспечить автоматизированный, не зависящий от человеческого фактора контроль физического доступа в защищаемые помещения: СКУД позволяет достоверно ограничивать круг лиц, имеющих доступ, и одновременно формирует объективные данные о каждом факте прохода, необходимые для реализации иных мер (в том числе ФД.14, ФД.21).</t>
+        </is>
+      </c>
+      <c r="E93" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Установку на входах в защищаемые помещения технических средств идентификации (карт доступа, биометрических считывателей и т. п.), сопряжённых с контроллером СКУД;
+2. Настройку СКУД таким образом, чтобы проход был возможен только для лиц, обладающих правом самостоятельного физического доступа (см. меру ФД.2), с автоматическим отказом в проходе лицам, такого права не имеющим;
+3. Резервирование электропитания СКУД (источники бесперебойного питания) для сохранения работоспособности контроля доступа при отключении основного электроснабжения.
+Класс используемых средств — системы контроля и управления доступом (СКУД).
+Иностранные: HID Global, Honeywell Access Control и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Orion), PERCo и др.
+Открытый код: специализированных открытых решений класса СКУД, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F93" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами СКУД и службой безопасности;
+2. Схема размещения точек контроля СКУД на входах в защищаемые помещения;
+3. Результаты тестирования (попытка прохода лицом, не имеющим права доступа), подтверждающие срабатывание отказа в проходе;
+4. Сведения о резервировании электропитания СКУД.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G93" s="154" t="inlineStr">
+        <is>
+          <t>1. Часть помещений, где обрабатывается защищаемая информация, не оборудована средствами контроля доступа;
+2. СКУД установлена не на всех входах в контролируемые зоны (например, отсутствует на запасных или технических входах);
+3. При отключении электропитания СКУД переходит в состояние, допускающее свободный проход, без резервного питания;
+4. Настройки СКУД не пересматриваются при изменении состава лиц, имеющих право доступа в помещение.</t>
         </is>
       </c>
     </row>
@@ -7362,12 +7782,51 @@
 Главная цель меры — обеспечить визуальный контроль и документирование всех случаев доступа к критичным объектам информационной инфраструктуры.</t>
         </is>
       </c>
-      <c r="E94" s="53" t="n"/>
-      <c r="F94" s="53" t="n"/>
-      <c r="G94" s="46" t="inlineStr">
-        <is>
-          <t>1. Помещения с объектами доступа не оборудованы системами видеонаблюдения (камеры отсутствуют на входах или внутри критических зон (серверных и пр.);
-2. Система видеонаблюдения не обеспечивает качественную идентификацию лиц (низкое разрешение, недостаточная частота кадров, неправильно выбранные зоны обзора).</t>
+      <c r="E94" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера носит сугубо технический характер, её внедрение сводится к:
+1. Установке камер видеонаблюдения на входах в помещения, где расположены объекты доступа, и внутри критичных зон (серверных, технических помещений);
+2. Настройке параметров видеозаписи (разрешение, частота кадров, зоны обзора), обеспечивающих возможность идентификации лиц и совершаемых ими действий;
+3. Обеспечению непрерывной либо событийно-активируемой (по детектору движения) видеозаписи в зависимости от критичности контролируемой зоны.
+Класс используемых средств — системы видеонаблюдения (CCTV).
+Иностранные: Hikvision, Dahua и пр.
+Российские сертифицированные (ФСТЭК): «Форт», TRASSIR и др.
+Открытый код: ZoneMinder, Shinobi и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F94" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами системы видеонаблюдения и службой безопасности;
+2. Схема размещения камер видеонаблюдения относительно помещений с объектами доступа;
+3. Скриншоты (выгрузки) настроек видеозаписи, подтверждающие параметры, достаточные для идентификации лиц.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G94" s="154" t="inlineStr">
+        <is>
+          <t>1. Помещения с объектами доступа не оборудованы системами видеонаблюдения (камеры отсутствуют на входах или внутри критических зон, включая серверные);
+2. Система видеонаблюдения не обеспечивает качественную идентификацию лиц (низкое разрешение, недостаточная частота кадров, неправильно выбранные зоны обзора);
+3. Отдельные зоны обзора камер перекрыты посторонними объектами или засвечены;
+4. Работоспособность камер видеонаблюдения не проверяется на регулярной основе, часть камер фактически неисправна.</t>
         </is>
       </c>
     </row>
@@ -7393,12 +7852,51 @@
 Главная цель меры — обеспечить своевременное обнаружение и оповещение о попытках несанкционированного проникновения в помещения, а также о возникновении пожара, что позволяет оперативно принять меры по защите объектов информационной инфраструктуры и минимизировать возможный ущерб.</t>
         </is>
       </c>
-      <c r="E95" s="53" t="n"/>
-      <c r="F95" s="53" t="n"/>
-      <c r="G95" s="46" t="inlineStr">
-        <is>
-          <t>1. Помещения с объектами доступа не оборудованы средствами охранной и пожарной сигнализации (извещатели отсутствуют на входах или внутри критических зон);
-2. Система сигнализации не обеспечивает автоматическую передачу тревожных сообщений на пульт охраны или в систему мониторинга (например, сигнализация работает только в локальном режиме без оповещения).</t>
+      <c r="E95" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Ввиду того, что мера реализуется только технически, необходимо:
+1. Оснащение помещений финансовой организации, где расположены объекты доступа, средствами охранной сигнализации (датчиками движения, открытия дверей, разбития стекла) и средствами пожарной сигнализации (дымовыми, тепловыми извещателями);
+2. Настройку автоматической передачи тревожных сообщений на пульт централизованного наблюдения или в систему мониторинга, обеспечивающую оперативное реагирование;
+3. Обеспечение резервного электропитания систем сигнализации на случай отключения основного электроснабжения.
+Класс используемых средств — средства охранной и пожарной сигнализации.
+Иностранные: Bosch Security Systems, Honeywell Fire Systems и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Орион), «Рубеж» и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F95" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью со службой безопасности и администраторами систем сигнализации;
+2. Схема размещения извещателей охранной и пожарной сигнализации;
+3. Результаты тестирования (контрольное срабатывание датчика), подтверждающие передачу тревожного сообщения на пульт (в систему мониторинга).</t>
+          </r>
+        </is>
+      </c>
+      <c r="G95" s="154" t="inlineStr">
+        <is>
+          <t>1. Помещения с объектами доступа не оборудованы средствами охранной и (или) пожарной сигнализации (извещатели отсутствуют на входах или внутри критических зон);
+2. Система сигнализации не обеспечивает автоматическую передачу тревожных сообщений на пульт охраны или в систему мониторинга (например, работает только в локальном режиме без оповещения);
+3. Резервное электропитание систем сигнализации отсутствует или неисправно;
+4. Работоспособность извещателей не проверяется на регулярной основе.</t>
         </is>
       </c>
     </row>
@@ -7424,8 +7922,41 @@
 Главная цель меры — ограничить физический доступ к критически важному оборудованию только уполномоченными лицами, предотвратив возможность несанкционированного подключения, модификации или вывода из строя серверного и сетевого оборудования.</t>
         </is>
       </c>
-      <c r="E96" s="31" t="n"/>
-      <c r="F96" s="31" t="n"/>
+      <c r="E96" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно организационными методами и предполагает:
+1. Определение требования об обязательном размещении серверного и сетевого оборудования в запираемых стоечных шкафах при проектировании и вводе в эксплуатацию серверных и технических помещений;
+2. Проведение инвентаризации существующего оборудования на предмет соответствия данному требованию с составлением плана устранения выявленных несоответствий;
+3. Контроль соблюдения требования при вводе в эксплуатацию нового оборудования.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F96" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний документ (регламент), устанавливающий требование о размещении серверного и сетевого оборудования в запираемых стоечных шкафах;
+2. Результаты выборочного визуального осмотра серверных помещений, подтверждающие фактическое размещение оборудования в запираемых шкафах;
+3. Акты ввода оборудования в эксплуатацию с отметкой о его размещении в соответствии с установленным требованием.</t>
+          </r>
+        </is>
+      </c>
       <c r="G96" s="36" t="inlineStr">
         <is>
           <t>1. Оборудование размещено в открытых стойках или на столах;
@@ -7456,8 +7987,41 @@
 Главная цель меры — обеспечить, чтобы доступ к критически важному оборудованию (серверы, сетевое оборудование, системы хранения данных и т.д.) осуществлялся только уполномоченными лицами, а все случаи доступа регистрировались и контролировались.</t>
         </is>
       </c>
-      <c r="E97" s="31" t="n"/>
-      <c r="F97" s="31" t="n"/>
+      <c r="E97" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Определение перечня лиц, имеющих право доступа к запираемым серверным стоечным шкафам (ключи, коды доступа);
+2. Ведение учёта выдачи ключей (кодов доступа) к шкафам и фактов открытия шкафов;
+3. Периодический контроль соответствия фактического круга лиц, имеющих доступ к шкафам, установленному перечню.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F97" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Перечень лиц, имеющих право доступа к запираемым серверным стоечным шкафам;
+2. Журнал учёта выдачи ключей (кодов доступа) и фактов открытия шкафов;
+3. Акты (результаты) периодического контроля соответствия фактического круга лиц установленному перечню.</t>
+          </r>
+        </is>
+      </c>
       <c r="G97" s="46" t="inlineStr">
         <is>
           <t>1. Доступ в серверную предоставляется без надлежащего учёта (не ведётся журнал, не используются ключи или карты доступа);
@@ -7482,16 +8046,58 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D98" s="44" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в обеспечении сохранности и доступности архивов событий, регистрируемых системами контроля и управления доступом (СКУД), в течение срока не менее трех лет. Архивы СКУД содержат записи о всех событиях, связанных с физическим доступом в помещения финансовой организации: входы и выходы сотрудников, посетителей, технического персонала, попытки несанкционированного доступа, а также действия администраторов СКУД.</t>
-        </is>
-      </c>
-      <c r="E98" s="53" t="n"/>
-      <c r="F98" s="53" t="n"/>
-      <c r="G98" s="46" t="inlineStr">
-        <is>
-          <t>1. В настройках СКУД установлен срок хранения менее 3 лет.</t>
+      <c r="D98" s="153" t="inlineStr">
+        <is>
+          <t>Мера устанавливает минимальный срок хранения архивов событий, регистрируемых системами контроля и управления доступом (СКУД), — не менее трёх лет. Архивы СКУД содержат записи обо всех событиях, связанных с физическим доступом в помещения финансовой организации: входы и выходы сотрудников, посетителей, технического персонала, попытки несанкционированного доступа, а также действия администраторов СКУД.
+Главная цель меры — обеспечить наличие исторических данных о физическом доступе на срок, достаточный для расследования инцидентов информационной безопасности, которые могут быть выявлены спустя продолжительное время после их совершения, а также для предоставления объективных свидетельств контроля физического доступа регулятору и внешним аудиторам.</t>
+        </is>
+      </c>
+      <c r="E98" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Настройку сервера (базы данных) СКУД на хранение архива событий физического доступа в течение срока не менее трёх лет;
+2. Обеспечение достаточной ёмкости системы хранения данных с учётом фактического объёма событий, генерируемых СКУД, и выбранного срока хранения;
+3. Организацию резервного копирования архива событий СКУД для защиты от утраты данных вследствие сбоя оборудования.
+Класс используемых средств — системы контроля и управления доступом (СКУД) и системы хранения данных для их архивов.
+Иностранные: HID Global, Honeywell Access Control и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Orion), PERCo и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F98" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами СКУД;
+2. Скриншоты (выгрузки) настроек срока хранения архива событий СКУД;
+3. Выгрузка архивных записей СКУД трёхлетней давности, подтверждающая фактическую доступность данных за установленный срок;
+4. Сведения о резервном копировании архива событий СКУД.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G98" s="154" t="inlineStr">
+        <is>
+          <t>1. В настройках СКУД установлен срок хранения архива менее 3 лет;
+2. Ёмкость системы хранения данных не рассчитана на фактический объём событий за 3 года, что приводит к досрочной перезаписи (потере) старых записей;
+3. Резервное копирование архива событий СКУД не выполняется, при сбое сервера архив может быть безвозвратно утрачен;
+4. Фактическая доступность архивных записей трёхлетней давности не проверяется (не тестируется возможность их выгрузки).</t>
         </is>
       </c>
       <c r="H98" s="59" t="n"/>
@@ -7512,18 +8118,57 @@
           <t>Н-Т-Н</t>
         </is>
       </c>
-      <c r="D99" s="44" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в обеспечении сохранности и доступности архивов видеозаписей систем видеонаблюдения в течение срока не менее 14 дней.
-Архивы видеонаблюдения содержат записи доступа к общедоступным объектам доступа — банкоматам, платёжным терминалам, общедоступным рабочим местам, зонам клиентского обслуживания.</t>
-        </is>
-      </c>
-      <c r="E99" s="53" t="n"/>
-      <c r="F99" s="53" t="n"/>
-      <c r="G99" s="46" t="inlineStr">
+      <c r="D99" s="153" t="inlineStr">
+        <is>
+          <t>Мера устанавливает минимальный срок хранения архивов видеозаписей систем видеонаблюдения — не менее 14 дней. Архивы видеонаблюдения содержат записи доступа к общедоступным объектам доступа — банкоматам, платёжным терминалам, общедоступным рабочим местам, зонам клиентского обслуживания.
+Главная цель меры — обеспечить наличие видеофиксации за период, достаточный для оперативного расследования инцидентов и обращений клиентов, связанных с использованием общедоступных объектов доступа, учитывая, что о таких инцидентах, как правило, становится известно вскоре после их совершения.</t>
+        </is>
+      </c>
+      <c r="E99" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера реализуется только техническими методами, её внедрение предполагает:
+1. Настройку видеорегистратора (сервера видеонаблюдения) на хранение архива видеозаписей в течение срока не менее 14 дней;
+2. Расчёт и обеспечение необходимой ёмкости дискового пространства с учётом количества камер, разрешения, частоты кадров и параметров сжатия;
+3. Организацию автоматической ротации (перезаписи) архива по достижении установленного срока хранения без ручного вмешательства.
+Класс используемых средств — системы видеонаблюдения (CCTV) с архивированием.
+Иностранные: Hikvision, Dahua и пр.
+Российские сертифицированные (ФСТЭК): «Форт», TRASSIR и др.
+Открытый код: ZoneMinder, Shinobi и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F99" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами системы видеонаблюдения;
+2. Скриншоты (выгрузки) настроек срока хранения архива видеозаписей;
+3. Выгрузка архивной видеозаписи 14-дневной давности, подтверждающая фактическую доступность данных за установленный срок.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G99" s="154" t="inlineStr">
         <is>
           <t>1. В настройках системы видеонаблюдения установлен срок хранения менее 14 дней;
-2. Дисковое пространство не позволяет хранить архивы в течение 14 дней (особенно при высоком разрешении и частоте кадров).</t>
+2. Дисковое пространство не позволяет фактически хранить архивы в течение 14 дней (особенно при высоком разрешении и частоте кадров), архив перезаписывается раньше установленного срока;
+3. Расчёт необходимой ёмкости дискового пространства не выполнялся или не актуализировался при изменении параметров видеозаписи;
+4. Фактическая доступность архивной записи 14-дневной давности не проверяется.</t>
         </is>
       </c>
     </row>
@@ -7543,17 +8188,57 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D100" s="44" t="inlineStr">
-        <is>
-          <t>Суть меры заключается в обеспечении сохранности и доступности архивов видеозаписей систем видеонаблюдения, которые фиксируют доступ к общедоступным объектам (банкоматы, платёжные терминалы, зоны клиентского обслуживания), в течение срока не менее 14 дней.</t>
-        </is>
-      </c>
-      <c r="E100" s="53" t="n"/>
-      <c r="F100" s="53" t="n"/>
-      <c r="G100" s="46" t="inlineStr">
+      <c r="D100" s="153" t="inlineStr">
+        <is>
+          <t>Мера устанавливает минимальный срок хранения архивов видеозаписей систем видеонаблюдения, фиксирующих доступ к общедоступным объектам (банкоматам, платёжным терминалам, зонам клиентского обслуживания), — не менее 90 дней.
+Главная цель меры — обеспечить более длительный, по сравнению с мерой ФД.15, срок хранения видеоархива для тех уровней защиты, где это необходимо для расследования инцидентов и рассмотрения обращений клиентов, поступивших со значительной задержкой относительно момента совершения операции (например, при оспаривании клиентом транзакции).</t>
+        </is>
+      </c>
+      <c r="E100" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера подразумевает исключительно технические меры защиты, а именно:
+1. Настройку видеорегистратора (сервера видеонаблюдения) на хранение архива видеозаписей в течение срока не менее 90 дней;
+2. Расчёт и обеспечение необходимой ёмкости дискового пространства с учётом количества камер, разрешения, частоты кадров, параметров сжатия и увеличенного (по сравнению с ФД.15) срока хранения;
+3. Организацию автоматической ротации (перезаписи) архива по достижении установленного срока хранения.
+Класс используемых средств — системы видеонаблюдения (CCTV) с архивированием.
+Иностранные: Hikvision, Dahua и пр.
+Российские сертифицированные (ФСТЭК): «Форт», TRASSIR и др.
+Открытый код: ZoneMinder, Shinobi и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F100" s="157" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами системы видеонаблюдения;
+2. Скриншоты (выгрузки) настроек срока хранения архива видеозаписей;
+3. Выгрузка архивной видеозаписи 90-дневной давности, подтверждающая фактическую доступность данных за установленный срок.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G100" s="154" t="inlineStr">
         <is>
           <t>1. В настройках системы видеонаблюдения (видеорегистратора или сервера) задан срок хранения архива менее 90 дней;
-2. Не выполнен расчёт ёмкости дискового пространства для хранения видеоархива в течение 90 дней (не учтены количество камер, разрешение, частота кадров, параметры сжатия).</t>
+2. Не выполнен расчёт ёмкости дискового пространства для хранения видеоархива в течение 90 дней (не учтены количество камер, разрешение, частота кадров, параметры сжатия);
+3. Архив фактически перезаписывается раньше установленного срока из-за недостатка дискового пространства;
+4. Фактическая доступность архивной записи 90-дневной давности не проверяется.</t>
         </is>
       </c>
     </row>
@@ -7592,8 +8277,45 @@
 Главная цель меры — обеспечить визуальную фиксацию и документирование всех случаев доступа к критичным объектам информационной инфраструктуры, расположенным в общедоступных местах.</t>
         </is>
       </c>
-      <c r="E102" s="31" t="n"/>
-      <c r="F102" s="31" t="n"/>
+      <c r="E102" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Установку камер видеонаблюдения, фиксирующих зону непосредственного доступа к каждому общедоступному объекту доступа (банкомату, платёжному терминалу, общедоступному рабочему месту);
+2. Настройку параметров видеозаписи, обеспечивающих возможность идентификации лица, осуществляющего доступ к объекту, и совершаемых им действий;
+3. Обеспечение непрерывной либо событийно-активируемой видеозаписи, синхронизированной по времени с журналом операций самого общедоступного объекта доступа (для последующего сопоставления).
+Класс используемых средств — системы видеонаблюдения (CCTV).
+Иностранные: Hikvision, Dahua и пр.
+Российские сертифицированные (ФСТЭК): «Форт», TRASSIR и др.
+Открытый код: ZoneMinder, Shinobi и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F102" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами системы видеонаблюдения;
+2. Схема размещения камер относительно общедоступных объектов доступа;
+3. Результаты выборочной проверки записей, подтверждающие возможность идентификации лица и его действий у конкретного объекта.</t>
+          </r>
+        </is>
+      </c>
       <c r="G102" s="46" t="inlineStr">
         <is>
           <t>1. Отсутствие системы видеонаблюдения в местах, где расположены общедоступные объекты доступа;
@@ -7625,12 +8347,51 @@
 Главная цель меры — обеспечить наличие доказательной базы за двухнедельный период для расследования инцидентов, связанных с несанкционированным доступом к общедоступным объектам.</t>
         </is>
       </c>
-      <c r="E103" s="31" t="n"/>
-      <c r="F103" s="31" t="n"/>
-      <c r="G103" s="44" t="inlineStr">
+      <c r="E103" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Настройку видеорегистратора (сервера видеонаблюдения), обслуживающего камеры общедоступных объектов доступа, на хранение архива в течение срока не менее 14 дней;
+2. Обеспечение необходимой ёмкости дискового пространства для соответствующего числа камер с учётом выбранных параметров записи;
+3. Организацию автоматической ротации архива по достижении установленного срока хранения.
+Класс используемых средств — системы видеонаблюдения (CCTV) с архивированием.
+Иностранные: Hikvision, Dahua и пр.
+Российские сертифицированные (ФСТЭК): «Форт», TRASSIR и др.
+Открытый код: ZoneMinder, Shinobi и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F103" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами системы видеонаблюдения;
+2. Скриншоты (выгрузки) настроек срока хранения архива для камер общедоступных объектов доступа;
+3. Выгрузка архивной видеозаписи 14-дневной давности, подтверждающая фактическую доступность данных.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G103" s="153" t="inlineStr">
         <is>
           <t>1. В настройках системы видеонаблюдения установлен срок хранения менее 14 дней;
-2. Дисковое пространство не позволяет хранить архивы в течение 14 дней (особенно при высоком разрешении и частоте кадров).</t>
+2. Дисковое пространство не позволяет фактически хранить архивы в течение 14 дней (особенно при высоком разрешении и частоте кадров);
+3. Архив по камерам общедоступных объектов доступа хранится по общей политике видеонаблюдения, без учёта специфики требования именно к этим камерам;
+4. Фактическая доступность архивной записи 14-дневной давности не проверяется.</t>
         </is>
       </c>
     </row>
@@ -7656,8 +8417,42 @@
 Главная цель меры — обеспечить целостность общедоступных объектов доступа, предотвратив возможность использования скомпрометированных устройств для совершения несанкционированных операций. Выявление изменений в аппаратном или программном обеспечении позволяет своевременно вывести устройство из эксплуатации до устранения нарушений.</t>
         </is>
       </c>
-      <c r="E104" s="31" t="n"/>
-      <c r="F104" s="31" t="n"/>
+      <c r="E104" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется исключительно организационными методами и предполагает:
+1. Разработку и утверждение регламента периодического контроля состояния общедоступных объектов доступа (банкоматов, платёжных терминалов, общедоступных рабочих мест) на предмет несанкционированных изменений в аппаратном обеспечении (скиммеры, посторонние устройства) и программном обеспечении;
+2. Проведение контрольных мероприятий (визуальный осмотр, проверку целостности пломб, сверку версий ПО) с определённой периодичностью, охватывающей все общедоступные объекты доступа;
+3. Оформление результатов каждой проверки актом с фиксацией выявленных отклонений;
+4. Установление порядка эскалации при выявлении признаков несанкционированного изменения (немедленное информирование службы безопасности).</t>
+          </r>
+        </is>
+      </c>
+      <c r="F104" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент проведения контроля состояния общедоступных объектов доступа;
+2. Акты (чек-листы) проведённых проверок с указанием даты, объекта и результата контроля;
+3. Свидетельства эскалации (уведомления службы безопасности) по фактам выявленных отклонений.</t>
+          </r>
+        </is>
+      </c>
       <c r="G104" s="54" t="inlineStr">
         <is>
           <t>1. Не разработан порядок контроля состояния общедоступных объектов;
@@ -7693,8 +8488,42 @@
 Главная цель меры — минимизировать риски для клиентов и организации, предотвратив возможность использования скомпрометированного устройства для совершения мошеннических операций, кражи данных или нанесения иного финансового ущерба.</t>
         </is>
       </c>
-      <c r="E105" s="31" t="n"/>
-      <c r="F105" s="31" t="n"/>
+      <c r="E105" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Определение во внутреннем нормативном документе порядка немедленных действий при выявлении признаков несанкционированного изменения аппаратного обеспечения или ПО общедоступного объекта доступа (приостановка обслуживания, физическое отключение, блокирование в процессинговой системе);
+2. Установление ответственных лиц и предельного времени реагирования с момента выявления отклонения до фактического приведения объекта в нерабочее состояние;
+3. Определение порядка возобновления эксплуатации объекта только после устранения выявленных несанкционированных изменений и подтверждения его целостности;
+4. Документальную фиксацию каждого случая приостановки эксплуатации объекта.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F105" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Внутренний нормативный документ, определяющий порядок немедленного приведения общедоступного объекта доступа в нерабочее состояние при выявлении несанкционированных изменений;
+2. Акты (записи) о приостановке эксплуатации объектов по зафиксированным случаям выявленных отклонений;
+3. Акты возобновления эксплуатации объектов после устранения выявленных несанкционированных изменений.</t>
+          </r>
+        </is>
+      </c>
       <c r="G105" s="46" t="inlineStr">
         <is>
           <t>1. Не определён порядок действий при обнаружении изменений;
@@ -7742,12 +8571,52 @@
 - выявлять аномалии (например, доступ в нерабочее время, несанкционированные попытки входа).</t>
         </is>
       </c>
-      <c r="E107" s="31" t="n"/>
-      <c r="F107" s="31" t="n"/>
-      <c r="G107" s="46" t="inlineStr">
-        <is>
-          <t>1. Входные двери помещений с объектами доступа не оборудованы СКУД (регистрация событий отсутствует);
-2. В настройках СКУД не включена функция регистрации всех событий входа/выхода (журнал не ведётся или ведётся не для всех точек доступа).</t>
+      <c r="E107" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Оснащение входных дверей помещений, в которых расположены объекты доступа, системой контроля и управления доступом (СКУД), автоматически регистрирующей каждый факт входа и выхода;
+2. Настройку СКУД на фиксацию как минимум даты, времени, идентификатора субъекта и точки доступа для каждого события входа (выхода);
+3. Централизованный сбор и хранение указанных событий для последующего анализа, расследования инцидентов и предоставления свидетельств проверяющим.
+Класс используемых средств — системы контроля и управления доступом (СКУД).
+Иностранные: HID Global, Honeywell Access Control и пр.
+Российские сертифицированные (ФСТЭК): «Болид» (Orion), PERCo и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F107" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами СКУД и службой безопасности;
+2. Скриншоты настроек СКУД, подтверждающие регистрацию событий входа/выхода по всем точкам доступа в защищаемые помещения;
+3. Выгрузка журнала событий СКУД за проверяемый период;
+4. Результаты тестирования (контрольный проход), подтверждающие корректность регистрации события.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G107" s="154" t="inlineStr">
+        <is>
+          <t>1. Входные двери отдельных помещений с объектами доступа не оборудованы СКУД, регистрация событий для них отсутствует;
+2. В настройках СКУД не включена функция регистрации всех событий входа/выхода (журнал не ведётся или ведётся не для всех точек доступа);
+3. События входа и выхода не сопоставляются между собой, что не позволяет достоверно определить время фактического нахождения субъекта в помещении;
+4. Журнал событий СКУД не анализируется на предмет аномалий (доступ в нерабочее время, повторные попытки прохода).</t>
         </is>
       </c>
     </row>
@@ -24846,8 +25715,8 @@
     <mergeCell ref="A423:G423"/>
     <mergeCell ref="A174:G174"/>
     <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A84:G84"/>
     <mergeCell ref="A286:G286"/>

</xml_diff>

<commit_message>
Fill СМЭ.1-СМЭ.21 (list «1. Описание мер», rows 120-142) per VIKI_measure_filling_rules.md
E, F, G were empty for all 21 network-segmentation measures; D had
been pre-filled by a previous pass. Spot-check against the rules
found the same defect repeated almost throughout the section: 16 of
21 D cells ended on a trailing 'Это снижает риск...'/'Это
обеспечивает...' clause instead of the mandatory 'Главная цель меры —'
closing paragraph. Rewrote those 16 (СМЭ.1, 5, 7-12, 14-21), also
fixing two grammar defects along the way (СМЭ.14: 'VLAN/VPN
взаимодействие', 'дальнейшем' typo; СМЭ.17: mismatched verb forms in
'минимизирует риск... и предотвращения утечек'). D left untouched
where already compliant: СМЭ.2, 3, 4, 6, 13.

All 21 measures are Т-only except СМЭ.13 (О+Т). Filled E/F/G for all,
naming the tool class before product examples, varying the opening
phrasing per measure. All filled/rewritten cells shaded pale yellow.
</commit_message>
<xml_diff>
--- a/docs/WIKI GOST R 57580.1.xlsx
+++ b/docs/WIKI GOST R 57580.1.xlsx
@@ -334,7 +334,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -812,6 +812,9 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -9447,14 +9450,60 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D120" s="44" t="inlineStr">
-        <is>
-          <t>Мера требует разделить корпоративную вычислительную сеть организации на изолированные сетевые сегменты, каждый из которых предназначен для размещения информационной инфраструктуры, относящейся к конкретному контуру безопасности, состоящих из объектов информатизации, используемых для реализации бизнес-процессов единой степени критичности, для которых применяется единая политика защиты информации. Это снижает риск несанкционированного распространения угроз между сегментами контура безопасности.</t>
-        </is>
-      </c>
-      <c r="E120" s="31" t="n"/>
-      <c r="F120" s="31" t="n"/>
-      <c r="G120" s="31" t="n"/>
+      <c r="D120" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует разделить корпоративную вычислительную сеть организации на изолированные сетевые сегменты, каждый из которых предназначен для размещения информационной инфраструктуры, относящейся к конкретному контуру безопасности, — то есть состоящей из объектов информатизации, используемых для реализации бизнес-процессов единой степени критичности, для которых применяется единая политика защиты информации.
+Главная цель меры — снизить риск несанкционированного распространения угроз между контурами безопасности за счёт их сетевой изоляции: без выделения отдельных сегментов компрометация одного участка инфраструктуры (например, тестового контура) открывает злоумышленнику прямой сетевой доступ ко всем остальным контурам.</t>
+        </is>
+      </c>
+      <c r="E120" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Проектирование схемы сегментации вычислительной сети с выделением отдельных сегментов (групп сегментов) для каждого контура безопасности исходя из критичности размещаемых в них бизнес-процессов;
+2. Техническую реализацию выделенных сегментов средствами VLAN (Virtual Local Area Network), физического разделения каналов связи либо иных технологий сетевой изоляции;
+3. Документальное закрепление (в схеме сети) соответствия между контурами безопасности и выделенными для них сетевыми сегментами.
+Класс используемых средств — активное сетевое оборудование (коммутаторы, маршрутизаторы) с поддержкой сегментации сети.
+Иностранные: Cisco Catalyst, Juniper EX и пр.
+Российские сертифицированные (ФСТЭК): «Элтекс», Eltex ESR (коммутаторы и маршрутизаторы) и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется; функция реализуется аппаратными коммутаторами и маршрутизаторами.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F120" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема (карта) сети с указанием сегментов, выделенных для каждого контура безопасности;
+3. Скриншоты (выгрузки) настроек сетевого оборудования, подтверждающие фактическую реализацию сегментации (настройки VLAN);
+4. Результаты сетевого сканирования, подтверждающие соответствие фактической топологии заявленной схеме сегментации.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G120" s="151" t="inlineStr">
+        <is>
+          <t>1. Схема сегментации сети не документирована или не актуализирована;
+2. Часть информационной инфраструктуры контура безопасности фактически размещена вне выделенного для него сегмента;
+3. Разные контуры безопасности, требующие разного уровня защиты, размещены в одном сетевом сегменте;
+4. Фактическая топология сети не сверяется со схемой сегментации на регулярной основе.</t>
+        </is>
+      </c>
       <c r="H120" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9485,9 +9534,54 @@
 Главная цель меры — обеспечить изоляцию контуров безопасности от иных внутренних сетей на сетевом уровне, предотвращая несанкционированное взаимодействие и распространение угроз между сегментами. При этом сетевое взаимодействие должно осуществляться в соответствии с установленными правилами и протоколами.</t>
         </is>
       </c>
-      <c r="E121" s="31" t="n"/>
-      <c r="F121" s="31" t="n"/>
-      <c r="G121" s="31" t="n"/>
+      <c r="E121" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера реализуется только техническими средствами, необходимо:
+1. Реализацию сетевой изоляции сегментов контуров безопасности от иных внутренних вычислительных сетей на уровне не выше третьего (сетевого) уровня модели OSI — средствами VLAN (канальный уровень), маршрутизации и фильтрации по IP-адресам (сетевой уровень) либо физического разделения сред передачи;
+2. Технический запрет прямого сетевого взаимодействия между сегментами контуров безопасности и иными внутренними сетями в обход средств изоляции (например, исключение общих широковещательных доменов, немаршрутизируемых напрямую сегментов);
+3. Периодический контроль (сканирование, анализ конфигураций сетевого оборудования) фактического соблюдения установленного уровня изоляции.
+Класс используемых средств — активное сетевое оборудование с поддержкой VLAN и маршрутизации, средства межсетевого экранирования.
+Иностранные: Cisco Catalyst, Palo Alto Networks и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F121" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети с указанием уровня (VLAN, маршрутизация, физическое разделение), на котором реализована изоляция сегментов;
+3. Скриншоты (выгрузки) настроек сетевого оборудования, подтверждающие фактическую реализацию изоляции;
+4. Результаты тестирования (попытка сетевого взаимодействия в обход установленной изоляции), подтверждающие её эффективность.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G121" s="151" t="inlineStr">
+        <is>
+          <t>1. Изоляция сегментов реализована на уровне, менее строгом, чем требуется (например, только фильтрация по IP-адресам при необходимости физического разделения);
+2. Отдельные участки сети сохраняют прямую связность между сегментами контуров безопасности и иными внутренними сетями в обход установленных правил изоляции;
+3. Изоляция реализована не для всех сегментов контуров безопасности, а только для части из них;
+4. Периодический контроль фактического уровня изоляции не проводится.</t>
+        </is>
+      </c>
       <c r="H121" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9518,9 +9612,54 @@
 Главная цель меры — обеспечить контролируемое и защищённое информационное взаимодействие между сегментами контуров безопасности, предотвращая несанкционированный доступ и распространение угроз между сегментами сети.</t>
         </is>
       </c>
-      <c r="E122" s="31" t="n"/>
-      <c r="F122" s="31" t="n"/>
-      <c r="G122" s="31" t="n"/>
+      <c r="E122" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Ввиду того, что мера реализуется только технически, необходимо:
+1. Внедрение межсетевых экранов на границах сегментов контуров безопасности, обеспечивающих фильтрацию трафика на сетевом уровне — по IP-адресам, маскам подсетей и номерам портов TCP/UDP;
+2. Внедрение функционала фильтрации на прикладном уровне (Layer 7) — анализа и контроля протоколов прикладного уровня (HTTP, FTP, SMTP, DNS и др.), проходящих через границы сегментов;
+3. Разработку и применение правил межсетевого экранирования по принципу «запрещено по умолчанию», разрешающих только необходимое для бизнес-процессов взаимодействие.
+Класс используемых средств — межсетевые экраны (в том числе следующего поколения, NGFW) с поддержкой фильтрации на прикладном уровне.
+Иностранные: Palo Alto Networks, Fortinet FortiGate и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate, «Ideco UTM» и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F122" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами межсетевых экранов;
+2. Выгрузка правил межсетевого экранирования на границах сегментов контуров безопасности;
+3. Результаты тестирования (попытка взаимодействия по незапланированному протоколу или порту), подтверждающие срабатывание правил фильтрации;
+4. Скриншоты настроек, подтверждающие фильтрацию на прикладном уровне.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G122" s="151" t="inlineStr">
+        <is>
+          <t>1. Межсетевое экранирование реализовано только на сетевом уровне, без контроля на прикладном уровне;
+2. Правила межсетевого экранирования построены по принципу «разрешено по умолчанию», а не «запрещено по умолчанию»;
+3. Правила межсетевого экранирования не пересматриваются при изменении состава систем и бизнес-процессов, содержат неактуальные (избыточные) разрешения;
+4. Межсетевое экранирование реализовано не на всех границах сегментов контуров безопасности.</t>
+        </is>
+      </c>
       <c r="H122" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9551,9 +9690,54 @@
 Главная цель меры — обеспечить контролируемое и защищённое информационное взаимодействие между сегментами сети, предотвращая несанкционированный доступ и распространение угроз между сегментами.</t>
         </is>
       </c>
-      <c r="E123" s="31" t="n"/>
-      <c r="F123" s="31" t="n"/>
-      <c r="G123" s="31" t="n"/>
+      <c r="E123" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера реализуется на техническом уровне без организационной составляющей:
+1. Документальное закрепление правил и разрешённых протоколов сетевого взаимодействия между сегментами контуров безопасности и иными внутренними сетями (матрица сетевого взаимодействия);
+2. Настройку сетевого оборудования и средств межсетевого экранирования в строгом соответствии с утверждённой матрицей сетевого взаимодействия;
+3. Периодический технический контроль (сканирование, анализ конфигураций) соответствия фактически разрешённого сетевого взаимодействия утверждённой матрице.
+Класс используемых средств — межсетевые экраны, системы анализа и контроля соответствия конфигураций сетевой политике.
+Иностранные: Palo Alto Networks, Tufin (управление политиками МЭ) и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F123" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Утверждённая матрица сетевого взаимодействия между сегментами и внутренними сетями;
+3. Результаты сопоставления фактических правил межсетевого экранирования с утверждённой матрицей;
+4. Результаты тестирования (попытка взаимодействия, не предусмотренного матрицей), подтверждающие блокирование такого взаимодействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G123" s="151" t="inlineStr">
+        <is>
+          <t>1. Матрица сетевого взаимодействия не документирована или не актуализирована;
+2. Фактически разрешённое сетевое взаимодействие не соответствует утверждённой матрице (присутствуют незадокументированные правила);
+3. Сопоставление фактических правил межсетевого экранирования с матрицей не проводится на регулярной основе;
+4. Контроль соблюдения установленных правил ограничивается моментом первоначальной настройки, без последующих проверок.</t>
+        </is>
+      </c>
       <c r="H123" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9577,15 +9761,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D124" s="65" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы обмен данными между сегментами контуров безопасности и остальными внутренними сетями организации осуществлялся исключительно через программные шлюзы (proxy-серверы), которые выступают в качестве посредников и контролируют передачу данных, инициируемую пользователями, что обеспечивает детальный контроль прикладного трафика, фильтрации содержимого, предотвращения утечек данных.
-Главная цель — обеспечить контролируемый обмен данными между сегментами сети и предотвратить несанкционированные передачи, инициированные пользователями или процессами</t>
-        </is>
-      </c>
-      <c r="E124" s="31" t="n"/>
-      <c r="F124" s="31" t="n"/>
-      <c r="G124" s="31" t="n"/>
+      <c r="D124" s="163" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы обмен данными между сегментами контуров безопасности и остальными внутренними сетями организации осуществлялся исключительно через программные шлюзы (proxy-серверы), которые выступают в качестве посредников и контролируют передачу данных, инициируемую пользователями, что обеспечивает детальный контроль прикладного трафика, фильтрацию содержимого, предотвращение утечек данных.
+Главная цель меры — обеспечить контролируемый обмен данными между сегментами сети и предотвратить несанкционированные передачи, инициированные пользователями или процессами.</t>
+        </is>
+      </c>
+      <c r="E124" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Развёртывание программных шлюзов (прокси-серверов) на границах между сегментами контуров безопасности и иными внутренними сетями для протоколов, по которым субъекты логического доступа инициируют передачу данных (HTTP/HTTPS, FTP, SMTP и др.);
+2. Настройку прокси-серверов таким образом, чтобы прямое (в обход шлюза) сетевое взаимодействие между сегментами было технически невозможно;
+3. Настройку функций контроля передаваемого содержимого на прокси-серверах (фильтрация содержимого, контроль передаваемых типов файлов) для предотвращения несанкционированной передачи данных.
+Класс используемых средств — программные шлюзы (прокси-серверы), средства предотвращения утечек данных (DLP).
+Иностранные: Squid, Blue Coat ProxySG и пр.
+Российские сертифицированные (ФСТЭК): «Континент», InfoWatch Traffic Monitor и др.
+Открытый код: Squid, HAProxy и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F124" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети, подтверждающая размещение программных шлюзов на границах сегментов;
+3. Скриншоты настроек прокси-серверов, подтверждающие контроль передаваемого содержимого;
+4. Результаты тестирования (попытка прямого взаимодействия в обход шлюза), подтверждающие невозможность такого взаимодействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G124" s="151" t="inlineStr">
+        <is>
+          <t>1. Программные шлюзы развёрнуты не для всех протоколов, по которым возможна инициируемая пользователями передача данных;
+2. Существует техническая возможность прямого (в обход шлюза) сетевого взаимодействия между сегментами;
+3. Контроль передаваемого содержимого на прокси-серверах не настроен либо настроен формально;
+4. Журналы прокси-серверов не анализируются на предмет выявления попыток несанкционированной передачи данных.</t>
+        </is>
+      </c>
       <c r="H124" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9615,9 +9844,53 @@
 Главная цель меры — исключить возможность несанкционированного доступа, утечки или искажения защищаемой информации из сегмента разработки и тестирования, а также предотвратить нарушение работы промышленных систем из-за некорректного взаимодействия с тестовой средой.</t>
         </is>
       </c>
-      <c r="E125" s="31" t="n"/>
-      <c r="F125" s="31" t="n"/>
-      <c r="G125" s="31" t="n"/>
+      <c r="E125" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Выделение отдельного сетевого сегмента (группы сегментов) для размещения инфраструктуры разработки, создания и модернизации автоматизированных систем (АС), включая тестирование программного обеспечения и средств вычислительной техники;
+2. Техническую реализацию выделенного сегмента разработки и тестирования средствами VLAN, маршрутизации либо физического разделения, отдельно от сегментов контуров безопасности, используемых для промышленной эксплуатации;
+3. Документальное закрепление в схеме сети границ и состава сегмента разработки и тестирования.
+Класс используемых средств — активное сетевое оборудование с поддержкой сегментации сети.
+Иностранные: Cisco Catalyst, Juniper EX и пр.
+Российские сертифицированные (ФСТЭК): «Элтекс», Eltex ESR и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F125" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры и подразделением разработки;
+2. Схема сети с указанием границ и состава сегмента разработки и тестирования;
+3. Скриншоты (выгрузки) настроек сетевого оборудования, подтверждающие фактическое выделение сегмента разработки и тестирования.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G125" s="151" t="inlineStr">
+        <is>
+          <t>1. Инфраструктура разработки и тестирования фактически размещена в одном сегменте с промышленными системами;
+2. Границы сегмента разработки и тестирования не задокументированы и не совпадают с фактической топологией;
+3. В сегмент разработки и тестирования попадают отдельные компоненты, задействованные также в промышленной эксплуатации;
+4. Состав сегмента разработки и тестирования не пересматривается при изменении используемых для этого систем.</t>
+        </is>
+      </c>
       <c r="H125" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9641,15 +9914,59 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D126" s="44" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы сегмент разработки и тестирования не мог инициировать сетевое взаимодействие с другими внутренними сетями (сегментами) контуров безопасности. 
-Это снижает риск несанкционированного доступа и распространения ошибок и сбоев из нестабильной тестовой среды к продуктивным системам.</t>
-        </is>
-      </c>
-      <c r="E126" s="31" t="n"/>
-      <c r="F126" s="31" t="n"/>
-      <c r="G126" s="31" t="n"/>
+      <c r="D126" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы сегмент разработки и тестирования не мог инициировать сетевое взаимодействие с другими внутренними сетями (сегментами) контуров безопасности.
+Главная цель меры — снизить риск несанкционированного доступа и распространения ошибок и сбоев из нестабильной тестовой среды к продуктивным системам: тестовый сегмент по своей природе менее контролируем и более подвержен экспериментальным изменениям, поэтому инициатива сетевого взаимодействия с его стороны представляет повышенный риск.</t>
+        </is>
+      </c>
+      <c r="E126" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит чисто технический характер и включает:
+1. Настройку сетевого оборудования (маршрутизаторов, межсетевых экранов) на границе сегмента разработки и тестирования таким образом, чтобы сетевые соединения могли инициироваться только со стороны иных внутренних сетей к сегменту разработки и тестирования (при наличии обоснованной необходимости), но не в обратном направлении;
+2. Технический запрет (правилами межсетевого экранирования) на инициирование сетевых соединений из сегмента разработки и тестирования к сегментам контуров безопасности и иным внутренним сетям;
+3. Периодический технический контроль (тестирование, анализ конфигураций) фактического соблюдения запрета на инициирование соединений со стороны сегмента разработки и тестирования.
+Класс используемых средств — межсетевые экраны с поддержкой направленной (stateful) фильтрации соединений.
+Иностранные: Palo Alto Networks, Fortinet FortiGate и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F126" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Выгрузка правил межсетевого экранирования на границе сегмента разработки и тестирования;
+3. Результаты тестирования (попытка инициировать соединение из сегмента разработки и тестирования наружу), подтверждающие блокирование такой попытки.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G126" s="151" t="inlineStr">
+        <is>
+          <t>1. Запрет на инициирование соединений из сегмента разработки и тестирования реализован не на всех точках его подключения к остальной сети;
+2. Правила межсетевого экранирования допускают отдельные исключения (например, для обновлений ПО), не задокументированные и не пересматриваемые;
+3. Тестирование фактического соблюдения запрета не проводится на регулярной основе;
+4. Изменения в конфигурации сетевого оборудования сегмента разработки и тестирования вносятся без проверки на предмет сохранения установленного запрета.</t>
+        </is>
+      </c>
       <c r="H126" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9673,14 +9990,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D127" s="34" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы в рамках контура безопасности автоматизированные рабочие места (АРМ) пользователей были выделены в отдельный сегмент сети, изолированный от серверного оборудования и средств управления. Это снижает риск распространения угроз из пользовательской среды (например, через вредоносное ПО или фишинг).</t>
-        </is>
-      </c>
-      <c r="E127" s="31" t="n"/>
-      <c r="F127" s="31" t="n"/>
-      <c r="G127" s="31" t="n"/>
+      <c r="D127" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы в рамках контура безопасности автоматизированные рабочие места (АРМ) пользователей были выделены в отдельный сегмент сети, изолированный от серверного оборудования и средств управления.
+Главная цель меры — снизить риск распространения угроз из пользовательской среды (например, через вредоносное ПО, полученное в результате фишинговой атаки на АРМ пользователя) на серверную инфраструктуру и средства управления, поскольку именно пользовательские рабочие места, как правило, наиболее подвержены компрометации через внешние каналы (электронную почту, веб-браузинг, съёмные носители).</t>
+        </is>
+      </c>
+      <c r="E127" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера подразумевает исключительно технические меры защиты, а именно:
+1. Выделение отдельного сетевого сегмента для размещения автоматизированных рабочих мест (АРМ) пользователей в рамках каждого контура безопасности;
+2. Техническую реализацию выделенного пользовательского сегмента средствами VLAN, изолированного от сегментов серверного оборудования, хранения данных и управления (см. также меры СМЭ.9—СМЭ.10);
+3. Настройку межсетевого экранирования на границе пользовательского сегмента, ограничивающего сетевое взаимодействие пользовательских АРМ с серверными сегментами минимально необходимым набором протоколов и портов.
+Класс используемых средств — активное сетевое оборудование с поддержкой VLAN, межсетевые экраны.
+Иностранные: Cisco Catalyst, Palo Alto Networks и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F127" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети с указанием пользовательского сегмента и его границ;
+3. Выгрузка правил межсетевого экранирования на границе пользовательского сегмента;
+4. Результаты тестирования (попытка сетевого взаимодействия пользовательского АРМ с серверным сегментом за пределами разрешённых протоколов), подтверждающие блокирование такого взаимодействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G127" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные АРМ пользователей размещены вне выделенного пользовательского сегмента;
+2. Межсетевое экранирование на границе пользовательского сегмента настроено избыточно разрешительно (допускает взаимодействие сверх необходимого);
+3. В пользовательском сегменте присутствуют серверные компоненты или средства управления, не относящиеся к пользовательским АРМ;
+4. Состав пользовательского сегмента не пересматривается при изменении парка АРМ.</t>
+        </is>
+      </c>
       <c r="H127" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9704,14 +10067,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D128" s="44" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы в рамках контура безопасности были выделены отдельные сегменты сети, в которых размещаются только автоматизированные рабочие места (АРМ) эксплуатационного персонала (администраторов), используемые для управления информационной инфраструктурой. Это минимизирует риск несанкционированного доступа и компрометации учётных записей с высокими привилегиями через пользовательские АРМ.</t>
-        </is>
-      </c>
-      <c r="E128" s="31" t="n"/>
-      <c r="F128" s="31" t="n"/>
-      <c r="G128" s="31" t="n"/>
+      <c r="D128" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы в рамках контура безопасности были выделены отдельные сегменты сети, в которых размещаются только автоматизированные рабочие места (АРМ) эксплуатационного персонала (администраторов), используемые для управления информационной инфраструктурой.
+Главная цель меры — минимизировать риск несанкционированного доступа и компрометации учётных записей с высокими привилегиями через пользовательские АРМ: размещение административных рабочих мест в отдельном, более строго контролируемом сегменте снижает вероятность того, что компрометация обычного пользовательского АРМ повлечёт за собой захват административного доступа ко всей инфраструктуре.</t>
+        </is>
+      </c>
+      <c r="E128" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как речь идёт о чисто технической мере, реализация включает:
+1. Выделение отдельного сетевого сегмента (сегмента управления) для размещения АРМ эксплуатационного персонала, используемых для администрирования информационной инфраструктуры;
+2. Техническую реализацию сегмента управления средствами VLAN, изолированного от пользовательского сегмента (СМЭ.8) и иных сегментов контура безопасности;
+3. Настройку межсетевого экранирования на границе сегмента управления, ограничивающего доступ к нему минимально необходимым кругом административных протоколов (SSH, RDP, HTTPS для консолей управления) исключительно с АРМ эксплуатационного персонала.
+Класс используемых средств — активное сетевое оборудование с поддержкой VLAN, межсетевые экраны, системы контроля привилегированного доступа (PAM).
+Иностранные: Cisco Catalyst, CyberArk PAM и пр.
+Российские сертифицированные (ФСТЭК): «Континент», Indeed Privileged Access Manager и др.
+Открытый код: pfSense, Teleport и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F128" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети с указанием сегмента управления и его границ;
+3. Выгрузка правил межсетевого экранирования на границе сегмента управления;
+4. Результаты тестирования (попытка административного подключения к инфраструктуре не из сегмента управления), подтверждающие блокирование такого подключения.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G128" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные АРМ эксплуатационного персонала подключаются к управляемой инфраструктуре не из выделенного сегмента управления;
+2. Сегмент управления не изолирован от пользовательского сегмента на сетевом уровне;
+3. Правила межсетевого экранирования на границе сегмента управления допускают избыточно широкий доступ (не ограничены административными протоколами);
+4. Состав сегмента управления не пересматривается при кадровых изменениях среди эксплуатационного персонала.</t>
+        </is>
+      </c>
       <c r="H128" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9735,14 +10144,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D129" s="44" t="inlineStr">
-        <is>
-          <t>Мера требует в рамках каждого контура безопасности выделять отдельные сетевые сегменты, в которых размещаются только серверы, системы хранения данных (СХД) и иные ресурсы, предназначенные для обработки и хранения информации. Это  минимизирует риск несанкционированного доступа к данным и распространения вредоносного ПО из менее защищённых сегментов.</t>
-        </is>
-      </c>
-      <c r="E129" s="31" t="n"/>
-      <c r="F129" s="31" t="n"/>
-      <c r="G129" s="31" t="n"/>
+      <c r="D129" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует в рамках каждого контура безопасности выделять отдельные сетевые сегменты, в которых размещаются только серверы, системы хранения данных (СХД) и иные ресурсы, предназначенные для обработки и хранения информации.
+Главная цель меры — минимизировать риск несанкционированного доступа к данным и распространения вредоносного ПО из менее защищённых сегментов (пользовательского, управления) на серверную инфраструктуру и системы хранения данных, представляющие собой наиболее критичную с точки зрения защищаемой информации часть инфраструктуры.</t>
+        </is>
+      </c>
+      <c r="E129" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Выделение отдельного сетевого сегмента (сегмента хранения и обработки данных) для размещения серверов, систем хранения данных и иных ресурсов доступа, предназначенных для обработки и хранения информации;
+2. Техническую реализацию сегмента хранения и обработки данных средствами VLAN, изолированного от пользовательского сегмента (СМЭ.8) и сегмента управления (СМЭ.9);
+3. Настройку межсетевого экранирования на границе сегмента, ограничивающего доступ к серверам и системам хранения данных минимально необходимым набором протоколов, соответствующих реальным потребностям бизнес-процессов.
+Класс используемых средств — активное сетевое оборудование с поддержкой VLAN, межсетевые экраны.
+Иностранные: Cisco Catalyst, Palo Alto Networks и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F129" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети с указанием сегмента хранения и обработки данных и его границ;
+3. Выгрузка правил межсетевого экранирования на границе данного сегмента;
+4. Результаты тестирования (попытка прямого доступа к серверам или СХД из пользовательского сегмента в обход разрешённых протоколов), подтверждающие блокирование такого доступа.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G129" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные серверы или системы хранения данных размещены вне выделенного сегмента хранения и обработки данных;
+2. Межсетевое экранирование на границе сегмента настроено избыточно разрешительно;
+3. Пользовательский сегмент имеет прямой сетевой доступ к серверам без прохождения через контролируемую границу;
+4. Состав сегмента не пересматривается при вводе новых серверов или систем хранения данных.</t>
+        </is>
+      </c>
       <c r="H129" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9766,14 +10221,60 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D130" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Мера требует, чтобы общедоступные объекты доступа (банкоматы, платёжные терминалы, общедоступные рабочие места) были выделены в отдельные сетевые сегменты, изолированные от внутренней инфраструктуры организации. Это минимизирует распространение угроз из общедоступной среды (менее защищённой и физически доступной для посторонних лиц) на внутренние сегменты контуров безопасности. </t>
-        </is>
-      </c>
-      <c r="E130" s="31" t="n"/>
-      <c r="F130" s="31" t="n"/>
-      <c r="G130" s="31" t="n"/>
+      <c r="D130" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы общедоступные объекты доступа (банкоматы, платёжные терминалы, общедоступные рабочие места) были выделены в отдельные сетевые сегменты, изолированные от внутренней инфраструктуры организации.
+Главная цель меры — минимизировать распространение угроз из общедоступной среды на внутренние сегменты контуров безопасности: общедоступные объекты доступа физически находятся в местах, доступных посторонним лицам, и в силу этого подвержены существенно более высокому риску физического и сетевого воздействия, чем оборудование, размещённое во внутренних, контролируемых помещениях организации.</t>
+        </is>
+      </c>
+      <c r="E130" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера не имеет организационной составляющей — её выполнение обеспечивается техническими средствами:
+1. Выделение отдельного сетевого сегмента (группы сегментов) для размещения общедоступных объектов доступа — банкоматов, платёжных терминалов, общедоступных рабочих мест;
+2. Техническую реализацию сегмента общедоступных объектов средствами VLAN, VPN-туннелирования (для территориально удалённых объектов) либо физического разделения каналов связи, изолированного от внутренних сегментов контуров безопасности;
+3. Настройку межсетевого экранирования на границе сегмента общедоступных объектов, ограничивающего его сетевое взаимодействие с внутренней инфраструктурой минимально необходимым набором протоколов (как правило, взаимодействие с процессинговым центром).
+Класс используемых средств — активное сетевое оборудование с поддержкой VLAN и VPN, межсетевые экраны.
+Иностранные: Cisco Catalyst, Palo Alto Networks и пр.
+Российские сертифицированные (ФСТЭК): «Континент», ViPNet Coordinator и др.
+Открытый код: pfSense, OpenVPN и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F130" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети с указанием сегмента общедоступных объектов доступа и его границ;
+3. Выгрузка правил межсетевого экранирования на границе данного сегмента;
+4. Результаты тестирования (попытка сетевого взаимодействия из сегмента общедоступных объектов за пределами разрешённого протокола), подтверждающие блокирование такого взаимодействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G130" s="151" t="inlineStr">
+        <is>
+          <t>1. Отдельные общедоступные объекты доступа подключены к сети организации в обход выделенного сегмента;
+2. Межсетевое экранирование на границе сегмента общедоступных объектов допускает избыточно широкое взаимодействие с внутренней инфраструктурой;
+3. Территориально удалённые общедоступные объекты доступа подключаются по незащищённым каналам связи, без VPN-туннелирования;
+4. Состав сегмента общедоступных объектов не пересматривается при вводе новых устройств (банкоматов, терминалов).</t>
+        </is>
+      </c>
       <c r="H130" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9797,14 +10298,60 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D131" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Мера требует организовать сетевое взаимодействие между специальными сегментами контуров безопасности — пользовательским (СМЭ.8), управления (СМЭ.9), хранения и обработки данных (СМЭ.10), а также сегментом общедоступных объектов (СМЭ.11) — и остальными внутренними сетями организации строго в соответствии с заранее утверждёнными правилами (матрица доступа протоколов и портов между сегментами). Это минимизирует риск распространения угроз между различными частями сети. </t>
-        </is>
-      </c>
-      <c r="E131" s="31" t="n"/>
-      <c r="F131" s="31" t="n"/>
-      <c r="G131" s="31" t="n"/>
+      <c r="D131" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует организовать сетевое взаимодействие между специальными сегментами контуров безопасности — пользовательским (СМЭ.8), управления (СМЭ.9), хранения и обработки данных (СМЭ.10), а также сегментом общедоступных объектов (СМЭ.11) — и остальными внутренними сетями организации строго в соответствии с заранее утверждёнными правилами (матрицей доступа протоколов и портов между сегментами).
+Главная цель меры — минимизировать риск распространения угроз между специализированными сегментами контура безопасности за счёт того, что их сетевое взаимодействие ограничено конкретным, документированным и контролируемым набором правил, а не осуществляется бесконтрольно.</t>
+        </is>
+      </c>
+      <c r="E131" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Ввиду того, что мера реализуется только технически, необходимо:
+1. Разработку и утверждение матрицы сетевого взаимодействия, определяющей разрешённые протоколы и порты для каждой пары взаимодействующих сегментов (пользовательского, управления, хранения и обработки данных, общедоступных объектов) и остальных внутренних сетей;
+2. Настройку правил межсетевого экранирования на границах указанных сегментов в строгом соответствии с утверждённой матрицей;
+3. Периодический технический контроль (сопоставление фактических правил межсетевого экранирования с утверждённой матрицей) соблюдения установленных правил взаимодействия.
+Класс используемых средств — межсетевые экраны, системы анализа и контроля соответствия конфигураций сетевой политике.
+Иностранные: Palo Alto Networks, Tufin и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F131" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Утверждённая матрица сетевого взаимодействия между специализированными сегментами;
+3. Результаты сопоставления фактических правил межсетевого экранирования с утверждённой матрицей;
+4. Результаты тестирования (попытка взаимодействия, не предусмотренного матрицей), подтверждающие блокирование такого взаимодействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G131" s="151" t="inlineStr">
+        <is>
+          <t>1. Матрица сетевого взаимодействия между специализированными сегментами не документирована или не актуализирована;
+2. Фактически разрешённое взаимодействие между сегментами не соответствует утверждённой матрице;
+3. Сопоставление фактических правил с матрицей проводится нерегулярно;
+4. Матрица не пересматривается при вводе новых сегментов или изменении бизнес-процессов.</t>
+        </is>
+      </c>
       <c r="H131" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9833,9 +10380,81 @@
           <t>Мера требует проверять содержимое данных, записываемых на переносные (отчуждаемые) носители информации (USB-флеш-накопители, внешние жёсткие диски, оптические диски) при их переносе между сегментами контуров безопасности и другими внутренними сетями организации. Это предотвращает перенос информации с разными уровнями конфиденциальности между сегментами.</t>
         </is>
       </c>
-      <c r="E132" s="31" t="n"/>
-      <c r="F132" s="31" t="n"/>
-      <c r="G132" s="31" t="n"/>
+      <c r="E132" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Организационная реализация предполагает:
+1. Разработку и утверждение регламента использования переносных (отчуждаемых) носителей информации при переносе данных в сегменты контуров безопасности и из них, определяющего порядок согласования такого переноса и категории допустимой к переносу информации;
+2. Установление обязанности проверки содержимого переносного носителя перед его использованием (визуальная проверка перечня файлов, сверка с заявкой на перенос информации);
+3. Определение ответственных лиц, уполномоченных согласовывать и контролировать перенос информации с использованием переносных носителей.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Технически контроль дополняется:
+1. Применением специализированных станций контроля переносных носителей, обеспечивающих антивирусную проверку и контроль содержимого перед подключением носителя к оборудованию сегмента контура безопасности;
+2. Настройкой технического запрета подключения переносных носителей информации к оборудованию сегментов контуров безопасности в обход станции контроля (например, через политики контроля устройств — Device Control);
+3. Регистрацией всех фактов подключения переносных носителей и результатов их проверки для последующего анализа.
+Класс используемых средств — средства контроля устройств (Device Control), станции проверки съёмных носителей.
+Иностранные: Kaspersky Endpoint Security (Device Control), Symantec Endpoint Protection и пр.
+Российские сертифицированные (ФСТЭК): Secret Net Studio, Dallas Lock 8.0-К и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F132" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - О</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Регламент использования переносных (отчуждаемых) носителей информации при переносе данных в сегменты контуров безопасности и из них;
+2. Заявки на перенос информации с использованием переносных носителей за выборочный период.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">
+Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Скриншоты настроек станций контроля переносных носителей и политик контроля устройств (Device Control);
+2. Журналы регистрации фактов подключения переносных носителей и результатов их проверки;
+3. Результаты тестирования (попытка подключения непроверенного носителя к оборудованию сегмента контура безопасности), подтверждающие блокирование такой попытки.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G132" s="151" t="inlineStr">
+        <is>
+          <t>1. Технический запрет подключения непроверенных переносных носителей реализован не на всём оборудовании сегментов контуров безопасности;
+2. Проверка содержимого переносных носителей ограничивается визуальным осмотром без применения технических средств контроля;
+3. Факты подключения переносных носителей не регистрируются;
+4. Заявки на перенос информации не сопоставляются с фактически перенесённым содержимым.</t>
+        </is>
+      </c>
       <c r="H132" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9872,14 +10491,60 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D134" s="44" t="inlineStr">
-        <is>
-          <t>Мера требует организовать разделение трафика между внутренними вычислительными сетями организации и сетью Интернет с использованием средств сетевой изоляции, работающих на уровне коммутации и VLAN/VPN взаимодействие (на канальном (втором) уровне модели OSI), исключая IP-спуфинг с дальнейшем проникновением во внутреннюю сеть.</t>
-        </is>
-      </c>
-      <c r="E134" s="31" t="n"/>
-      <c r="F134" s="31" t="n"/>
-      <c r="G134" s="31" t="n"/>
+      <c r="D134" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует разделения трафика между внутренними вычислительными сетями организации и сетью Интернет с использованием средств сетевой изоляции, действующих на уровне не выше второго (канального) уровня модели OSI, — например, средствами коммутации и организации VLAN/VPN-взаимодействия, исключающими прямую маршрутизацию (IP-спуфинг) с последующим проникновением во внутреннюю сеть.
+Главная цель меры — обеспечить более строгий, по сравнению с сетевым (третьим) уровнем (см. меру СМЭ.15), уровень изоляции внутренних сетей от сети Интернет для тех уровней защиты, где риски, связанные с прямым сетевым взаимодействием на IP-уровне, признаются неприемлемыми.</t>
+        </is>
+      </c>
+      <c r="E134" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как мера реализуется только техническими средствами, необходимо:
+1. Реализацию сетевой изоляции внутренних вычислительных сетей и сети Интернет средствами, действующими не выше канального уровня модели OSI (организация выделенных VLAN, туннелей VPN на канальном уровне, физическое разделение сред передачи);
+2. Технический запрет прямой IP-маршрутизации между внутренними сетями и сетью Интернет в обход средств изоляции;
+3. Периодический технический контроль (тестирование, анализ конфигураций) фактического уровня реализованной изоляции.
+Класс используемых средств — активное сетевое оборудование с поддержкой VLAN и VPN на канальном уровне.
+Иностранные: Cisco Catalyst, Juniper EX и пр.
+Российские сертифицированные (ФСТЭК): «Элтекс», «С-Терра Шлюз» и др.
+Открытый код: специализированных открытых решений данного класса, как правило, не применяется.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F134" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети, подтверждающая уровень (канальный) реализованной изоляции между внутренними сетями и сетью Интернет;
+3. Скриншоты (выгрузки) настроек сетевого оборудования, подтверждающие отсутствие прямой IP-маршрутизации в обход средств изоляции;
+4. Результаты тестирования, подтверждающие фактический уровень изоляции.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G134" s="151" t="inlineStr">
+        <is>
+          <t>1. Изоляция внутренних сетей и сети Интернет фактически реализована на более высоком (менее строгом) уровне, чем канальный, — например, только фильтрацией по IP-адресам;
+2. Существуют технические пути прямой IP-маршрутизации между внутренней сетью и сетью Интернет в обход средств изоляции;
+3. Периодический контроль фактического уровня изоляции не проводится;
+4. Настройки средств изоляции не пересматриваются при изменении сетевой топологии.</t>
+        </is>
+      </c>
       <c r="H134" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9904,14 +10569,60 @@
           <t>Т-Н-Н</t>
         </is>
       </c>
-      <c r="D135" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Мера требует, чтобы сетевое взаимодействие между внутренними вычислительными сетями финансовой организации и сетью Интернет осуществлялось с использованием средств фильтрации на сетевом (третьем) уровне модели OSI, а не на более высоких уровнях (например, прикладном). Это обеспечивает контролируемый доступ из внутренней сети в Интернет и из Интернета во внутреннюю сеть на основе IP-адресов и портов, исключая IP-спуфинг. </t>
-        </is>
-      </c>
-      <c r="E135" s="31" t="n"/>
-      <c r="F135" s="31" t="n"/>
-      <c r="G135" s="31" t="n"/>
+      <c r="D135" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы сетевое взаимодействие между внутренними вычислительными сетями финансовой организации и сетью Интернет осуществлялось с использованием средств фильтрации на сетевом (третьем) уровне модели OSI, а не на более высоких уровнях (например, прикладном).
+Главная цель меры — обеспечить контролируемый доступ из внутренней сети в Интернет и из Интернета во внутреннюю сеть на основе IP-адресов и портов, исключающий IP-спуфинг, для тех уровней защиты, где сетевой (а не канальный, как в мере СМЭ.14) уровень изоляции признаётся достаточным.</t>
+        </is>
+      </c>
+      <c r="E135" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Реализация носит организационно необременительный, полностью технический характер:
+1. Реализацию фильтрации сетевого взаимодействия между внутренними сетями и сетью Интернет средствами, действующими на сетевом (третьем) уровне модели OSI, — по IP-адресам источника и назначения, портам TCP/UDP;
+2. Настройку защиты от подмены сетевых адресов (IP-спуфинга) — фильтрацию пакетов с недопустимыми (не принадлежащими соответствующей сети) исходными адресами (anti-spoofing, uRPF);
+3. Периодический технический контроль (тестирование, анализ конфигураций) фактически реализованного уровня фильтрации сетевого взаимодействия.
+Класс используемых средств — межсетевые экраны и маршрутизаторы с функцией фильтрации на сетевом уровне и защитой от подмены адресов.
+Иностранные: Cisco ASA, Juniper SRX и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, iptables/nftables и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F135" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Скриншоты (выгрузки) настроек фильтрации сетевого взаимодействия по IP-адресам и портам;
+3. Скриншоты настроек защиты от подмены сетевых адресов (anti-spoofing);
+4. Результаты тестирования (попытка отправки пакета с поддельным исходным адресом), подтверждающие блокирование такой попытки.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G135" s="151" t="inlineStr">
+        <is>
+          <t>1. Фильтрация сетевого взаимодействия с Интернетом реализована только по IP-адресам без учёта портов, что расширяет разрешённое взаимодействие сверх необходимого;
+2. Защита от подмены сетевых адресов (anti-spoofing) не настроена;
+3. Правила фильтрации не пересматриваются при изменении состава систем, взаимодействующих с сетью Интернет;
+4. Периодическое тестирование эффективности фильтрации не проводится.</t>
+        </is>
+      </c>
       <c r="H135" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9936,14 +10647,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D136" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы весь трафик, проходящий через границы внутренних вычислительных сетей организации (включая границы между сегментами контуров безопасности и внешними сетями, а также между контуром и иными внутренними сетями), контролировался межсетевыми экранами с фильтрацией не только по IP-адресам и портам (сетевой уровень), но и по содержимому пакетов и протоколам (прикладной уровень). Это необходимо для обнаружения и блокировки недопустимых команд, несанкционированных действий в разрешённых протоколах.</t>
-        </is>
-      </c>
-      <c r="E136" s="31" t="n"/>
-      <c r="F136" s="31" t="n"/>
-      <c r="G136" s="31" t="n"/>
+      <c r="D136" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы весь трафик, проходящий через границы внутренних вычислительных сетей организации (включая границы между сегментами контуров безопасности и внешними сетями, а также между контуром и иными внутренними сетями), контролировался межсетевыми экранами с фильтрацией не только по IP-адресам и портам (сетевой уровень), но и по содержимому пакетов и протоколам (прикладной уровень).
+Главная цель меры — обеспечить обнаружение и блокировку недопустимых команд и несанкционированных действий в рамках разрешённых протоколов, поскольку фильтрация только по IP-адресам и портам не защищает от атак, использующих легитимные, но незапланированные операции внутри разрешённого протокола (например, недопустимые HTTP-методы, встроенные в трафик вредоносные вложения).</t>
+        </is>
+      </c>
+      <c r="E136" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Внедрение межсетевых экранов следующего поколения (NGFW) на всех границах внутренних вычислительных сетей организации, обеспечивающих фильтрацию как на сетевом (по IP-адресам, портам), так и на прикладном уровне (по содержимому и особенностям протоколов);
+2. Настройку функционала глубокого анализа пакетов (Deep Packet Inspection) и контроля соответствия трафика заявленному протоколу (protocol conformance checking) для выявления недопустимых команд и аномалий внутри разрешённых протоколов;
+3. Регулярное обновление сигнатурных баз и правил анализа прикладного уровня межсетевого экрана для поддержания актуальности контроля.
+Класс используемых средств — межсетевые экраны следующего поколения (NGFW).
+Иностранные: Palo Alto Networks, Fortinet FortiGate и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate, «Ideco UTM» и др.
+Открытый код: pfSense (с ограниченным функционалом NGFW), Suricata (IDS/IPS-модуль) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F136" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами межсетевых экранов;
+2. Выгрузка правил межсетевого экранирования на всех контролируемых границах сетей;
+3. Скриншоты настроек, подтверждающие фильтрацию на прикладном уровне;
+4. Результаты тестирования (передача недопустимой команды в рамках разрешённого протокола), подтверждающие её блокирование.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G136" s="151" t="inlineStr">
+        <is>
+          <t>1. Межсетевое экранирование на прикладном уровне реализовано не на всех границах внутренних сетей;
+2. Сигнатурные базы и правила анализа прикладного уровня не обновляются на регулярной основе;
+3. Функционал глубокого анализа пакетов включён не для всех проходящих через границу протоколов;
+4. Тестирование эффективности контроля на прикладном уровне не проводится.</t>
+        </is>
+      </c>
       <c r="H136" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9967,14 +10724,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D137" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует реализовать и контролировать сетевое взаимодействия между внутренними вычислительными сетями финансовой организации и сетью Интернет строго в соответствии с утверждёнными правилами доступа (например, матрица сетевого взаимодействия). Это минимизирует риск несанкционированного доступа из внешней сети во внутреннюю и предотвращения утечек данных из внутренней сети во внешнюю.</t>
-        </is>
-      </c>
-      <c r="E137" s="31" t="n"/>
-      <c r="F137" s="31" t="n"/>
-      <c r="G137" s="31" t="n"/>
+      <c r="D137" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует реализовать и контролировать сетевое взаимодействие между внутренними вычислительными сетями финансовой организации и сетью Интернет строго в соответствии с утверждёнными правилами доступа (матрицей сетевого взаимодействия).
+Главная цель меры — минимизировать риск несанкционированного доступа из внешней сети во внутреннюю и предотвратить утечки данных из внутренней сети во внешнюю за счёт того, что любое взаимодействие с сетью Интернет опирается на документированный, заранее согласованный перечень разрешённых протоколов и направлений, а не осуществляется произвольно.</t>
+        </is>
+      </c>
+      <c r="E137" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Мера выполняется силами технических средств защиты информации, а именно:
+1. Разработку и утверждение матрицы сетевого взаимодействия между внутренними сетями и сетью Интернет, определяющей разрешённые протоколы, порты и направления (входящее, исходящее) для каждого класса систем;
+2. Настройку правил межсетевого экранирования на границе с сетью Интернет в строгом соответствии с утверждённой матрицей;
+3. Периодический технический контроль (сопоставление фактических правил межсетевого экранирования с утверждённой матрицей) соблюдения установленных правил взаимодействия.
+Класс используемых средств — межсетевые экраны, системы анализа и контроля соответствия конфигураций сетевой политике.
+Иностранные: Palo Alto Networks, Tufin и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F137" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Утверждённая матрица сетевого взаимодействия с сетью Интернет;
+3. Результаты сопоставления фактических правил межсетевого экранирования с утверждённой матрицей;
+4. Результаты тестирования (попытка взаимодействия, не предусмотренного матрицей), подтверждающие блокирование такого взаимодействия.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G137" s="151" t="inlineStr">
+        <is>
+          <t>1. Матрица сетевого взаимодействия с сетью Интернет не документирована или не актуализирована;
+2. Фактически разрешённое взаимодействие с Интернетом не соответствует утверждённой матрице (присутствуют незадокументированные правила);
+3. Сопоставление фактических правил с матрицей проводится нерегулярно;
+4. Матрица не пересматривается при вводе новых систем, взаимодействующих с сетью Интернет.</t>
+        </is>
+      </c>
       <c r="H137" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -9999,14 +10802,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D138" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы внешние устройства не имели возможности получить информацию о структуре внутренней сети организации, то есть чтобы применялась технология трансляции сетевых адресов (NAT). Это позволяет замаскировать реальные IP-адреса внутренних устройств за одним или несколькими публичными адресами.</t>
-        </is>
-      </c>
-      <c r="E138" s="31" t="n"/>
-      <c r="F138" s="31" t="n"/>
-      <c r="G138" s="31" t="n"/>
+      <c r="D138" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы внешние устройства не имели возможности получить информацию о структуре внутренней сети организации — то есть чтобы применялась технология трансляции сетевых адресов (NAT), маскирующая реальные IP-адреса внутренних устройств за одним или несколькими публичными адресами.
+Главная цель меры — затруднить злоумышленнику разведку (reconnaissance) внутренней сетевой инфраструктуры организации: без сокрытия топологии внешний наблюдатель способен по прямым IP-адресам внутренних узлов оценить масштаб и структуру сети, что облегчает планирование целенаправленной атаки.</t>
+        </is>
+      </c>
+      <c r="E138" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Применение технологии трансляции сетевых адресов (NAT) на границе внутренней сети и сети Интернет, скрывающей реальные IP-адреса внутренних узлов за публичным адресом (адресами) организации;
+2. Настройку сетевого оборудования и служб (DNS, маршрутизации) таким образом, чтобы информация о внутренней адресации и топологии сети не передавалась во внешнюю сеть в открытом виде (в том числе через служебные заголовки протоколов, сообщения об ошибках);
+3. Периодический технический контроль (сканирование извне, анализ исходящего трафика) на предмет непреднамеренного раскрытия сведений о внутренней топологии сети.
+Класс используемых средств — межсетевые экраны и маршрутизаторы с функцией трансляции сетевых адресов (NAT).
+Иностранные: Cisco ASA, Juniper SRX и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, iptables/nftables и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F138" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Скриншоты (выгрузки) настроек трансляции сетевых адресов (NAT) на границе с сетью Интернет;
+3. Результаты сканирования сети организации извне, подтверждающие отсутствие видимых реальных внутренних адресов;
+4. Результаты анализа исходящего трафика на предмет утечки сведений о внутренней топологии.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G138" s="151" t="inlineStr">
+        <is>
+          <t>1. Часть внешних сервисов организации опубликована с прямым (без NAT) внутренним адресом;
+2. Служебные заголовки или сообщения об ошибках внешних сервисов раскрывают сведения о внутренней сетевой топологии;
+3. Периодическая проверка (сканирование извне) на предмет раскрытия топологии не проводится;
+4. Настройки NAT не пересматриваются при изменении состава внешних сервисов.</t>
+        </is>
+      </c>
       <c r="H138" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -10031,14 +10880,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D139" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы обмен данными между внутренней инфраструктурой организации и глобальной сетью осуществлялся только через строго определённые, минимально необходимые точки входа/выхода, что позволяет централизованно контролировать и фильтровать весь внешний трафик. Это снижает риск несанкционированного доступа к внутренним ресурсам извне.</t>
-        </is>
-      </c>
-      <c r="E139" s="31" t="n"/>
-      <c r="F139" s="31" t="n"/>
-      <c r="G139" s="31" t="n"/>
+      <c r="D139" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы обмен данными между внутренней инфраструктурой организации и глобальной сетью осуществлялся только через строго определённые, минимально необходимые точки входа/выхода, что позволяет централизованно контролировать и фильтровать весь внешний трафик.
+Главная цель меры — исключить возможность бесконтрольного, неучтённого подключения внутренних сегментов сети напрямую к сети Интернет в обход централизованных точек контроля, поскольку каждая дополнительная нерегламентированная точка выхода в Интернет — это ещё один потенциальный канал для несанкционированного доступа или утечки данных, не охваченный установленными правилами фильтрации и мониторинга (мерами СМЭ.16—СМЭ.17).</t>
+        </is>
+      </c>
+      <c r="E139" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как речь идёт о чисто технической мере, реализация включает:
+1. Определение и документальное закрепление ограниченного перечня точек подключения внутренней сети организации к сети Интернет (пограничных маршрутизаторов, межсетевых экранов);
+2. Техническое исключение иных, нерегламентированных каналов выхода в сеть Интернет (например, точек доступа Wi-Fi с прямым выходом в Интернет, модемов, мобильного интернета на серверном оборудовании);
+3. Периодический технический контроль (сканирование, анализ конфигураций сетевого оборудования) на предмет выявления несанкционированных точек подключения к сети Интернет.
+Класс используемых средств — межсетевые экраны и маршрутизаторы, средства контроля сетевого периметра.
+Иностранные: Cisco ASA, Palo Alto Networks и пр.
+Российские сертифицированные (ФСТЭК): «Континент», UserGate и др.
+Открытый код: pfSense, OPNsense и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F139" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры;
+2. Схема сети с указанием утверждённых точек подключения к сети Интернет;
+3. Результаты сканирования (аудита) сети на предмет выявления несанкционированных точек выхода в Интернет;
+4. Скриншоты (выгрузки) настроек сетевого оборудования, подтверждающие отсутствие незадокументированных каналов подключения.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G139" s="151" t="inlineStr">
+        <is>
+          <t>1. Перечень утверждённых точек подключения к сети Интернет не документирован;
+2. Выявляются нерегламентированные каналы выхода в Интернет (например, через мобильные модемы или незарегистрированные точки доступа Wi-Fi);
+3. Периодический контроль (сканирование) на предмет несанкционированных точек подключения не проводится;
+4. Перечень утверждённых точек подключения не пересматривается при изменении сетевой инфраструктуры.</t>
+        </is>
+      </c>
       <c r="H139" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -10062,14 +10957,60 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D140" s="56" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы весь почтовый трафик между организацией и сетью Интернет проходил через строго определённые контролируемые узлы, состоящие из внешнего почтового сервера и внутреннего почтового сервера. Это снижает риск получения спам-сообщений и вредоносных вложений на внутренний сервер.</t>
-        </is>
-      </c>
-      <c r="E140" s="31" t="n"/>
-      <c r="F140" s="31" t="n"/>
-      <c r="G140" s="31" t="n"/>
+      <c r="D140" s="158" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы весь почтовый трафик между организацией и сетью Интернет проходил через строго определённые контролируемые узлы, состоящие из внешнего почтового сервера (подключённого к сети Интернет) и внутреннего почтового сервера (размещённого во внутренних сетях организации) с безопасной репликацией почтовых сообщений между ними.
+Главная цель меры — снизить риск получения спам-сообщений и вредоносных вложений непосредственно на внутренний почтовый сервер за счёт промежуточной обработки (фильтрации) корреспонденции на внешнем сервере, физически и логически отделённом от внутренней инфраструктуры, прежде чем сообщения будут реплицированы во внутренний контур.</t>
+        </is>
+      </c>
+      <c r="E140" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Поскольку мера реализуется только техническими методами, её внедрение предполагает:
+1. Развёртывание внешнего почтового сервера (шлюза), принимающего и отправляющего почту непосредственно из (в) сеть Интернет, и внутреннего почтового сервера, обслуживающего почтовые ящики пользователей организации;
+2. Настройку безопасной репликации (передачи) почтовых сообщений между внешним и внутренним почтовыми серверами по защищённому каналу связи, без предоставления внутреннему серверу прямого доступа к сети Интернет;
+3. Настройку на внешнем почтовом сервере функций фильтрации (антиспам, антивирусная проверка вложений) до передачи сообщений во внутренний контур.
+Класс используемых средств — почтовые шлюзы с функцией фильтрации (Secure Email Gateway).
+Иностранные: Proofpoint Email Security, Cisco Secure Email и пр.
+Российские сертифицированные (ФСТЭК): Kaspersky Security для почтовых серверов, Dr.Web Mail Security Suite и др.
+Открытый код: Postfix (совместно с SpamAssassin, ClamAV) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F140" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами почтовой инфраструктуры;
+2. Схема почтовой инфраструктуры, подтверждающая наличие раздельных внешнего и внутреннего почтовых серверов;
+3. Скриншоты настроек репликации почты между внешним и внутренним серверами;
+4. Скриншоты настроек фильтрации (антиспам, антивирусная проверка) на внешнем почтовом сервере.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G140" s="151" t="inlineStr">
+        <is>
+          <t>1. Внутренний почтовый сервер имеет прямой доступ к сети Интернет в обход внешнего сервера-шлюза;
+2. Фильтрация (антиспам, антивирусная проверка) на внешнем почтовом сервере отключена либо настроена не в полном объёме;
+3. Канал репликации почты между внешним и внутренним серверами не защищён (передача в открытом виде);
+4. Сигнатурные базы средств фильтрации почты не обновляются на регулярной основе.</t>
+        </is>
+      </c>
       <c r="H140" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -10106,14 +11047,60 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D142" s="44" t="inlineStr">
-        <is>
-          <t>Мера требует фиксировать в системных журналах все события, связанные с изменением конфигураций сетевого оборудования и средств защиты, отвечающих за сегментацию сети, фильтрацию трафика и защиту вычислительных сетей (например, модификацию правил межсетевого экранирования, настроек VLAN, параметров маршрутизации, списков контроля доступа (ACL) и т. п.). Это  необходимо для выявления несанкционированных или ошибочных изменений, нарушений изоляции сегментов.</t>
-        </is>
-      </c>
-      <c r="E142" s="31" t="n"/>
-      <c r="F142" s="31" t="n"/>
-      <c r="G142" s="31" t="n"/>
+      <c r="D142" s="153" t="inlineStr">
+        <is>
+          <t>Мера требует фиксировать в системных журналах все события, связанные с изменением конфигураций сетевого оборудования и средств защиты, отвечающих за сегментацию сети, фильтрацию трафика и защиту вычислительных сетей (модификацию правил межсетевого экранирования, настроек VLAN, параметров маршрутизации, списков контроля доступа (ACL) и т. п.).
+Главная цель меры — обеспечить возможность выявления несанкционированных или ошибочных изменений сетевой конфигурации, способных нарушить изоляцию сегментов (меры СМЭ.1—СМЭ.13) или ослабить фильтрацию трафика (меры СМЭ.3, СМЭ.16), поскольку без регистрации таких изменений факт нарушения сетевой защиты может долгое время оставаться незамеченным.</t>
+        </is>
+      </c>
+      <c r="E142" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+Так как данная мера — целиком техническая, для её выполнения необходимо:
+1. Настройку встроенных средств аудита сетевого оборудования и средств защиты информации (межсетевых экранов, коммутаторов, маршрутизаторов), регистрирующих каждое изменение параметров настроек, влияющих на сегментацию, фильтрацию и защиту сети;
+2. Фиксацию в журнале как минимум даты и времени изменения, идентификатора администратора, выполнившего изменение, и содержания изменённого параметра (старое и новое значение);
+3. Централизованный сбор журналов изменений конфигураций сетевого оборудования и средств защиты в SIEM-системе для последующего анализа и длительного хранения.
+Класс используемых средств — системы управления событиями информационной безопасности (SIEM), системы управления конфигурациями сетевого оборудования.
+Иностранные: Splunk, SolarWinds Network Configuration Manager и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, RuSIEM и др.
+Открытый код: Wazuh, RANCID (для контроля конфигураций) и др.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F142" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Проверочные процедуры (свидетельства) - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+1. Итоги интервью с администраторами сетевой инфраструктуры и подразделением информационной безопасности;
+2. Скриншоты настроек аудита на сетевом оборудовании и средствах защиты, подтверждающие регистрацию изменений конфигураций;
+3. Выгрузка журналов событий изменения конфигураций за проверяемый период;
+4. Настройки SIEM-системы, подтверждающие централизованный сбор указанных событий.</t>
+          </r>
+        </is>
+      </c>
+      <c r="G142" s="151" t="inlineStr">
+        <is>
+          <t>1. Регистрация изменений конфигураций включена не для всего сетевого оборудования и средств защиты, отвечающих за сегментацию и фильтрацию;
+2. Журналы не содержат достаточного набора атрибутов для определения того, кто и какое именно изменение внёс;
+3. Журналы изменений конфигураций не собираются централизованно, что затрудняет их анализ;
+4. Журналы не анализируются на предмет выявления несанкционированных или ошибочных изменений.</t>
+        </is>
+      </c>
       <c r="H142" s="26" t="inlineStr">
         <is>
           <t>Нет недостатков. 
@@ -25894,8 +26881,8 @@
     <mergeCell ref="A423:G423"/>
     <mergeCell ref="A174:G174"/>
     <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A84:G84"/>
     <mergeCell ref="A286:G286"/>

</xml_diff>

<commit_message>
Review fixes for ЗБС.1-ЗБС.10 (list «1. Описание мер», rows 163-173)
All 10 measures were already filled (D/E/F/G), but every single one
shared the same two defects found in earlier sections:
- D ran on without the mandatory 'Главная цель меры —' closing —
  appended it to all 10, keeping the existing explanation intact.
- E's product-examples block used dash bullets straight under
  'Примеры средств защиты:' with no tool class named first — replaced
  with the class-first, no-dash style used elsewhere in the document.
G expanded from 2 to 4 items (rule: 3-6) on 8 of the 10 measures
(ЗБС.3-10); ЗБС.1 and ЗБС.2 already had 3 and were left alone. F was
already good throughout and was not touched.
All touched cells shaded pale yellow for review.
</commit_message>
<xml_diff>
--- a/docs/WIKI GOST R 57580.1.xlsx
+++ b/docs/WIKI GOST R 57580.1.xlsx
@@ -12172,51 +12172,28 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D163" s="34" t="inlineStr">
-        <is>
-          <t>Точка доступа Wi-Fi должна проверять подлинность подключающегося устройства, а не пускать любое устройство, знающее пароль сети. Мера закрывает возможность подключения постороннего устройства к корпоративной беспроводной сети при компрометации общего пароля и обязует привязывать доступ к конкретному устройству/пользователю.</t>
-        </is>
-      </c>
-      <c r="E163" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D163" s="144" t="inlineStr">
+        <is>
+          <t>Точка доступа Wi-Fi должна проверять подлинность подключающегося устройства, а не пускать любое устройство, знающее пароль сети. Мера закрывает возможность подключения постороннего устройства к корпоративной беспроводной сети при компрометации общего пароля и обязует привязывать доступ к конкретному устройству/пользователю.
+Главная цель меры — исключить возможность подключения к корпоративной беспроводной сети любого устройства, знающего лишь общий пароль, не связывая доступ с конкретным устройством или пользователем, поскольку общий предварительный ключ (PSK) в случае утечки компрометирует сеть целиком, тогда как индивидуальная аутентификация позволяет отозвать доступ точечно.</t>
+        </is>
+      </c>
+      <c r="E163" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-На точках доступа настраивается аутентификация устройств по протоколу 802.1X с проверкой через RADIUS/сертификаты устройства, либо (как минимум) индивидуальные учётные данные вместо общего PSK-пароля. Не аутентифицированные устройства к сети не допускаются.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Примеры средств защиты:
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>- Иностранные: Cisco ISE + WLC, Aruba ClearPass и пр.
-- Российские сертифицированные: Ideco NGFW (RADIUS-модуль), «Атликс» Wi-Fi (сертифицированные точки доступа с 802.1X) и пр.
-- Открытый код: FreeRADIUS + hostapd и пр.</t>
+            <t xml:space="preserve">
+На точках доступа настраивается аутентификация устройств по протоколу 802.1X с проверкой через RADIUS/сертификаты устройства, либо (как минимум) индивидуальные учётные данные вместо общего PSK-пароля. Неаутентифицированные устройства к сети не допускаются.
+Класс используемых средств — RADIUS-серверы и контроллеры точек доступа с поддержкой 802.1X.
+Иностранные: Cisco ISE + WLC, Aruba ClearPass и пр.
+Российские сертифицированные (ФСТЭК): Ideco NGFW (RADIUS-модуль), точки доступа «Атликс» с поддержкой 802.1X и др.
+Открытый код: FreeRADIUS + hostapd и др.</t>
           </r>
         </is>
       </c>
@@ -12268,51 +12245,28 @@
           <t>Т-Т-Т</t>
         </is>
       </c>
-      <c r="D164" s="34" t="inlineStr">
-        <is>
-          <t>Трафик между устройством и точкой доступа должен быть зашифрован и защищён от подмены, чтобы защититься от перехвата передаваемых данных при слабом или устаревшем шифровании (например, WEP, WPA) и от внедрения поддельных пакетов в сессию при отсутствии контроля целостности.</t>
-        </is>
-      </c>
-      <c r="E164" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D164" s="144" t="inlineStr">
+        <is>
+          <t>Трафик между устройством и точкой доступа должен быть зашифрован и защищён от подмены, чтобы защититься от перехвата передаваемых данных при слабом или устаревшем шифровании (например, WEP, WPA) и от внедрения поддельных пакетов в сессию при отсутствии контроля целостности.
+Главная цель меры — защититься от перехвата передаваемых данных при слабом или устаревшем шифровании (например, WEP, WPA) и от внедрения поддельных пакетов в сессию при отсутствии контроля целостности, поскольку беспроводная среда передачи в принципе доступна для прослушивания любому находящемуся в зоне действия сигнала, и только стойкое шифрование делает перехваченный трафик бесполезным для злоумышленника.</t>
+        </is>
+      </c>
+      <c r="E164" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
             <t xml:space="preserve">
 На точках доступа и клиентских устройствах настраивается современный протокол шифрования беспроводного канала (WPA2-Enterprise/WPA3) с индивидуальными ключами сессии для каждого устройства. Устаревшие протоколы (WEP, WPA-PSK с общим ключом) отключаются.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Cisco WLC (WPA3-Enterprise), Aruba (WPA3) и пр.
-- Российские сертифицированные: точки доступа «Атликс» с поддержкой WPA2/WPA3-Enterprise и пр.
-- Открытый код: hostapd (WPA2/WPA3-Enterprise) и пр.</t>
+Класс используемых средств — точки доступа и контроллеры беспроводных сетей с поддержкой WPA2/WPA3-Enterprise.
+Иностранные: Cisco WLC (WPA3-Enterprise), Aruba (WPA3) и пр.
+Российские сертифицированные (ФСТЭК): точки доступа «Атликс» с поддержкой WPA2/WPA3-Enterprise и др.
+Открытый код: hostapd (WPA2/WPA3-Enterprise) и др.</t>
           </r>
         </is>
       </c>
@@ -12364,51 +12318,28 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D165" s="34" t="inlineStr">
-        <is>
-          <t>Точки доступа Wi-Fi и связанное с ними оборудование должны находиться в отдельном сетевом сегменте, а не подключаться напрямую во внутреннюю сеть наравне с другими устройствами, что сразу исключает компрометацию точки доступа (физическую или удалённую) и не даёт прямого доступа во внутреннюю сеть.</t>
-        </is>
-      </c>
-      <c r="E165" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D165" s="144" t="inlineStr">
+        <is>
+          <t>Точки доступа Wi-Fi и связанное с ними оборудование должны находиться в отдельном сетевом сегменте, а не подключаться напрямую во внутреннюю сеть наравне с другими устройствами, что сразу исключает компрометацию точки доступа (физическую или удалённую) и не даёт прямого доступа во внутреннюю сеть.
+Главная цель меры — исключить прямой доступ во внутреннюю сеть в случае компрометации точки доступа (физической или удалённой), поскольку выделенный сегмент ограничивает последствия такой компрометации периметром самого беспроводного сегмента, а не всей внутренней инфраструктурой.</t>
+        </is>
+      </c>
+      <c r="E165" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Точки доступа и их управляющие контроллеры выносятся в отдельный VLAN/сегмент, изолированный от прочих внутренних сетей на сетевом уровне (L3). Все дальнейшие требования по изоляции и МЭ (ЗБС.4–ЗБС.7) применяются именно к этому сегменту.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Примеры средств защиты:
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>- Иностранные: Cisco WLC + dedicated VLAN, Aruba Mobility Controller и пр.
-- Российские сертифицированные: PT NGFW, UserGate NGFW (сегментация VLAN), Континент 4 и пр.
-- Открытый код: VLAN-конфигурация на управляемых коммутаторах (например, через OpenWRT-инфраструктуру) и пр.</t>
+            <t xml:space="preserve">
+Точки доступа и их управляющие контроллеры выносятся в отдельный VLAN/сегмент, изолированный от прочих внутренних сетей на сетевом уровне (L3). Все дальнейшие требования по изоляции и межсетевому экранированию (меры ЗБС.4—ЗБС.7) применяются именно к этому сегменту.
+Класс используемых средств — активное сетевое оборудование с поддержкой сегментации сети (VLAN).
+Иностранные: Cisco WLC (выделенный VLAN), Aruba Mobility Controller и пр.
+Российские сертифицированные (ФСТЭК): PT NGFW, UserGate NGFW (сегментация VLAN), «Континент 4» и др.
+Открытый код: управляемые коммутаторы с поддержкой VLAN (например, на базе OpenWRT) и др.</t>
           </r>
         </is>
       </c>
@@ -12436,10 +12367,12 @@
           </r>
         </is>
       </c>
-      <c r="G165" s="36" t="inlineStr">
-        <is>
-          <t>1. Часть точек доступа подключена в общий сегмент с пользовательскими устройствами.
-2. Управляющий трафик контроллера точек доступа не изолирован от пользовательского Wi-Fi-трафика.</t>
+      <c r="G165" s="151" t="inlineStr">
+        <is>
+          <t>1. Часть точек доступа подключена в общий сегмент с пользовательскими устройствами;
+2. Управляющий трафик контроллера точек доступа не изолирован от пользовательского Wi-Fi-трафика;
+3. Выделенный сегмент не документирован в общей схеме сегментации сети (см. также меру СМЭ.1);
+4. Состав сегмента не пересматривается при подключении новых точек доступа.</t>
         </is>
       </c>
     </row>
@@ -12459,52 +12392,28 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D166" s="34" t="inlineStr">
-        <is>
-          <t>Требуется строгая изоляция беспроводного сегмента (ЗБС.3) от остальной внутренней сети на канальном уровне (L2) — без общего broadcast-домена и ARP-видимости, чтобы не происходила компрометация беспроводной инфраструктуры и нельзя было получить прямой L2-доступ к остальной внутренней сети (ARP-спуфинг, сниффинг широковещательного трафика).</t>
-        </is>
-      </c>
-      <c r="E166" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D166" s="144" t="inlineStr">
+        <is>
+          <t>Требуется строгая изоляция беспроводного сегмента (ЗБС.3) от остальной внутренней сети на канальном уровне (L2) — без общего broadcast-домена и ARP-видимости, чтобы не происходила компрометация беспроводной инфраструктуры и нельзя было получить прямой L2-доступ к остальной внутренней сети (ARP-спуфинг, сниффинг широковещательного трафика).
+Главная цель меры — не допустить компрометацию беспроводной инфраструктуры с получением прямого канального (L2) доступа к остальной внутренней сети, поскольку на канальном уровне возможны атаки (ARP-спуфинг, прослушивание широковещательного трафика), не блокируемые обычной маршрутизацией и фильтрацией на более высоких уровнях.</t>
+        </is>
+      </c>
+      <c r="E166" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
             <t xml:space="preserve">
 Беспроводной сегмент выносится в отдельный L2-домен без прямой канальной связности с прочими сетями, взаимодействие с остальной инфраструктурой строится только через контролируемый L3-шлюз с фильтрацией.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Cisco Catalyst (private VLAN, L2 isolation) и пр.
-- Российские сертифицированные: PT NGFW, UserGate NGFW и пр.
-- Открытый код: управляемые коммутаторы с private VLAN и пр.</t>
+Класс используемых средств — активное сетевое оборудование с поддержкой изоляции на канальном уровне (private VLAN).
+Иностранные: Cisco Catalyst (private VLAN, L2 isolation) и пр.
+Российские сертифицированные (ФСТЭК): PT NGFW, UserGate NGFW и др.
+Открытый код: управляемые коммутаторы с поддержкой private VLAN и др.</t>
           </r>
         </is>
       </c>
@@ -12532,10 +12441,12 @@
           </r>
         </is>
       </c>
-      <c r="G166" s="36" t="inlineStr">
-        <is>
-          <t>1. Обнаружена остаточная L2-связность (общий broadcast-домен) с внутренней сетью.
-2. Изоляция реализована только на сетевом уровне (L3), что не соответствует требованию УЗ1.</t>
+      <c r="G166" s="151" t="inlineStr">
+        <is>
+          <t>1. Обнаружена остаточная L2-связность (общий широковещательный домен) с внутренней сетью;
+2. Изоляция реализована только на сетевом уровне (L3), что не соответствует требованию для уровня защиты 1 (УЗ1);
+3. Контроллер точек доступа имеет канальную связность с сегментами, не относящимися к беспроводной инфраструктуре;
+4. Отсутствие L2-связности не подтверждается периодическим тестированием.</t>
         </is>
       </c>
     </row>
@@ -12555,51 +12466,28 @@
           <t>Н-Т-Н</t>
         </is>
       </c>
-      <c r="D167" s="34" t="inlineStr">
-        <is>
-          <t>Требуется изоляция беспроводного сегмента (ЗБС.3) от остальной внутренней сети на сетевом уровне (L3) — маршрутизация и списки управления доступом (ACL) между сегментами, без обязательной канальной изоляции. Это защищает от случаев, когда скомпрометированное Wi-Fi-устройство может свободно маршрутизировать трафик во внутреннюю сеть.</t>
-        </is>
-      </c>
-      <c r="E167" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D167" s="144" t="inlineStr">
+        <is>
+          <t>Требуется изоляция беспроводного сегмента (ЗБС.3) от остальной внутренней сети на сетевом уровне (L3) — маршрутизация и списки управления доступом (ACL) между сегментами, без обязательной канальной изоляции. Это защищает от случаев, когда скомпрометированное Wi-Fi-устройство может свободно маршрутизировать трафик во внутреннюю сеть.
+Главная цель меры — задать менее строгий (по сравнению с мерой ЗБС.4), но обязательный минимум изоляции беспроводного сегмента для уровней защиты, где полная канальная изоляция не требуется: маршрутизация и списки контроля доступа на сетевом уровне всё равно не позволяют скомпрометированному Wi-Fi-устройству свободно взаимодействовать с внутренней сетью в обход установленных правил.</t>
+        </is>
+      </c>
+      <c r="E167" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Между беспроводным сегментом и прочими внутренними сетями настраивается маршрутизация с контролем доступа (ACL/МЭ) на сетевом уровне, прямая L2-связность не обязательна к исключению.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Cisco Catalyst/WLC (L3 ACL) и пр.
-- Российские сертифицированные: PT NGFW, UserGate NGFW и пр.
-- Открытый код: iptables/nftables на пограничном маршрутизаторе сегмента и пр.</t>
+            <t xml:space="preserve">
+Между беспроводным сегментом и прочими внутренними сетями настраивается маршрутизация с контролем доступа (списками контроля доступа, межсетевым экраном) на сетевом уровне; прямая канальная (L2) изоляция при этом не обязательна.
+Класс используемых средств — маршрутизаторы и межсетевые экраны с поддержкой списков контроля доступа (ACL).
+Иностранные: Cisco Catalyst/WLC (ACL на сетевом уровне) и пр.
+Российские сертифицированные (ФСТЭК): PT NGFW, UserGate NGFW и др.
+Открытый код: iptables/nftables на пограничном маршрутизаторе сегмента и др.</t>
           </r>
         </is>
       </c>
@@ -12627,10 +12515,12 @@
           </r>
         </is>
       </c>
-      <c r="G167" s="36" t="inlineStr">
-        <is>
-          <t>1. ACL между сегментами не покрывают все направления трафика (например, только исходящий, без входящего контроля).
-2. Правила маршрутизации/ACL не пересматривались при изменении состава сегмента.</t>
+      <c r="G167" s="151" t="inlineStr">
+        <is>
+          <t>1. Списки контроля доступа между сегментами не покрывают все направления трафика (например, только исходящий, без входящего контроля);
+2. Правила маршрутизации и ACL не пересматривались при изменении состава сегмента;
+3. Часть трафика между беспроводным сегментом и внутренней сетью проходит в обход настроенной маршрутизации;
+4. Тестирование фактической изоляции (попытка недопустимого маршрута) не проводится.</t>
         </is>
       </c>
     </row>
@@ -12650,51 +12540,28 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D168" s="34" t="inlineStr">
-        <is>
-          <t>Между беспроводным сегментом (ЗБС.3) и остальной внутренней сетью должен стоять межсетевой экран, фильтрующий трафик не только по адресам/портам (сетевой уровень), но и по содержимому/приложениям (прикладной уровень). Это позволяет исключать случаи, когда вредоносный трафик или туннелирование внутри разрешённого протокола проходят через фильтр, ограниченный только сетевым уровнем, а также когда происходит обход политики доступа через разрешённые порты с нелегитимным содержимым.</t>
-        </is>
-      </c>
-      <c r="E168" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Реализация - Т
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">На стыке беспроводного сегмента с остальной сетью устанавливается межсетевой экран нового поколения (NGFW) с включённой фильтрацией на прикладном уровне (App-ID/DPI), а не только классический stateful-МЭ. Политики фильтрации формируются по принципу минимально необходимого доступа.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Palo Alto NGFW, Fortinet FortiGate и прочие.
-- Российские сертифицированные: PT NGFW (Positive Technologies, фильтрация на сетевом и прикладном уровнях, DPI), UserGate NGFW и прочие.
-- Открытый код: pfSense + Suricata (в режиме inline) и прочие.</t>
+      <c r="D168" s="144" t="inlineStr">
+        <is>
+          <t>Между беспроводным сегментом (ЗБС.3) и остальной внутренней сетью должен стоять межсетевой экран, фильтрующий трафик не только по адресам/портам (сетевой уровень), но и по содержимому/приложениям (прикладной уровень). Это позволяет исключать случаи, когда вредоносный трафик или туннелирование внутри разрешённого протокола проходят через фильтр, ограниченный только сетевым уровнем, а также когда происходит обход политики доступа через разрешённые порты с нелегитимным содержимым.
+Главная цель меры — исключить обход политики доступа, при котором вредоносный трафик или туннелирование маскируется под разрешённый протокол: фильтрация только по адресам и портам не способна выявить такую маскировку, тогда как анализ на прикладном уровне позволяет распознать несоответствие фактического содержимого заявленному протоколу.</t>
+        </is>
+      </c>
+      <c r="E168" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
+            </rPr>
+            <t>Реализация - Т</t>
+          </r>
+          <r>
+            <t xml:space="preserve">
+На стыке беспроводного сегмента с остальной сетью устанавливается межсетевой экран нового поколения (NGFW) с включённой фильтрацией на прикладном уровне (App-ID/DPI), а не только классический stateful-межсетевой экран. Политики фильтрации формируются по принципу минимально необходимого доступа.
+Класс используемых средств — межсетевые экраны следующего поколения (NGFW) с функцией глубокого анализа пакетов (DPI).
+Иностранные: Palo Alto NGFW, Fortinet FortiGate и пр.
+Российские сертифицированные (ФСТЭК): PT NGFW, UserGate NGFW и др.
+Открытый код: pfSense совместно с Suricata (в режиме inline) и др.</t>
           </r>
         </is>
       </c>
@@ -12722,10 +12589,12 @@
           </r>
         </is>
       </c>
-      <c r="G168" s="36" t="inlineStr">
-        <is>
-          <t>1. Фильтрация настроена только на сетевом уровне (адреса/порты), прикладной уровень не задействован.
-2. Политики МЭ избыточно широкие (правила «разрешить всё» вместо точечных правил).</t>
+      <c r="G168" s="151" t="inlineStr">
+        <is>
+          <t>1. Фильтрация настроена только на сетевом уровне (по адресам и портам), прикладной уровень не задействован;
+2. Политики межсетевого экрана избыточно широкие (правила «разрешить всё» вместо точечных правил);
+3. Сигнатурные базы и правила анализа прикладного уровня не обновляются на регулярной основе;
+4. Эффективность фильтрации на прикладном уровне не проверяется тестированием.</t>
         </is>
       </c>
     </row>
@@ -12745,52 +12614,28 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D169" s="34" t="inlineStr">
-        <is>
-          <t>Взаимодействие беспроводного сегмента с остальной сетью должно происходить строго по заранее определённым правилам и протоколам, а не произвольным образом. Это соответствие нужно постоянно контролировать, а не только настроить один раз, чтобы не возникал постепенный «дрейф» правил межсетевого экранирования (накопление избыточных разрешений со временем) и было запрещено использование нештатных протоколов или портов в обход утверждённой схемы взаимодействия.</t>
-        </is>
-      </c>
-      <c r="E169" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D169" s="144" t="inlineStr">
+        <is>
+          <t>Взаимодействие беспроводного сегмента с остальной сетью должно происходить строго по заранее определённым правилам и протоколам, а не произвольным образом. Это соответствие нужно постоянно контролировать, а не только настроить один раз, чтобы не возникал постепенный «дрейф» правил межсетевого экранирования (накопление избыточных разрешений со временем) и было запрещено использование нештатных протоколов или портов в обход утверждённой схемы взаимодействия.
+Главная цель меры — не допустить постепенного «дрейфа» правил межсетевого экранирования (накопления избыточных, никем не пересматриваемых разрешений с течением времени) и использования нештатных протоколов или портов в обход утверждённой схемы взаимодействия, поскольку однократной настройки правил недостаточно — соответствие фактической конфигурации утверждённым правилам нужно подтверждать регулярно.</t>
+        </is>
+      </c>
+      <c r="E169" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Реализация правил взаимодействия (матрица допустимых протоколов и направлений трафика между сегментом ЗБС.3 и остальной сетью) на межсетевое экранирование (МЭ) и периодическая сверка задокументированных правил с фактической конфигурацией — вручную или средствами анализа конфигураций.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Cisco Firepower Management Center (аудит правил) и прочие.
-- Российские сертифицированные: PT NGFW (журналирование и анализ применяемых правил), UserGate NGFW и прочие.
-- Открытый код: nftables + скрипты сверки конфигурации с эталоном и прочие.</t>
+            <t xml:space="preserve">
+Правила взаимодействия (матрица допустимых протоколов и направлений трафика между сегментом ЗБС.3 и остальной сетью) реализуются на межсетевом экране, а соответствие задокументированных правил фактической конфигурации периодически сверяется — вручную либо средствами анализа конфигураций.
+Класс используемых средств — межсетевые экраны, средства анализа и контроля соответствия конфигураций сетевой политике.
+Иностранные: Cisco Firepower Management Center (аудит правил) и пр.
+Российские сертифицированные (ФСТЭК): PT NGFW (журналирование и анализ применяемых правил), UserGate NGFW и др.
+Открытый код: nftables совместно со скриптами сверки конфигурации с эталоном и др.</t>
           </r>
         </is>
       </c>
@@ -12818,10 +12663,12 @@
           </r>
         </is>
       </c>
-      <c r="G169" s="36" t="inlineStr">
-        <is>
-          <t>1. Матрица допустимого взаимодействия устарела или не работает.
-2. Фактическая конфигурация МЭ расходится с утверждённой матрицей (избыточные правила не удаляются).</t>
+      <c r="G169" s="151" t="inlineStr">
+        <is>
+          <t>1. Матрица допустимого взаимодействия устарела и не отражает фактически используемые протоколы и направления;
+2. Фактическая конфигурация межсетевого экрана расходится с утверждённой матрицей (избыточные правила не удаляются);
+3. Периодическая сверка фактической конфигурации с матрицей не проводится или проводится формально;
+4. Ответственный за актуальность матрицы и её сверку с конфигурацией не определён.</t>
         </is>
       </c>
     </row>
@@ -12841,51 +12688,28 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D170" s="34" t="inlineStr">
-        <is>
-          <t>Точки доступа должны отклонять подключение любых устройств, не внесённых в реестр разрешённых, включая попытки подключения снаружи здания (с парковки, соседних помещений). Реализация меры не допустит подключение постороннего устройства к корпоративному Wi-Fi при перехвате или подборе учётных данных и предотвратит атаку с территориально удалённой точки (через направленную антенну) без физического проникновения в здание.</t>
-        </is>
-      </c>
-      <c r="E170" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D170" s="144" t="inlineStr">
+        <is>
+          <t>Точки доступа должны отклонять подключение любых устройств, не внесённых в реестр разрешённых, включая попытки подключения снаружи здания (с парковки, соседних помещений). Реализация меры не допустит подключение постороннего устройства к корпоративному Wi-Fi при перехвате или подборе учётных данных и предотвратит атаку с территориально удалённой точки (через направленную антенну) без физического проникновения в здание.
+Главная цель меры — не допустить подключения постороннего устройства к корпоративной беспроводной сети при перехвате или подборе учётных данных, а также предотвратить атаку с территориально удалённой точки (например, через направленную антенну с парковки или соседнего помещения) без физического проникновения в контролируемые здания и сооружения организации.</t>
+        </is>
+      </c>
+      <c r="E170" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-На точках доступа включается whitelist-контроль по MAC-адресу/сертификату устройства в дополнение к аутентификации устройств по 802.1X (ЗБС.1). Мощность сигнала точек доступа настраивается так, чтобы минимизировать покрытие за пределами контролируемой территории. Опционально — WIPS (беспроводная система предотвращения вторжений) для активного обнаружения и блокировки rogue-подключений через дополнительный анализ политик безопасности и классификацию устройств.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Cisco WLC (rogue containment), Aruba WIPS и прочие.
-- Российские сертифицированные: точки доступа «Атликс» с whitelist-фильтрацией и прочие.
-- Открытый код: hostapd (MAC ACL) и прочие.</t>
+            <t xml:space="preserve">
+На точках доступа включается контроль по списку разрешённых устройств (whitelist) по MAC-адресу или сертификату устройства в дополнение к аутентификации по протоколу 802.1X (мера ЗБС.1). Мощность сигнала точек доступа настраивается так, чтобы минимизировать покрытие за пределами контролируемой территории. Дополнительно может применяться беспроводная система предотвращения вторжений (WIPS) для активного обнаружения и блокирования несанкционированных (rogue) точек доступа и подключений.
+Класс используемых средств — точки доступа с функцией контроля устройств по списку разрешённых, беспроводные системы предотвращения вторжений (WIPS).
+Иностранные: Cisco WLC (rogue containment), Aruba WIPS и пр.
+Российские сертифицированные (ФСТЭК): точки доступа «Атликс» с контролем по списку разрешённых устройств и др.
+Открытый код: hostapd (контроль по MAC-адресам) и др.</t>
           </r>
         </is>
       </c>
@@ -12913,10 +12737,12 @@
           </r>
         </is>
       </c>
-      <c r="G170" s="36" t="inlineStr">
-        <is>
-          <t>1. Блокировка реализована только через 802.1X без дополнительного контроля по устройству (whitelist).
-2. Мощность сигнала не оптимизирована — сеть уверенно принимается за пределами здания.</t>
+      <c r="G170" s="151" t="inlineStr">
+        <is>
+          <t>1. Блокировка реализована только через 802.1X без дополнительного контроля по списку разрешённых устройств;
+2. Мощность сигнала не оптимизирована — сеть уверенно принимается за пределами здания;
+3. Система предотвращения вторжений (WIPS), выявляющая несанкционированные точки доступа, не развёрнута;
+4. Список разрешённых устройств не актуализируется при выводе устройств из эксплуатации.</t>
         </is>
       </c>
     </row>
@@ -12949,51 +12775,28 @@
           <t>Н-Н-Т</t>
         </is>
       </c>
-      <c r="D172" s="34" t="inlineStr">
-        <is>
-          <t>Мера требует, что каждая отклонённая попытка подключения незарегистрированного устройства (следуя ЗБС.8) должна фиксироваться как событие, а не просто блокироваться молча. Такой подход позволит предотвратить серию попыток подбора доступа, которая обычно остаётся незамеченной при отсутствии регистрации. Также без этой меры невозможно расследовать инцидент постфактум без истории попыток подключения.</t>
-        </is>
-      </c>
-      <c r="E172" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D172" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует, что каждая отклонённая попытка подключения незарегистрированного устройства (следуя ЗБС.8) должна фиксироваться как событие, а не просто блокироваться молча. Такой подход позволит предотвратить серию попыток подбора доступа, которая обычно остаётся незамеченной при отсутствии регистрации. Также без этой меры невозможно расследовать инцидент постфактум без истории попыток подключения.
+Главная цель меры — обеспечить возможность выявления серии попыток подбора доступа к беспроводной сети, которая обычно остаётся незамеченной при отсутствии регистрации, а также сформировать историю попыток подключения, без которой невозможно расследовать инцидент постфактум.</t>
+        </is>
+      </c>
+      <c r="E172" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Точки доступа настраиваются на генерацию события при каждой отклонённой попытке подключения (MAC-адрес устройства, время, точка доступа), дополнительно события могут передаваться в SIEM для корреляции и алертинга при аномальной частоте попыток.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">Примеры средств защиты:
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t>- Иностранные: Cisco WLC + Splunk и прочие.
-- Российские сертифицированные: PT MaxPatrol SIEM, Kaspersky KUMA — приём и корреляция событий с точек доступа и прочие
-- Открытый код: Wazuh и прочие.</t>
+            <t xml:space="preserve">
+Точки доступа настраиваются на генерацию события при каждой отклонённой попытке подключения (с фиксацией MAC-адреса устройства, времени и точки доступа); дополнительно события могут передаваться в SIEM-систему для корреляции и оповещения при аномальной частоте попыток.
+Класс используемых средств — точки доступа со встроенным журналированием, системы управления событиями информационной безопасности (SIEM).
+Иностранные: Cisco WLC совместно со Splunk и пр.
+Российские сертифицированные (ФСТЭК): MaxPatrol SIEM, Kaspersky KUMA (приём и корреляция событий с точек доступа) и др.
+Открытый код: Wazuh и др.</t>
           </r>
         </is>
       </c>
@@ -13021,10 +12824,12 @@
           </r>
         </is>
       </c>
-      <c r="G172" s="36" t="inlineStr">
-        <is>
-          <t>1. События регистрируются локально на точке доступа, но отдельно не выделяются попытки подключения за пределами периметра.
-2. Отсутствует алертинг при массовых или повторяющихся попытках подключения (событие фиксируется, но не анализируется).</t>
+      <c r="G172" s="151" t="inlineStr">
+        <is>
+          <t>1. События регистрируются локально на точке доступа, но отдельно не выделяются попытки подключения из-за пределов контролируемой территории;
+2. Оповещение при массовых или повторяющихся попытках подключения не настроено (событие фиксируется, но не анализируется);
+3. События отклонённых подключений не передаются в централизованную систему (SIEM), что затрудняет корреляцию с иными событиями;
+4. Журналы отклонённых подключений хранятся менее срока, необходимого для расследования.</t>
         </is>
       </c>
     </row>
@@ -13044,52 +12849,28 @@
           <t>Н-Т-Т</t>
         </is>
       </c>
-      <c r="D173" s="34" t="inlineStr">
-        <is>
-          <t>Мера требует, чтобы любое изменение настроек межсетевого экранирования (МЭ) или сегментации, защищающих беспроводной сегмент (ЗБС.4–ЗБС.7), фиксировалось как полноценное событие — кто, когда и что изменил. Именно так можно вовремя предотвратить несанкционированное или ошибочное изменение правил (например, добавление избыточного разрешения), которое иначе осталось бы незамеченным без журнала изменений, и когда невозможно установить причину появления такой «дыры» в правилах при расследовании.</t>
-        </is>
-      </c>
-      <c r="E173" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
+      <c r="D173" s="144" t="inlineStr">
+        <is>
+          <t>Мера требует, чтобы любое изменение настроек межсетевого экранирования (МЭ) или сегментации, защищающих беспроводной сегмент (ЗБС.4–ЗБС.7), фиксировалось как полноценное событие — кто, когда и что изменил. Именно так можно вовремя предотвратить несанкционированное или ошибочное изменение правил (например, добавление избыточного разрешения), которое иначе осталось бы незамеченным без журнала изменений, и когда невозможно установить причину появления такой «дыры» в правилах при расследовании.
+Главная цель меры — своевременно выявлять несанкционированное или ошибочное изменение правил защиты беспроводного сегмента (например, добавление избыточного разрешения), которое иначе осталось бы незамеченным, и обеспечить возможность установить причину появления такой «дыры» в правилах при расследовании.</t>
+        </is>
+      </c>
+      <c r="E173" s="151" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Roboto"/>
+              <b val="1"/>
             </rPr>
             <t>Реализация - Т</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-На МЭ/системах сегментации включается журналирование изменений конфигурации (аудит-лог) с фиксацией учётной записи администратора, времени и содержания. События по изменениям дополнительно могут передаваться в SIEM/систему управления изменениями.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <b val="1"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-Примеры средств защиты:</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Roboto"/>
-              <color theme="1"/>
-              <sz val="11"/>
-            </rPr>
-            <t xml:space="preserve">
-- Иностранные: Cisco Firepower (change audit log) и прочие.
-- Российские сертифицированные: PT NGFW для журнал изменений конфигурации сети, PT MaxPatrol SIEM / Kaspersky KUMA для централизованного сбора и прочие.
-- Открытый код: Git-репозиторий конфигураций (config-as-code) + аудит коммитов и прочие.</t>
+            <t xml:space="preserve">
+На межсетевых экранах и системах сегментации включается журналирование изменений конфигурации (аудит-лог) с фиксацией учётной записи администратора, времени и содержания изменения. События об изменениях дополнительно могут передаваться в SIEM-систему или систему управления изменениями.
+Класс используемых средств — межсетевые экраны и системы сегментации со встроенным аудитом изменений, системы управления событиями информационной безопасности (SIEM).
+Иностранные: Cisco Firepower (журнал изменений конфигурации) и пр.
+Российские сертифицированные (ФСТЭК): PT NGFW (журнал изменений конфигурации сети), MaxPatrol SIEM, Kaspersky KUMA (централизованный сбор) и др.
+Открытый код: Git-репозиторий конфигураций (config-as-code) совместно с аудитом коммитов и др.</t>
           </r>
         </is>
       </c>
@@ -13117,10 +12898,12 @@
           </r>
         </is>
       </c>
-      <c r="G173" s="36" t="inlineStr">
-        <is>
-          <t>1. Изменения конфигурации фиксируются не на всех устройствах сегментации.
-2. Журнал изменений не содержит привязки к конкретным учётным записям (используется общая административная учётная запись).</t>
+      <c r="G173" s="151" t="inlineStr">
+        <is>
+          <t>1. Изменения конфигурации фиксируются не на всех устройствах сегментации;
+2. Журнал изменений не содержит привязки к конкретным учётным записям (используется общая административная учётная запись);
+3. События изменения конфигурации не передаются в централизованную систему (SIEM);
+4. Журнал изменений не анализируется на предмет выявления несанкционированных или ошибочных изменений.</t>
         </is>
       </c>
     </row>
@@ -27030,8 +26813,8 @@
     <mergeCell ref="A423:G423"/>
     <mergeCell ref="A174:G174"/>
     <mergeCell ref="A108:G108"/>
+    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A309:G309"/>
     <mergeCell ref="A133:G133"/>
     <mergeCell ref="A84:G84"/>
     <mergeCell ref="A286:G286"/>

</xml_diff>